<commit_message>
Updated spreadsheet to include actual L of winded inductor.
</commit_message>
<xml_diff>
--- a/Excel/Boost Converter Design Params.xlsx
+++ b/Excel/Boost Converter Design Params.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\weiwi\OneDrive\Documents\GitHub\311\Excel\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A21EF389-5E2F-4FE6-B20B-22B3D5565A13}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{53354F8C-67C8-49BA-99E6-BFE737A9FF7B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-98" yWindow="-98" windowWidth="21795" windowHeight="12975" xr2:uid="{0EA872C3-4804-43CB-9F0B-5F94DB7B4351}"/>
+    <workbookView xWindow="-98" yWindow="-98" windowWidth="21795" windowHeight="12975" activeTab="1" xr2:uid="{0EA872C3-4804-43CB-9F0B-5F94DB7B4351}"/>
   </bookViews>
   <sheets>
     <sheet name="SS_Analysis" sheetId="1" r:id="rId1"/>
@@ -1736,7 +1736,7 @@
     <xf numFmtId="0" fontId="1" fillId="3" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="133">
+  <cellXfs count="134">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
@@ -1886,6 +1886,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="64" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="2" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="167" fontId="0" fillId="0" borderId="34" xfId="0" applyNumberFormat="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="4">
     <cellStyle name="20% - Accent1" xfId="2" builtinId="30"/>
@@ -4414,18 +4415,18 @@
     <col min="2" max="9" width="12.875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" ht="20.65">
+    <row r="1" spans="1:5" ht="20.65">
       <c r="A1" s="1" t="s">
         <v>90</v>
       </c>
     </row>
-    <row r="3" spans="1:3" ht="17.649999999999999">
+    <row r="3" spans="1:5" ht="17.649999999999999">
       <c r="A3" s="2" t="s">
         <v>61</v>
       </c>
     </row>
-    <row r="4" spans="1:3" ht="13.9" thickBot="1"/>
-    <row r="5" spans="1:3" ht="14.65" thickTop="1" thickBot="1">
+    <row r="4" spans="1:5" ht="13.9" thickBot="1"/>
+    <row r="5" spans="1:5" ht="14.65" thickTop="1" thickBot="1">
       <c r="A5" s="3" t="s">
         <v>0</v>
       </c>
@@ -4435,8 +4436,9 @@
       <c r="C5" s="3" t="s">
         <v>2</v>
       </c>
-    </row>
-    <row r="6" spans="1:3" ht="13.9" thickTop="1">
+      <c r="E5" s="73"/>
+    </row>
+    <row r="6" spans="1:5" ht="13.9" thickTop="1">
       <c r="A6" s="37" t="s">
         <v>101</v>
       </c>
@@ -4448,7 +4450,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="7" spans="1:3">
+    <row r="7" spans="1:5">
       <c r="A7" s="38" t="s">
         <v>92</v>
       </c>
@@ -4460,7 +4462,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="8" spans="1:3">
+    <row r="8" spans="1:5">
       <c r="A8" s="38" t="s">
         <v>93</v>
       </c>
@@ -4472,7 +4474,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="9" spans="1:3">
+    <row r="9" spans="1:5">
       <c r="A9" s="38" t="s">
         <v>91</v>
       </c>
@@ -4484,7 +4486,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="10" spans="1:3">
+    <row r="10" spans="1:5">
       <c r="A10" s="7" t="s">
         <v>62</v>
       </c>
@@ -4495,7 +4497,7 @@
         <v>63</v>
       </c>
     </row>
-    <row r="11" spans="1:3" ht="13.9" thickBot="1">
+    <row r="11" spans="1:5" ht="13.9" thickBot="1">
       <c r="A11" s="10" t="s">
         <v>5</v>
       </c>
@@ -4507,18 +4509,18 @@
         <v>6</v>
       </c>
     </row>
-    <row r="12" spans="1:3" ht="15.4" thickTop="1">
+    <row r="12" spans="1:5" ht="15.4" thickTop="1">
       <c r="A12" s="13"/>
     </row>
-    <row r="14" spans="1:3" ht="17.649999999999999">
+    <row r="14" spans="1:5" ht="17.649999999999999">
       <c r="A14" s="2" t="s">
         <v>64</v>
       </c>
     </row>
-    <row r="15" spans="1:3" ht="18" thickBot="1">
+    <row r="15" spans="1:5" ht="18" thickBot="1">
       <c r="A15" s="2"/>
     </row>
-    <row r="16" spans="1:3" ht="14.65" thickTop="1" thickBot="1">
+    <row r="16" spans="1:5" ht="14.65" thickTop="1" thickBot="1">
       <c r="A16" s="3" t="s">
         <v>0</v>
       </c>
@@ -4862,7 +4864,9 @@
       <c r="A52" s="81" t="s">
         <v>98</v>
       </c>
-      <c r="B52" s="75"/>
+      <c r="B52" s="75">
+        <v>48.296999999999997</v>
+      </c>
       <c r="C52" s="76" t="s">
         <v>89</v>
       </c>
@@ -4871,7 +4875,10 @@
       <c r="A53" s="74" t="s">
         <v>85</v>
       </c>
-      <c r="B53" s="88"/>
+      <c r="B53" s="133">
+        <f>(B52*B8)/(B34*B19)</f>
+        <v>0.20769450283115989</v>
+      </c>
       <c r="C53" s="64" t="s">
         <v>63</v>
       </c>
@@ -4880,16 +4887,20 @@
       <c r="A54" s="81" t="s">
         <v>145</v>
       </c>
-      <c r="B54" s="88"/>
+      <c r="B54" s="88">
+        <v>50</v>
+      </c>
       <c r="C54" s="64" t="s">
-        <v>63</v>
+        <v>100</v>
       </c>
     </row>
     <row r="55" spans="1:3" ht="13.9" thickBot="1">
       <c r="A55" s="82" t="s">
         <v>99</v>
       </c>
-      <c r="B55" s="86"/>
+      <c r="B55" s="86">
+        <v>273</v>
+      </c>
       <c r="C55" s="87" t="s">
         <v>100</v>
       </c>

</xml_diff>

<commit_message>
Ran tests on a breadboard for open loop. Values on third slide of "Boost Converter Design Params"
</commit_message>
<xml_diff>
--- a/Excel/Boost Converter Design Params.xlsx
+++ b/Excel/Boost Converter Design Params.xlsx
@@ -1,20 +1,22 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="24334"/>
-  <workbookPr/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30326"/>
+  <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\weiwi\OneDrive\Documents\GitHub\311\Excel\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\tytom\Documents\GitHub\311\Excel\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{53354F8C-67C8-49BA-99E6-BFE737A9FF7B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{93275298-0660-4CC6-B32F-DE681B0E9495}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-98" yWindow="-98" windowWidth="21795" windowHeight="12975" activeTab="1" xr2:uid="{0EA872C3-4804-43CB-9F0B-5F94DB7B4351}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="2" xr2:uid="{0EA872C3-4804-43CB-9F0B-5F94DB7B4351}"/>
   </bookViews>
   <sheets>
     <sheet name="SS_Analysis" sheetId="1" r:id="rId1"/>
     <sheet name="Inductor_Design" sheetId="2" r:id="rId2"/>
+    <sheet name="Testing_OpenLoop" sheetId="3" r:id="rId3"/>
+    <sheet name="Testing_ClosedLoop" sheetId="4" r:id="rId4"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -30,15 +32,12 @@
         <xcalcf:feature name="microsoft.com:LET_WF"/>
       </xcalcf:calcFeatures>
     </ext>
-    <ext xmlns:xlwcv="http://schemas.microsoft.com/office/spreadsheetml/2024/workbookCompatibilityVersion" uri="{D14903EA-33C4-47F7-8F05-3474C54BE107}">
-      <xlwcv:version setVersion="1"/>
-    </ext>
   </extLst>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="459" uniqueCount="220">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="544" uniqueCount="262">
   <si>
     <t>Parameter</t>
   </si>
@@ -698,6 +697,132 @@
   </si>
   <si>
     <t xml:space="preserve">Limits current through IC. </t>
+  </si>
+  <si>
+    <t>Input V</t>
+  </si>
+  <si>
+    <t>Duty Cycle</t>
+  </si>
+  <si>
+    <t>Testing Items for each:</t>
+  </si>
+  <si>
+    <t>Output V</t>
+  </si>
+  <si>
+    <t>Current through inductor</t>
+  </si>
+  <si>
+    <t>Current through shunt branch</t>
+  </si>
+  <si>
+    <t>Rl values</t>
+  </si>
+  <si>
+    <t>*</t>
+  </si>
+  <si>
+    <t>Rl protection testing</t>
+  </si>
+  <si>
+    <t>&gt; E12 Standard</t>
+  </si>
+  <si>
+    <t>Rl_E12 values</t>
+  </si>
+  <si>
+    <t>Testing with breadboard: E12 values</t>
+  </si>
+  <si>
+    <t>Rl = 5.6</t>
+  </si>
+  <si>
+    <t>Rl = 10</t>
+  </si>
+  <si>
+    <t>Rl = 22</t>
+  </si>
+  <si>
+    <t>Rl = 33</t>
+  </si>
+  <si>
+    <t>Rl = 47</t>
+  </si>
+  <si>
+    <t>Order list: breadboard testing</t>
+  </si>
+  <si>
+    <t>Breadboard</t>
+  </si>
+  <si>
+    <t>5.6, 10, 22, 33, 47 ohm resistors</t>
+  </si>
+  <si>
+    <t>47uH inductor</t>
+  </si>
+  <si>
+    <t>Schotty diode</t>
+  </si>
+  <si>
+    <t>&gt; Input V given by DC power supply</t>
+  </si>
+  <si>
+    <t>&gt;Switch operated using oscilloscope</t>
+  </si>
+  <si>
+    <t>3.5V</t>
+  </si>
+  <si>
+    <t>3.9V</t>
+  </si>
+  <si>
+    <t>4.3V</t>
+  </si>
+  <si>
+    <t>4.2V</t>
+  </si>
+  <si>
+    <t>3.8V</t>
+  </si>
+  <si>
+    <t>4.26V</t>
+  </si>
+  <si>
+    <t>Real R: 47.13</t>
+  </si>
+  <si>
+    <t>Real R: 10.07</t>
+  </si>
+  <si>
+    <t>Real R: 5.58</t>
+  </si>
+  <si>
+    <t>3V</t>
+  </si>
+  <si>
+    <t>Real R: 22.08</t>
+  </si>
+  <si>
+    <t>3.4V</t>
+  </si>
+  <si>
+    <t>4V</t>
+  </si>
+  <si>
+    <t>4.1V</t>
+  </si>
+  <si>
+    <t>Real R: 32.89</t>
+  </si>
+  <si>
+    <t>^Note: Others were not measured</t>
+  </si>
+  <si>
+    <t xml:space="preserve">due to time constraints, and lack of </t>
+  </si>
+  <si>
+    <t>0.1ohm shunt resistors available.</t>
   </si>
 </sst>
 </file>
@@ -712,7 +837,7 @@
     <numFmt numFmtId="168" formatCode="0.0000000"/>
     <numFmt numFmtId="169" formatCode="0.0000"/>
   </numFmts>
-  <fonts count="10">
+  <fonts count="10" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -785,10 +910,11 @@
       <sz val="11"/>
       <color theme="1"/>
       <name val="Aptos Narrow"/>
+      <family val="2"/>
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="7">
+  <fills count="9">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -824,6 +950,18 @@
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="4" tint="0.59999389629810485"/>
+        <bgColor indexed="65"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="9" tint="0.79998168889431442"/>
+        <bgColor indexed="65"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="65">
     <border>
@@ -1730,13 +1868,15 @@
       <diagonal/>
     </border>
   </borders>
-  <cellStyleXfs count="4">
+  <cellStyleXfs count="6">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="1" applyNumberFormat="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="1" fillId="3" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="1" fillId="7" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="1" fillId="8" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="134">
+  <cellXfs count="138">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
@@ -1874,7 +2014,7 @@
     <xf numFmtId="49" fontId="8" fillId="0" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
     <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="169" fontId="0" fillId="0" borderId="49" xfId="0" applyNumberFormat="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="44" xfId="0" applyNumberFormat="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="44" xfId="0" applyBorder="1"/>
     <xf numFmtId="2" fontId="0" fillId="0" borderId="49" xfId="0" applyNumberFormat="1" applyBorder="1"/>
     <xf numFmtId="1" fontId="0" fillId="0" borderId="49" xfId="0" applyNumberFormat="1" applyBorder="1"/>
     <xf numFmtId="169" fontId="0" fillId="0" borderId="53" xfId="0" applyNumberFormat="1" applyBorder="1"/>
@@ -1882,17 +2022,23 @@
     <xf numFmtId="169" fontId="0" fillId="0" borderId="63" xfId="0" applyNumberFormat="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="64" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="1" fillId="3" borderId="0" xfId="2" applyBorder="1"/>
-    <xf numFmtId="166" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="64" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="2" applyFont="1" applyBorder="1"/>
     <xf numFmtId="167" fontId="0" fillId="0" borderId="34" xfId="0" applyNumberFormat="1" applyBorder="1"/>
+    <xf numFmtId="9" fontId="0" fillId="0" borderId="0" xfId="3" applyFont="1"/>
+    <xf numFmtId="9" fontId="0" fillId="0" borderId="0" xfId="3" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="0" xfId="2"/>
+    <xf numFmtId="0" fontId="1" fillId="7" borderId="0" xfId="4"/>
+    <xf numFmtId="0" fontId="1" fillId="8" borderId="0" xfId="5"/>
+    <xf numFmtId="9" fontId="1" fillId="8" borderId="0" xfId="5" applyNumberFormat="1"/>
   </cellXfs>
-  <cellStyles count="4">
+  <cellStyles count="6">
     <cellStyle name="20% - Accent1" xfId="2" builtinId="30"/>
+    <cellStyle name="20% - Accent6" xfId="5" builtinId="50"/>
+    <cellStyle name="40% - Accent1" xfId="4" builtinId="31"/>
     <cellStyle name="Check Cell" xfId="1" builtinId="23"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
-    <cellStyle name="Per cent" xfId="3" builtinId="5"/>
+    <cellStyle name="Percent" xfId="3" builtinId="5"/>
   </cellStyles>
   <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
@@ -2274,30 +2420,30 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E4C28CAE-7D6E-414C-9BF7-B54583CFEE9E}">
   <dimension ref="A1:N129"/>
-  <sheetFormatPr defaultColWidth="12" defaultRowHeight="13.5"/>
+  <sheetFormatPr defaultColWidth="12" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="20.4375" customWidth="1"/>
-    <col min="2" max="2" width="13.5625" customWidth="1"/>
-    <col min="3" max="3" width="13.3125" customWidth="1"/>
-    <col min="4" max="7" width="12.875" customWidth="1"/>
+    <col min="1" max="1" width="20.44140625" customWidth="1"/>
+    <col min="2" max="2" width="13.5546875" customWidth="1"/>
+    <col min="3" max="3" width="13.33203125" customWidth="1"/>
+    <col min="4" max="7" width="12.88671875" customWidth="1"/>
     <col min="8" max="8" width="22" customWidth="1"/>
-    <col min="9" max="11" width="12.875" customWidth="1"/>
-    <col min="12" max="12" width="17.4375" customWidth="1"/>
-    <col min="13" max="13" width="18.875" customWidth="1"/>
+    <col min="9" max="11" width="12.88671875" customWidth="1"/>
+    <col min="12" max="12" width="17.44140625" customWidth="1"/>
+    <col min="13" max="13" width="18.88671875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" ht="20.65">
+    <row r="1" spans="1:3" ht="21" x14ac:dyDescent="0.4">
       <c r="A1" s="1" t="s">
         <v>58</v>
       </c>
     </row>
-    <row r="3" spans="1:3" ht="17.649999999999999">
+    <row r="3" spans="1:3" ht="18" x14ac:dyDescent="0.35">
       <c r="A3" s="2" t="s">
         <v>137</v>
       </c>
     </row>
-    <row r="4" spans="1:3" ht="13.9" thickBot="1"/>
-    <row r="5" spans="1:3" ht="14.65" thickTop="1" thickBot="1">
+    <row r="4" spans="1:3" ht="15" thickBot="1" x14ac:dyDescent="0.35"/>
+    <row r="5" spans="1:3" ht="15.6" thickTop="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A5" s="3" t="s">
         <v>0</v>
       </c>
@@ -2308,7 +2454,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="6" spans="1:3" ht="13.9" thickTop="1">
+    <row r="6" spans="1:3" ht="15" thickTop="1" x14ac:dyDescent="0.3">
       <c r="A6" s="37" t="s">
         <v>36</v>
       </c>
@@ -2319,7 +2465,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="7" spans="1:3">
+    <row r="7" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A7" s="38" t="s">
         <v>37</v>
       </c>
@@ -2330,7 +2476,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="8" spans="1:3">
+    <row r="8" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A8" s="38" t="s">
         <v>38</v>
       </c>
@@ -2341,7 +2487,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="9" spans="1:3">
+    <row r="9" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A9" s="38" t="s">
         <v>56</v>
       </c>
@@ -2352,7 +2498,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="10" spans="1:3">
+    <row r="10" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A10" s="38" t="s">
         <v>57</v>
       </c>
@@ -2363,7 +2509,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="11" spans="1:3" ht="13.9" thickBot="1">
+    <row r="11" spans="1:3" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A11" s="10" t="s">
         <v>5</v>
       </c>
@@ -2374,16 +2520,16 @@
         <v>6</v>
       </c>
     </row>
-    <row r="12" spans="1:3" ht="15.4" thickTop="1">
+    <row r="12" spans="1:3" ht="16.2" thickTop="1" x14ac:dyDescent="0.3">
       <c r="A12" s="13"/>
     </row>
-    <row r="14" spans="1:3" ht="17.649999999999999">
+    <row r="14" spans="1:3" ht="18" x14ac:dyDescent="0.35">
       <c r="A14" s="2" t="s">
         <v>55</v>
       </c>
     </row>
-    <row r="15" spans="1:3" ht="13.9" thickBot="1"/>
-    <row r="16" spans="1:3" ht="14.65" thickTop="1" thickBot="1">
+    <row r="15" spans="1:3" ht="15" thickBot="1" x14ac:dyDescent="0.35"/>
+    <row r="16" spans="1:3" ht="15.6" thickTop="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A16" s="3" t="s">
         <v>0</v>
       </c>
@@ -2394,7 +2540,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="17" spans="1:3" ht="13.9" thickTop="1">
+    <row r="17" spans="1:3" ht="15" thickTop="1" x14ac:dyDescent="0.3">
       <c r="A17" s="45" t="s">
         <v>41</v>
       </c>
@@ -2406,7 +2552,7 @@
         <v>102</v>
       </c>
     </row>
-    <row r="18" spans="1:3">
+    <row r="18" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A18" s="47" t="s">
         <v>40</v>
       </c>
@@ -2418,7 +2564,7 @@
         <v>103</v>
       </c>
     </row>
-    <row r="19" spans="1:3">
+    <row r="19" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A19" s="56" t="s">
         <v>59</v>
       </c>
@@ -2430,7 +2576,7 @@
         <v>104</v>
       </c>
     </row>
-    <row r="20" spans="1:3">
+    <row r="20" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A20" s="49" t="s">
         <v>60</v>
       </c>
@@ -2442,7 +2588,7 @@
         <v>105</v>
       </c>
     </row>
-    <row r="21" spans="1:3">
+    <row r="21" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A21" s="52" t="s">
         <v>43</v>
       </c>
@@ -2454,7 +2600,7 @@
         <v>106</v>
       </c>
     </row>
-    <row r="22" spans="1:3">
+    <row r="22" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A22" s="52" t="s">
         <v>146</v>
       </c>
@@ -2466,7 +2612,7 @@
         <v>151</v>
       </c>
     </row>
-    <row r="23" spans="1:3">
+    <row r="23" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A23" s="52" t="s">
         <v>44</v>
       </c>
@@ -2478,7 +2624,7 @@
         <v>152</v>
       </c>
     </row>
-    <row r="24" spans="1:3">
+    <row r="24" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A24" s="93" t="s">
         <v>147</v>
       </c>
@@ -2490,7 +2636,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="25" spans="1:3" ht="13.9" thickBot="1">
+    <row r="25" spans="1:3" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A25" s="85" t="s">
         <v>101</v>
       </c>
@@ -2501,14 +2647,14 @@
         <v>8</v>
       </c>
     </row>
-    <row r="26" spans="1:3" ht="13.9" thickTop="1"/>
-    <row r="28" spans="1:3" ht="17.649999999999999">
+    <row r="26" spans="1:3" ht="15" thickTop="1" x14ac:dyDescent="0.3"/>
+    <row r="28" spans="1:3" ht="18" x14ac:dyDescent="0.35">
       <c r="A28" s="2" t="s">
         <v>9</v>
       </c>
     </row>
-    <row r="29" spans="1:3" ht="13.9" thickBot="1"/>
-    <row r="30" spans="1:3" ht="14.65" thickTop="1" thickBot="1">
+    <row r="29" spans="1:3" ht="15" thickBot="1" x14ac:dyDescent="0.35"/>
+    <row r="30" spans="1:3" ht="15.6" thickTop="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A30" s="3" t="s">
         <v>0</v>
       </c>
@@ -2519,7 +2665,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="31" spans="1:3" ht="13.9" thickTop="1">
+    <row r="31" spans="1:3" ht="15" thickTop="1" x14ac:dyDescent="0.3">
       <c r="A31" s="4" t="s">
         <v>10</v>
       </c>
@@ -2530,7 +2676,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="32" spans="1:3">
+    <row r="32" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A32" s="95" t="s">
         <v>148</v>
       </c>
@@ -2542,7 +2688,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="33" spans="1:11">
+    <row r="33" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A33" s="15" t="s">
         <v>11</v>
       </c>
@@ -2554,7 +2700,7 @@
         <v>150</v>
       </c>
     </row>
-    <row r="34" spans="1:11">
+    <row r="34" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A34" s="27" t="s">
         <v>149</v>
       </c>
@@ -2566,7 +2712,7 @@
         <v>107</v>
       </c>
     </row>
-    <row r="35" spans="1:11" ht="13.9" thickBot="1">
+    <row r="35" spans="1:11" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A35" s="10" t="s">
         <v>12</v>
       </c>
@@ -2577,14 +2723,14 @@
         <v>107</v>
       </c>
     </row>
-    <row r="36" spans="1:11" ht="13.9" thickTop="1"/>
-    <row r="38" spans="1:11" ht="17.649999999999999">
+    <row r="36" spans="1:11" ht="15" thickTop="1" x14ac:dyDescent="0.3"/>
+    <row r="38" spans="1:11" ht="18" x14ac:dyDescent="0.35">
       <c r="A38" s="2" t="s">
         <v>13</v>
       </c>
     </row>
-    <row r="39" spans="1:11" ht="13.9" thickBot="1"/>
-    <row r="40" spans="1:11" ht="14.65" thickTop="1" thickBot="1">
+    <row r="39" spans="1:11" ht="15" thickBot="1" x14ac:dyDescent="0.35"/>
+    <row r="40" spans="1:11" ht="15.6" thickTop="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A40" s="3" t="s">
         <v>0</v>
       </c>
@@ -2619,7 +2765,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="41" spans="1:11" ht="13.9" thickTop="1">
+    <row r="41" spans="1:11" ht="15" thickTop="1" x14ac:dyDescent="0.3">
       <c r="A41" s="4" t="s">
         <v>14</v>
       </c>
@@ -2654,7 +2800,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="42" spans="1:11">
+    <row r="42" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A42" s="44" t="s">
         <v>39</v>
       </c>
@@ -2689,7 +2835,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="43" spans="1:11">
+    <row r="43" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A43" s="7" t="s">
         <v>15</v>
       </c>
@@ -2725,7 +2871,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="44" spans="1:11">
+    <row r="44" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A44" s="7" t="s">
         <v>16</v>
       </c>
@@ -2765,7 +2911,7 @@
         <v>108</v>
       </c>
     </row>
-    <row r="45" spans="1:11">
+    <row r="45" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A45" s="7" t="s">
         <v>17</v>
       </c>
@@ -2805,7 +2951,7 @@
         <v>109</v>
       </c>
     </row>
-    <row r="46" spans="1:11">
+    <row r="46" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A46" s="38" t="s">
         <v>46</v>
       </c>
@@ -2845,7 +2991,7 @@
         <v>110</v>
       </c>
     </row>
-    <row r="47" spans="1:11">
+    <row r="47" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A47" s="38" t="s">
         <v>45</v>
       </c>
@@ -2885,7 +3031,7 @@
         <v>111</v>
       </c>
     </row>
-    <row r="48" spans="1:11">
+    <row r="48" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A48" s="7" t="s">
         <v>18</v>
       </c>
@@ -2915,7 +3061,7 @@
       </c>
       <c r="K48" s="23"/>
     </row>
-    <row r="49" spans="1:14">
+    <row r="49" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A49" s="7" t="s">
         <v>48</v>
       </c>
@@ -2955,7 +3101,7 @@
         <v>112</v>
       </c>
     </row>
-    <row r="50" spans="1:14">
+    <row r="50" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A50" s="7" t="s">
         <v>153</v>
       </c>
@@ -2995,7 +3141,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="51" spans="1:14">
+    <row r="51" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A51" s="7" t="s">
         <v>47</v>
       </c>
@@ -3035,7 +3181,7 @@
         <v>113</v>
       </c>
     </row>
-    <row r="52" spans="1:14">
+    <row r="52" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A52" s="27" t="s">
         <v>49</v>
       </c>
@@ -3075,7 +3221,7 @@
         <v>114</v>
       </c>
     </row>
-    <row r="53" spans="1:14">
+    <row r="53" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A53" s="27" t="s">
         <v>51</v>
       </c>
@@ -3115,7 +3261,7 @@
         <v>115</v>
       </c>
     </row>
-    <row r="54" spans="1:14">
+    <row r="54" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A54" s="27" t="s">
         <v>50</v>
       </c>
@@ -3155,7 +3301,7 @@
         <v>116</v>
       </c>
     </row>
-    <row r="55" spans="1:14">
+    <row r="55" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A55" s="7" t="s">
         <v>52</v>
       </c>
@@ -3190,7 +3336,7 @@
         <v>117</v>
       </c>
     </row>
-    <row r="56" spans="1:14">
+    <row r="56" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A56" s="27" t="s">
         <v>53</v>
       </c>
@@ -3234,7 +3380,7 @@
         <v>156</v>
       </c>
     </row>
-    <row r="57" spans="1:14" ht="13.9" thickBot="1">
+    <row r="57" spans="1:14" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A57" s="10" t="s">
         <v>54</v>
       </c>
@@ -3274,20 +3420,20 @@
         <v>119</v>
       </c>
     </row>
-    <row r="58" spans="1:14" ht="13.9" thickTop="1">
+    <row r="58" spans="1:14" ht="15" thickTop="1" x14ac:dyDescent="0.3">
       <c r="B58" s="32"/>
       <c r="C58" s="33"/>
     </row>
-    <row r="59" spans="1:14">
+    <row r="59" spans="1:14" x14ac:dyDescent="0.3">
       <c r="B59" s="32"/>
       <c r="C59" s="33"/>
     </row>
-    <row r="60" spans="1:14" ht="17.649999999999999">
+    <row r="60" spans="1:14" ht="18" x14ac:dyDescent="0.35">
       <c r="A60" s="2" t="s">
         <v>19</v>
       </c>
     </row>
-    <row r="62" spans="1:14" ht="14.25" thickBot="1">
+    <row r="62" spans="1:14" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A62" s="113" t="s">
         <v>0</v>
       </c>
@@ -3320,7 +3466,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="63" spans="1:14" ht="13.9" thickTop="1">
+    <row r="63" spans="1:14" ht="15" thickTop="1" x14ac:dyDescent="0.3">
       <c r="A63" s="7" t="s">
         <v>16</v>
       </c>
@@ -3360,7 +3506,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="64" spans="1:14">
+    <row r="64" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A64" s="7" t="s">
         <v>17</v>
       </c>
@@ -3390,7 +3536,7 @@
       </c>
       <c r="K64" s="23"/>
     </row>
-    <row r="65" spans="1:12">
+    <row r="65" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A65" s="38" t="s">
         <v>158</v>
       </c>
@@ -3425,7 +3571,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="66" spans="1:12">
+    <row r="66" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A66" s="38" t="s">
         <v>159</v>
       </c>
@@ -3460,7 +3606,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="67" spans="1:12">
+    <row r="67" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A67" s="7" t="s">
         <v>18</v>
       </c>
@@ -3485,7 +3631,7 @@
       </c>
       <c r="K67" s="23"/>
     </row>
-    <row r="68" spans="1:12">
+    <row r="68" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A68" s="38" t="s">
         <v>45</v>
       </c>
@@ -3525,7 +3671,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="69" spans="1:12">
+    <row r="69" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A69" s="7" t="s">
         <v>48</v>
       </c>
@@ -3560,7 +3706,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="70" spans="1:12">
+    <row r="70" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A70" s="7" t="s">
         <v>47</v>
       </c>
@@ -3596,7 +3742,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="71" spans="1:12">
+    <row r="71" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A71" s="27" t="s">
         <v>49</v>
       </c>
@@ -3631,7 +3777,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="72" spans="1:12">
+    <row r="72" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A72" s="27" t="s">
         <v>51</v>
       </c>
@@ -3666,7 +3812,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="73" spans="1:12">
+    <row r="73" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A73" s="27" t="s">
         <v>50</v>
       </c>
@@ -3702,7 +3848,7 @@
       </c>
       <c r="L73" s="106"/>
     </row>
-    <row r="74" spans="1:12">
+    <row r="74" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A74" s="7" t="s">
         <v>52</v>
       </c>
@@ -3737,7 +3883,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="75" spans="1:12">
+    <row r="75" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A75" s="27" t="s">
         <v>53</v>
       </c>
@@ -3772,7 +3918,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="76" spans="1:12" ht="13.9" thickBot="1">
+    <row r="76" spans="1:12" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A76" s="115" t="s">
         <v>54</v>
       </c>
@@ -3808,14 +3954,14 @@
         <v>160</v>
       </c>
     </row>
-    <row r="77" spans="1:12" ht="13.9" thickTop="1"/>
-    <row r="79" spans="1:12" ht="17.649999999999999">
+    <row r="77" spans="1:12" ht="15" thickTop="1" x14ac:dyDescent="0.3"/>
+    <row r="79" spans="1:12" ht="18" x14ac:dyDescent="0.35">
       <c r="A79" s="2" t="s">
         <v>22</v>
       </c>
     </row>
-    <row r="80" spans="1:12" ht="13.9" thickBot="1"/>
-    <row r="81" spans="1:3" ht="14.65" thickTop="1" thickBot="1">
+    <row r="80" spans="1:12" ht="15" thickBot="1" x14ac:dyDescent="0.35"/>
+    <row r="81" spans="1:3" ht="15.6" thickTop="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A81" s="3" t="s">
         <v>0</v>
       </c>
@@ -3826,7 +3972,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="82" spans="1:3" ht="13.9" thickTop="1">
+    <row r="82" spans="1:3" ht="15" thickTop="1" x14ac:dyDescent="0.3">
       <c r="A82" s="4" t="s">
         <v>122</v>
       </c>
@@ -3837,7 +3983,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="83" spans="1:3">
+    <row r="83" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A83" s="15" t="s">
         <v>123</v>
       </c>
@@ -3848,7 +3994,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="84" spans="1:3">
+    <row r="84" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A84" s="15" t="s">
         <v>23</v>
       </c>
@@ -3859,7 +4005,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="85" spans="1:3" ht="15">
+    <row r="85" spans="1:3" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A85" s="52" t="s">
         <v>128</v>
       </c>
@@ -3870,7 +4016,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="86" spans="1:3">
+    <row r="86" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A86" s="52" t="s">
         <v>127</v>
       </c>
@@ -3881,7 +4027,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="87" spans="1:3">
+    <row r="87" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A87" s="52" t="s">
         <v>126</v>
       </c>
@@ -3892,7 +4038,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="88" spans="1:3">
+    <row r="88" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A88" s="52" t="s">
         <v>125</v>
       </c>
@@ -3903,7 +4049,7 @@
         <v>132</v>
       </c>
     </row>
-    <row r="89" spans="1:3">
+    <row r="89" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A89" s="52" t="s">
         <v>129</v>
       </c>
@@ -3914,7 +4060,7 @@
         <v>191</v>
       </c>
     </row>
-    <row r="90" spans="1:3">
+    <row r="90" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A90" s="52" t="s">
         <v>130</v>
       </c>
@@ -3925,7 +4071,7 @@
         <v>192</v>
       </c>
     </row>
-    <row r="91" spans="1:3">
+    <row r="91" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A91" s="52" t="s">
         <v>131</v>
       </c>
@@ -3936,7 +4082,7 @@
         <v>133</v>
       </c>
     </row>
-    <row r="92" spans="1:3">
+    <row r="92" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A92" s="52" t="s">
         <v>27</v>
       </c>
@@ -3947,7 +4093,7 @@
         <v>134</v>
       </c>
     </row>
-    <row r="93" spans="1:3">
+    <row r="93" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A93" s="52" t="s">
         <v>28</v>
       </c>
@@ -3958,7 +4104,7 @@
         <v>135</v>
       </c>
     </row>
-    <row r="94" spans="1:3">
+    <row r="94" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A94" s="52" t="s">
         <v>124</v>
       </c>
@@ -3969,7 +4115,7 @@
         <v>136</v>
       </c>
     </row>
-    <row r="95" spans="1:3">
+    <row r="95" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A95" s="15" t="s">
         <v>120</v>
       </c>
@@ -3980,7 +4126,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="96" spans="1:3">
+    <row r="96" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A96" s="15" t="s">
         <v>121</v>
       </c>
@@ -3991,7 +4137,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="97" spans="1:11">
+    <row r="97" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A97" s="52" t="s">
         <v>163</v>
       </c>
@@ -4002,7 +4148,7 @@
         <v>162</v>
       </c>
     </row>
-    <row r="98" spans="1:11">
+    <row r="98" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A98" s="15" t="s">
         <v>30</v>
       </c>
@@ -4011,7 +4157,7 @@
       </c>
       <c r="C98" s="18"/>
     </row>
-    <row r="99" spans="1:11" ht="13.9" thickBot="1">
+    <row r="99" spans="1:11" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A99" s="10" t="s">
         <v>31</v>
       </c>
@@ -4020,14 +4166,14 @@
       </c>
       <c r="C99" s="19"/>
     </row>
-    <row r="100" spans="1:11" ht="13.9" thickTop="1"/>
-    <row r="102" spans="1:11" ht="17.649999999999999">
+    <row r="100" spans="1:11" ht="15" thickTop="1" x14ac:dyDescent="0.3"/>
+    <row r="102" spans="1:11" ht="18" x14ac:dyDescent="0.35">
       <c r="A102" s="2" t="s">
         <v>32</v>
       </c>
     </row>
-    <row r="103" spans="1:11" ht="13.9" thickBot="1"/>
-    <row r="104" spans="1:11" ht="14.65" thickTop="1" thickBot="1">
+    <row r="103" spans="1:11" ht="15" thickBot="1" x14ac:dyDescent="0.35"/>
+    <row r="104" spans="1:11" ht="15.6" thickTop="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A104" s="3" t="s">
         <v>0</v>
       </c>
@@ -4058,7 +4204,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="105" spans="1:11" ht="13.9" thickTop="1">
+    <row r="105" spans="1:11" ht="15" thickTop="1" x14ac:dyDescent="0.3">
       <c r="A105" s="7" t="s">
         <v>16</v>
       </c>
@@ -4097,7 +4243,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="106" spans="1:11">
+    <row r="106" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A106" s="7" t="s">
         <v>33</v>
       </c>
@@ -4132,7 +4278,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="107" spans="1:11">
+    <row r="107" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A107" s="38" t="s">
         <v>161</v>
       </c>
@@ -4167,7 +4313,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="108" spans="1:11" ht="13.9" thickBot="1">
+    <row r="108" spans="1:11" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A108" s="10" t="s">
         <v>34</v>
       </c>
@@ -4202,14 +4348,14 @@
         <v>35</v>
       </c>
     </row>
-    <row r="109" spans="1:11" ht="13.9" thickTop="1"/>
-    <row r="111" spans="1:11" ht="17.649999999999999">
+    <row r="109" spans="1:11" ht="15" thickTop="1" x14ac:dyDescent="0.3"/>
+    <row r="111" spans="1:11" ht="18" x14ac:dyDescent="0.35">
       <c r="A111" s="2" t="s">
         <v>164</v>
       </c>
     </row>
-    <row r="112" spans="1:11" ht="13.9" thickBot="1"/>
-    <row r="113" spans="1:8" ht="14.65" thickTop="1" thickBot="1">
+    <row r="112" spans="1:11" ht="15" thickBot="1" x14ac:dyDescent="0.35"/>
+    <row r="113" spans="1:8" ht="15.6" thickTop="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A113" s="3" t="s">
         <v>0</v>
       </c>
@@ -4229,7 +4375,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="114" spans="1:8" ht="13.9" thickTop="1">
+    <row r="114" spans="1:8" ht="15" thickTop="1" x14ac:dyDescent="0.3">
       <c r="A114" s="38" t="s">
         <v>165</v>
       </c>
@@ -4249,7 +4395,7 @@
         <v>185</v>
       </c>
     </row>
-    <row r="115" spans="1:8">
+    <row r="115" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A115" s="38" t="s">
         <v>172</v>
       </c>
@@ -4269,7 +4415,7 @@
         <v>185</v>
       </c>
     </row>
-    <row r="116" spans="1:8">
+    <row r="116" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A116" s="38" t="s">
         <v>178</v>
       </c>
@@ -4289,7 +4435,7 @@
         <v>184</v>
       </c>
     </row>
-    <row r="117" spans="1:8" ht="13.9" thickBot="1">
+    <row r="117" spans="1:8" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A117" s="85" t="s">
         <v>170</v>
       </c>
@@ -4309,7 +4455,7 @@
         <v>177</v>
       </c>
     </row>
-    <row r="118" spans="1:8" ht="14.25" thickTop="1" thickBot="1">
+    <row r="118" spans="1:8" ht="15.6" thickTop="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A118" s="85" t="s">
         <v>186</v>
       </c>
@@ -4329,69 +4475,69 @@
         <v>189</v>
       </c>
     </row>
-    <row r="119" spans="1:8" ht="13.9" thickTop="1"/>
-    <row r="120" spans="1:8" ht="13.9">
-      <c r="A120" s="131" t="s">
+    <row r="119" spans="1:8" ht="15" thickTop="1" x14ac:dyDescent="0.3"/>
+    <row r="120" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A120" s="129" t="s">
         <v>214</v>
       </c>
     </row>
-    <row r="121" spans="1:8">
-      <c r="A121" s="132" t="s">
+    <row r="121" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A121" s="130" t="s">
         <v>207</v>
       </c>
       <c r="B121" t="s">
         <v>204</v>
       </c>
     </row>
-    <row r="122" spans="1:8">
-      <c r="A122" s="132" t="s">
+    <row r="122" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A122" s="130" t="s">
         <v>206</v>
       </c>
     </row>
-    <row r="123" spans="1:8">
-      <c r="A123" s="132" t="s">
+    <row r="123" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A123" s="130" t="s">
         <v>208</v>
       </c>
       <c r="B123" t="s">
         <v>205</v>
       </c>
     </row>
-    <row r="124" spans="1:8">
-      <c r="A124" s="132" t="s">
+    <row r="124" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A124" s="130" t="s">
         <v>210</v>
       </c>
       <c r="B124" t="s">
         <v>209</v>
       </c>
     </row>
-    <row r="125" spans="1:8" ht="13.9">
-      <c r="A125" s="131" t="s">
+    <row r="125" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A125" s="129" t="s">
         <v>215</v>
       </c>
     </row>
-    <row r="126" spans="1:8">
-      <c r="A126" s="132" t="s">
+    <row r="126" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A126" s="130" t="s">
         <v>211</v>
       </c>
       <c r="B126" t="s">
         <v>213</v>
       </c>
     </row>
-    <row r="127" spans="1:8">
-      <c r="A127" s="132" t="s">
+    <row r="127" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A127" s="130" t="s">
         <v>212</v>
       </c>
     </row>
-    <row r="128" spans="1:8">
-      <c r="A128" s="132" t="s">
+    <row r="128" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A128" s="130" t="s">
         <v>216</v>
       </c>
       <c r="B128" t="s">
         <v>217</v>
       </c>
     </row>
-    <row r="129" spans="1:2">
-      <c r="A129" s="132" t="s">
+    <row r="129" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A129" s="130" t="s">
         <v>218</v>
       </c>
       <c r="B129" t="s">
@@ -4409,24 +4555,24 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{3F74A05D-7210-44AC-859D-2846F0884F7B}">
   <dimension ref="A1:G56"/>
-  <sheetFormatPr defaultColWidth="12" defaultRowHeight="13.5"/>
+  <sheetFormatPr defaultColWidth="12" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="24.4375" customWidth="1"/>
-    <col min="2" max="9" width="12.875" customWidth="1"/>
+    <col min="1" max="1" width="24.44140625" customWidth="1"/>
+    <col min="2" max="9" width="12.88671875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5" ht="20.65">
+    <row r="1" spans="1:5" ht="21" x14ac:dyDescent="0.4">
       <c r="A1" s="1" t="s">
         <v>90</v>
       </c>
     </row>
-    <row r="3" spans="1:5" ht="17.649999999999999">
+    <row r="3" spans="1:5" ht="18" x14ac:dyDescent="0.35">
       <c r="A3" s="2" t="s">
         <v>61</v>
       </c>
     </row>
-    <row r="4" spans="1:5" ht="13.9" thickBot="1"/>
-    <row r="5" spans="1:5" ht="14.65" thickTop="1" thickBot="1">
+    <row r="4" spans="1:5" ht="15" thickBot="1" x14ac:dyDescent="0.35"/>
+    <row r="5" spans="1:5" ht="15.6" thickTop="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A5" s="3" t="s">
         <v>0</v>
       </c>
@@ -4438,7 +4584,7 @@
       </c>
       <c r="E5" s="73"/>
     </row>
-    <row r="6" spans="1:5" ht="13.9" thickTop="1">
+    <row r="6" spans="1:5" ht="15" thickTop="1" x14ac:dyDescent="0.3">
       <c r="A6" s="37" t="s">
         <v>101</v>
       </c>
@@ -4450,7 +4596,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="7" spans="1:5">
+    <row r="7" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A7" s="38" t="s">
         <v>92</v>
       </c>
@@ -4462,7 +4608,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="8" spans="1:5">
+    <row r="8" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A8" s="38" t="s">
         <v>93</v>
       </c>
@@ -4474,7 +4620,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="9" spans="1:5">
+    <row r="9" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A9" s="38" t="s">
         <v>91</v>
       </c>
@@ -4486,7 +4632,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="10" spans="1:5">
+    <row r="10" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A10" s="7" t="s">
         <v>62</v>
       </c>
@@ -4497,7 +4643,7 @@
         <v>63</v>
       </c>
     </row>
-    <row r="11" spans="1:5" ht="13.9" thickBot="1">
+    <row r="11" spans="1:5" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A11" s="10" t="s">
         <v>5</v>
       </c>
@@ -4509,18 +4655,18 @@
         <v>6</v>
       </c>
     </row>
-    <row r="12" spans="1:5" ht="15.4" thickTop="1">
+    <row r="12" spans="1:5" ht="16.2" thickTop="1" x14ac:dyDescent="0.3">
       <c r="A12" s="13"/>
     </row>
-    <row r="14" spans="1:5" ht="17.649999999999999">
+    <row r="14" spans="1:5" ht="18" x14ac:dyDescent="0.35">
       <c r="A14" s="2" t="s">
         <v>64</v>
       </c>
     </row>
-    <row r="15" spans="1:5" ht="18" thickBot="1">
+    <row r="15" spans="1:5" ht="18.600000000000001" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A15" s="2"/>
     </row>
-    <row r="16" spans="1:5" ht="14.65" thickTop="1" thickBot="1">
+    <row r="16" spans="1:5" ht="15.6" thickTop="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A16" s="3" t="s">
         <v>0</v>
       </c>
@@ -4531,7 +4677,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="17" spans="1:3" ht="13.9" thickTop="1">
+    <row r="17" spans="1:3" ht="15" thickTop="1" x14ac:dyDescent="0.3">
       <c r="A17" s="59" t="s">
         <v>65</v>
       </c>
@@ -4540,7 +4686,7 @@
       </c>
       <c r="C17" s="61"/>
     </row>
-    <row r="18" spans="1:3">
+    <row r="18" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A18" s="62" t="s">
         <v>67</v>
       </c>
@@ -4549,7 +4695,7 @@
       </c>
       <c r="C18" s="64"/>
     </row>
-    <row r="19" spans="1:3">
+    <row r="19" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A19" s="62" t="s">
         <v>69</v>
       </c>
@@ -4560,7 +4706,7 @@
         <v>70</v>
       </c>
     </row>
-    <row r="20" spans="1:3">
+    <row r="20" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A20" s="62" t="s">
         <v>71</v>
       </c>
@@ -4571,7 +4717,7 @@
         <v>72</v>
       </c>
     </row>
-    <row r="21" spans="1:3">
+    <row r="21" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A21" s="62" t="s">
         <v>73</v>
       </c>
@@ -4582,7 +4728,7 @@
         <v>74</v>
       </c>
     </row>
-    <row r="22" spans="1:3">
+    <row r="22" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A22" s="62" t="s">
         <v>75</v>
       </c>
@@ -4593,7 +4739,7 @@
         <v>70</v>
       </c>
     </row>
-    <row r="23" spans="1:3">
+    <row r="23" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A23" s="62" t="s">
         <v>76</v>
       </c>
@@ -4604,7 +4750,7 @@
         <v>72</v>
       </c>
     </row>
-    <row r="24" spans="1:3">
+    <row r="24" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A24" s="62" t="s">
         <v>77</v>
       </c>
@@ -4616,7 +4762,7 @@
         <v>78</v>
       </c>
     </row>
-    <row r="25" spans="1:3">
+    <row r="25" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A25" s="62" t="s">
         <v>79</v>
       </c>
@@ -4628,7 +4774,7 @@
         <v>80</v>
       </c>
     </row>
-    <row r="26" spans="1:3">
+    <row r="26" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A26" s="67" t="s">
         <v>81</v>
       </c>
@@ -4636,7 +4782,7 @@
         <v>1510</v>
       </c>
     </row>
-    <row r="27" spans="1:3" ht="13.9" thickBot="1">
+    <row r="27" spans="1:3" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A27" s="68" t="s">
         <v>82</v>
       </c>
@@ -4645,14 +4791,14 @@
       </c>
       <c r="C27" s="70"/>
     </row>
-    <row r="28" spans="1:3" ht="13.9" thickTop="1"/>
-    <row r="30" spans="1:3" ht="17.649999999999999">
+    <row r="28" spans="1:3" ht="15" thickTop="1" x14ac:dyDescent="0.3"/>
+    <row r="30" spans="1:3" ht="18" x14ac:dyDescent="0.35">
       <c r="A30" s="2" t="s">
         <v>83</v>
       </c>
     </row>
-    <row r="31" spans="1:3" ht="13.9" thickBot="1"/>
-    <row r="32" spans="1:3" ht="14.65" thickTop="1" thickBot="1">
+    <row r="31" spans="1:3" ht="15" thickBot="1" x14ac:dyDescent="0.35"/>
+    <row r="32" spans="1:3" ht="15.6" thickTop="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A32" s="3" t="s">
         <v>0</v>
       </c>
@@ -4663,7 +4809,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="33" spans="1:7" ht="13.9" thickTop="1">
+    <row r="33" spans="1:7" ht="15" thickTop="1" x14ac:dyDescent="0.3">
       <c r="A33" s="59" t="s">
         <v>84</v>
       </c>
@@ -4675,7 +4821,7 @@
       </c>
       <c r="G33" s="73"/>
     </row>
-    <row r="34" spans="1:7">
+    <row r="34" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A34" s="74" t="s">
         <v>195</v>
       </c>
@@ -4688,7 +4834,7 @@
       </c>
       <c r="G34" s="73"/>
     </row>
-    <row r="35" spans="1:7">
+    <row r="35" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A35" s="74" t="s">
         <v>85</v>
       </c>
@@ -4702,7 +4848,7 @@
       <c r="F35" s="78"/>
       <c r="G35" s="73"/>
     </row>
-    <row r="36" spans="1:7" ht="15">
+    <row r="36" spans="1:7" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A36" s="74" t="s">
         <v>86</v>
       </c>
@@ -4715,7 +4861,7 @@
       <c r="F36" s="13"/>
       <c r="G36" s="13"/>
     </row>
-    <row r="37" spans="1:7">
+    <row r="37" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A37" s="74" t="s">
         <v>87</v>
       </c>
@@ -4727,7 +4873,7 @@
         <v>141</v>
       </c>
     </row>
-    <row r="38" spans="1:7">
+    <row r="38" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A38" s="81" t="s">
         <v>95</v>
       </c>
@@ -4738,7 +4884,7 @@
         <v>72</v>
       </c>
     </row>
-    <row r="39" spans="1:7">
+    <row r="39" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A39" s="81" t="s">
         <v>94</v>
       </c>
@@ -4750,7 +4896,7 @@
         <v>142</v>
       </c>
     </row>
-    <row r="40" spans="1:7">
+    <row r="40" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A40" s="81" t="s">
         <v>194</v>
       </c>
@@ -4759,7 +4905,7 @@
       </c>
       <c r="C40" s="76"/>
     </row>
-    <row r="41" spans="1:7">
+    <row r="41" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A41" s="81" t="s">
         <v>96</v>
       </c>
@@ -4771,7 +4917,7 @@
         <v>143</v>
       </c>
     </row>
-    <row r="42" spans="1:7" ht="13.9" thickBot="1">
+    <row r="42" spans="1:7" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A42" s="83" t="s">
         <v>88</v>
       </c>
@@ -4783,7 +4929,7 @@
         <v>144</v>
       </c>
     </row>
-    <row r="43" spans="1:7" ht="13.9" thickTop="1">
+    <row r="43" spans="1:7" ht="15" thickTop="1" x14ac:dyDescent="0.3">
       <c r="A43" s="125" t="s">
         <v>198</v>
       </c>
@@ -4795,7 +4941,7 @@
         <v>199</v>
       </c>
     </row>
-    <row r="44" spans="1:7">
+    <row r="44" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A44" s="125" t="s">
         <v>196</v>
       </c>
@@ -4807,7 +4953,7 @@
         <v>200</v>
       </c>
     </row>
-    <row r="45" spans="1:7">
+    <row r="45" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A45" s="125" t="s">
         <v>197</v>
       </c>
@@ -4819,7 +4965,7 @@
         <v>201</v>
       </c>
     </row>
-    <row r="46" spans="1:7">
+    <row r="46" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A46" s="74" t="s">
         <v>193</v>
       </c>
@@ -4831,25 +4977,25 @@
         <v>202</v>
       </c>
     </row>
-    <row r="47" spans="1:7">
+    <row r="47" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A47" s="128" t="s">
         <v>203</v>
       </c>
-      <c r="B47" s="129">
+      <c r="B47" s="114">
         <f>B34*B40*B39/B27</f>
         <v>24.166097335306102</v>
       </c>
-      <c r="C47" s="130" t="s">
+      <c r="C47" s="127" t="s">
         <v>70</v>
       </c>
     </row>
-    <row r="49" spans="1:3" ht="17.649999999999999">
+    <row r="49" spans="1:3" ht="18" x14ac:dyDescent="0.35">
       <c r="A49" s="2" t="s">
         <v>97</v>
       </c>
     </row>
-    <row r="50" spans="1:3" ht="13.9" thickBot="1"/>
-    <row r="51" spans="1:3" ht="14.65" thickTop="1" thickBot="1">
+    <row r="50" spans="1:3" ht="15" thickBot="1" x14ac:dyDescent="0.35"/>
+    <row r="51" spans="1:3" ht="15.6" thickTop="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A51" s="3" t="s">
         <v>0</v>
       </c>
@@ -4860,7 +5006,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="52" spans="1:3" ht="13.9" thickTop="1">
+    <row r="52" spans="1:3" ht="15" thickTop="1" x14ac:dyDescent="0.3">
       <c r="A52" s="81" t="s">
         <v>98</v>
       </c>
@@ -4871,11 +5017,11 @@
         <v>89</v>
       </c>
     </row>
-    <row r="53" spans="1:3">
+    <row r="53" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A53" s="74" t="s">
         <v>85</v>
       </c>
-      <c r="B53" s="133">
+      <c r="B53" s="131">
         <f>(B52*B8)/(B34*B19)</f>
         <v>0.20769450283115989</v>
       </c>
@@ -4883,7 +5029,7 @@
         <v>63</v>
       </c>
     </row>
-    <row r="54" spans="1:3">
+    <row r="54" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A54" s="81" t="s">
         <v>145</v>
       </c>
@@ -4894,7 +5040,7 @@
         <v>100</v>
       </c>
     </row>
-    <row r="55" spans="1:3" ht="13.9" thickBot="1">
+    <row r="55" spans="1:3" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A55" s="82" t="s">
         <v>99</v>
       </c>
@@ -4905,10 +5051,592 @@
         <v>100</v>
       </c>
     </row>
-    <row r="56" spans="1:3" ht="13.9" thickTop="1"/>
+    <row r="56" spans="1:3" ht="15" thickTop="1" x14ac:dyDescent="0.3"/>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C64046B5-8416-4E54-8EA3-123308D3390B}">
+  <dimension ref="B2:Z20"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="3" max="3" width="9.88671875" customWidth="1"/>
+    <col min="5" max="5" width="10.5546875" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="2" spans="2:25" x14ac:dyDescent="0.3">
+      <c r="B2" s="129" t="s">
+        <v>231</v>
+      </c>
+    </row>
+    <row r="3" spans="2:25" x14ac:dyDescent="0.3">
+      <c r="B3" t="s">
+        <v>226</v>
+      </c>
+      <c r="D3" t="s">
+        <v>230</v>
+      </c>
+      <c r="G3" t="s">
+        <v>222</v>
+      </c>
+      <c r="K3" t="s">
+        <v>237</v>
+      </c>
+    </row>
+    <row r="4" spans="2:25" x14ac:dyDescent="0.3">
+      <c r="B4">
+        <v>5</v>
+      </c>
+      <c r="C4" t="s">
+        <v>227</v>
+      </c>
+      <c r="D4" s="129">
+        <v>5.6</v>
+      </c>
+      <c r="E4" t="s">
+        <v>227</v>
+      </c>
+      <c r="G4" s="129" t="s">
+        <v>223</v>
+      </c>
+      <c r="K4" t="s">
+        <v>238</v>
+      </c>
+    </row>
+    <row r="5" spans="2:25" x14ac:dyDescent="0.3">
+      <c r="B5">
+        <v>10</v>
+      </c>
+      <c r="C5" t="s">
+        <v>227</v>
+      </c>
+      <c r="D5" s="129">
+        <v>10</v>
+      </c>
+      <c r="E5" t="s">
+        <v>227</v>
+      </c>
+      <c r="G5" t="s">
+        <v>224</v>
+      </c>
+      <c r="K5" t="s">
+        <v>239</v>
+      </c>
+    </row>
+    <row r="6" spans="2:25" x14ac:dyDescent="0.3">
+      <c r="B6">
+        <v>15</v>
+      </c>
+      <c r="C6" t="s">
+        <v>227</v>
+      </c>
+      <c r="D6">
+        <v>15</v>
+      </c>
+      <c r="G6" t="s">
+        <v>225</v>
+      </c>
+      <c r="K6" t="s">
+        <v>240</v>
+      </c>
+    </row>
+    <row r="7" spans="2:25" x14ac:dyDescent="0.3">
+      <c r="B7">
+        <v>20</v>
+      </c>
+      <c r="D7" s="129">
+        <v>22</v>
+      </c>
+      <c r="E7" t="s">
+        <v>227</v>
+      </c>
+      <c r="K7" t="s">
+        <v>241</v>
+      </c>
+    </row>
+    <row r="8" spans="2:25" x14ac:dyDescent="0.3">
+      <c r="B8">
+        <v>25</v>
+      </c>
+      <c r="C8" t="s">
+        <v>227</v>
+      </c>
+      <c r="D8">
+        <v>27</v>
+      </c>
+      <c r="G8" t="s">
+        <v>259</v>
+      </c>
+    </row>
+    <row r="9" spans="2:25" x14ac:dyDescent="0.3">
+      <c r="B9">
+        <v>30</v>
+      </c>
+      <c r="C9" t="s">
+        <v>227</v>
+      </c>
+      <c r="D9">
+        <v>33</v>
+      </c>
+      <c r="G9" t="s">
+        <v>260</v>
+      </c>
+      <c r="K9" t="s">
+        <v>242</v>
+      </c>
+    </row>
+    <row r="10" spans="2:25" x14ac:dyDescent="0.3">
+      <c r="B10">
+        <v>35</v>
+      </c>
+      <c r="D10" s="129">
+        <v>33</v>
+      </c>
+      <c r="E10" t="s">
+        <v>227</v>
+      </c>
+      <c r="G10" t="s">
+        <v>261</v>
+      </c>
+      <c r="K10" t="s">
+        <v>243</v>
+      </c>
+    </row>
+    <row r="11" spans="2:25" x14ac:dyDescent="0.3">
+      <c r="B11">
+        <v>40</v>
+      </c>
+      <c r="C11" t="s">
+        <v>227</v>
+      </c>
+      <c r="D11">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="12" spans="2:25" x14ac:dyDescent="0.3">
+      <c r="B12">
+        <v>45</v>
+      </c>
+      <c r="C12" t="s">
+        <v>227</v>
+      </c>
+      <c r="D12">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="13" spans="2:25" x14ac:dyDescent="0.3">
+      <c r="B13">
+        <v>50</v>
+      </c>
+      <c r="C13" t="s">
+        <v>227</v>
+      </c>
+      <c r="D13" s="129">
+        <v>47</v>
+      </c>
+      <c r="E13" t="s">
+        <v>227</v>
+      </c>
+    </row>
+    <row r="15" spans="2:25" x14ac:dyDescent="0.3">
+      <c r="B15" s="135" t="s">
+        <v>232</v>
+      </c>
+      <c r="C15" s="135" t="s">
+        <v>252</v>
+      </c>
+      <c r="D15" s="135"/>
+      <c r="E15" s="135"/>
+      <c r="G15" s="135" t="s">
+        <v>233</v>
+      </c>
+      <c r="H15" s="135" t="s">
+        <v>251</v>
+      </c>
+      <c r="I15" s="135"/>
+      <c r="J15" s="135"/>
+      <c r="L15" s="135" t="s">
+        <v>234</v>
+      </c>
+      <c r="M15" s="135" t="s">
+        <v>254</v>
+      </c>
+      <c r="N15" s="135"/>
+      <c r="O15" s="135"/>
+      <c r="Q15" s="135" t="s">
+        <v>235</v>
+      </c>
+      <c r="R15" s="135" t="s">
+        <v>258</v>
+      </c>
+      <c r="S15" s="135"/>
+      <c r="T15" s="135"/>
+      <c r="V15" s="135" t="s">
+        <v>236</v>
+      </c>
+      <c r="W15" s="135" t="s">
+        <v>250</v>
+      </c>
+      <c r="X15" s="135"/>
+      <c r="Y15" s="135"/>
+    </row>
+    <row r="16" spans="2:25" x14ac:dyDescent="0.3">
+      <c r="B16" s="134" t="s">
+        <v>220</v>
+      </c>
+      <c r="C16" s="136">
+        <v>2.5</v>
+      </c>
+      <c r="D16" s="136">
+        <v>3</v>
+      </c>
+      <c r="E16" s="136">
+        <v>3.5</v>
+      </c>
+      <c r="G16" s="134" t="s">
+        <v>220</v>
+      </c>
+      <c r="H16" s="136">
+        <v>2.5</v>
+      </c>
+      <c r="I16" s="136">
+        <v>3</v>
+      </c>
+      <c r="J16" s="136">
+        <v>3.5</v>
+      </c>
+      <c r="L16" s="134" t="s">
+        <v>220</v>
+      </c>
+      <c r="M16" s="136">
+        <v>2.5</v>
+      </c>
+      <c r="N16" s="136">
+        <v>3</v>
+      </c>
+      <c r="O16" s="136">
+        <v>3.5</v>
+      </c>
+      <c r="Q16" s="134" t="s">
+        <v>220</v>
+      </c>
+      <c r="R16" s="136">
+        <v>2.5</v>
+      </c>
+      <c r="S16" s="136">
+        <v>3</v>
+      </c>
+      <c r="T16" s="136">
+        <v>3.5</v>
+      </c>
+      <c r="V16" s="134" t="s">
+        <v>220</v>
+      </c>
+      <c r="W16" s="136">
+        <v>2.5</v>
+      </c>
+      <c r="X16" s="136">
+        <v>3</v>
+      </c>
+      <c r="Y16" s="136">
+        <v>3.5</v>
+      </c>
+    </row>
+    <row r="17" spans="2:26" x14ac:dyDescent="0.3">
+      <c r="B17" s="134" t="s">
+        <v>221</v>
+      </c>
+      <c r="C17" s="137">
+        <v>0.5</v>
+      </c>
+      <c r="D17" s="137">
+        <v>0.4</v>
+      </c>
+      <c r="E17" s="137">
+        <v>0.3</v>
+      </c>
+      <c r="G17" s="134" t="s">
+        <v>221</v>
+      </c>
+      <c r="H17" s="137">
+        <v>0.5</v>
+      </c>
+      <c r="I17" s="137">
+        <v>0.4</v>
+      </c>
+      <c r="J17" s="137">
+        <v>0.3</v>
+      </c>
+      <c r="L17" s="134" t="s">
+        <v>221</v>
+      </c>
+      <c r="M17" s="137">
+        <v>0.5</v>
+      </c>
+      <c r="N17" s="137">
+        <v>0.4</v>
+      </c>
+      <c r="O17" s="137">
+        <v>0.3</v>
+      </c>
+      <c r="Q17" s="134" t="s">
+        <v>221</v>
+      </c>
+      <c r="R17" s="137">
+        <v>0.5</v>
+      </c>
+      <c r="S17" s="137">
+        <v>0.4</v>
+      </c>
+      <c r="T17" s="137">
+        <v>0.3</v>
+      </c>
+      <c r="V17" s="134" t="s">
+        <v>221</v>
+      </c>
+      <c r="W17" s="137">
+        <v>0.5</v>
+      </c>
+      <c r="X17" s="137">
+        <v>0.4</v>
+      </c>
+      <c r="Y17" s="137">
+        <v>0.3</v>
+      </c>
+      <c r="Z17" s="132"/>
+    </row>
+    <row r="18" spans="2:26" x14ac:dyDescent="0.3">
+      <c r="B18" s="134" t="s">
+        <v>223</v>
+      </c>
+      <c r="C18" s="136" t="s">
+        <v>253</v>
+      </c>
+      <c r="D18" s="136">
+        <v>3.3</v>
+      </c>
+      <c r="E18" s="136">
+        <v>3.55</v>
+      </c>
+      <c r="G18" s="134" t="s">
+        <v>223</v>
+      </c>
+      <c r="H18" s="136" t="s">
+        <v>244</v>
+      </c>
+      <c r="I18" s="136" t="s">
+        <v>248</v>
+      </c>
+      <c r="J18" s="136" t="s">
+        <v>245</v>
+      </c>
+      <c r="L18" s="134" t="s">
+        <v>223</v>
+      </c>
+      <c r="M18" s="136" t="s">
+        <v>255</v>
+      </c>
+      <c r="N18" s="136" t="s">
+        <v>245</v>
+      </c>
+      <c r="O18" s="136" t="s">
+        <v>256</v>
+      </c>
+      <c r="Q18" s="134" t="s">
+        <v>223</v>
+      </c>
+      <c r="R18" s="136" t="s">
+        <v>256</v>
+      </c>
+      <c r="S18" s="136" t="s">
+        <v>257</v>
+      </c>
+      <c r="T18" s="136" t="s">
+        <v>247</v>
+      </c>
+      <c r="V18" s="134" t="s">
+        <v>223</v>
+      </c>
+      <c r="W18" s="136" t="s">
+        <v>247</v>
+      </c>
+      <c r="X18" s="136" t="s">
+        <v>249</v>
+      </c>
+      <c r="Y18" s="136" t="s">
+        <v>246</v>
+      </c>
+    </row>
+    <row r="20" spans="2:26" x14ac:dyDescent="0.3">
+      <c r="C20" s="133"/>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{859A8E3D-0A15-4683-B01F-C1772C7ACE06}">
+  <dimension ref="B2:G18"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetData>
+    <row r="2" spans="2:7" x14ac:dyDescent="0.3">
+      <c r="E2" t="s">
+        <v>229</v>
+      </c>
+    </row>
+    <row r="3" spans="2:7" x14ac:dyDescent="0.3">
+      <c r="B3" t="s">
+        <v>220</v>
+      </c>
+      <c r="C3" t="s">
+        <v>221</v>
+      </c>
+      <c r="E3" t="s">
+        <v>226</v>
+      </c>
+      <c r="G3" t="s">
+        <v>228</v>
+      </c>
+    </row>
+    <row r="4" spans="2:7" x14ac:dyDescent="0.3">
+      <c r="B4">
+        <v>2.5</v>
+      </c>
+      <c r="C4" s="133">
+        <v>0.5</v>
+      </c>
+      <c r="E4">
+        <v>5</v>
+      </c>
+      <c r="F4" t="s">
+        <v>227</v>
+      </c>
+      <c r="G4">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="5" spans="2:7" x14ac:dyDescent="0.3">
+      <c r="B5">
+        <v>2.75</v>
+      </c>
+      <c r="C5" s="133">
+        <v>0.45</v>
+      </c>
+      <c r="E5">
+        <v>10</v>
+      </c>
+      <c r="F5" t="s">
+        <v>227</v>
+      </c>
+      <c r="G5">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="6" spans="2:7" x14ac:dyDescent="0.3">
+      <c r="B6">
+        <v>3</v>
+      </c>
+      <c r="C6" s="133">
+        <v>0.4</v>
+      </c>
+      <c r="E6">
+        <v>15</v>
+      </c>
+      <c r="F6" t="s">
+        <v>227</v>
+      </c>
+    </row>
+    <row r="7" spans="2:7" x14ac:dyDescent="0.3">
+      <c r="B7">
+        <v>3.25</v>
+      </c>
+      <c r="C7" s="133">
+        <v>0.35</v>
+      </c>
+      <c r="E7">
+        <v>20</v>
+      </c>
+      <c r="G7">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="8" spans="2:7" x14ac:dyDescent="0.3">
+      <c r="B8">
+        <v>3.5</v>
+      </c>
+      <c r="C8" s="133">
+        <v>0.3</v>
+      </c>
+      <c r="E8">
+        <v>35</v>
+      </c>
+      <c r="F8" t="s">
+        <v>227</v>
+      </c>
+    </row>
+    <row r="9" spans="2:7" x14ac:dyDescent="0.3">
+      <c r="E9">
+        <v>30</v>
+      </c>
+      <c r="F9" t="s">
+        <v>227</v>
+      </c>
+    </row>
+    <row r="10" spans="2:7" x14ac:dyDescent="0.3">
+      <c r="E10">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="11" spans="2:7" x14ac:dyDescent="0.3">
+      <c r="E11">
+        <v>40</v>
+      </c>
+      <c r="F11" t="s">
+        <v>227</v>
+      </c>
+    </row>
+    <row r="12" spans="2:7" x14ac:dyDescent="0.3">
+      <c r="E12">
+        <v>45</v>
+      </c>
+      <c r="F12" t="s">
+        <v>227</v>
+      </c>
+    </row>
+    <row r="13" spans="2:7" x14ac:dyDescent="0.3">
+      <c r="E13">
+        <v>50</v>
+      </c>
+      <c r="F13" t="s">
+        <v>227</v>
+      </c>
+    </row>
+    <row r="15" spans="2:7" x14ac:dyDescent="0.3">
+      <c r="B15" t="s">
+        <v>222</v>
+      </c>
+    </row>
+    <row r="16" spans="2:7" x14ac:dyDescent="0.3">
+      <c r="B16" t="s">
+        <v>223</v>
+      </c>
+    </row>
+    <row r="17" spans="2:2" x14ac:dyDescent="0.3">
+      <c r="B17" t="s">
+        <v>224</v>
+      </c>
+    </row>
+    <row r="18" spans="2:2" x14ac:dyDescent="0.3">
+      <c r="B18" t="s">
+        <v>225</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
 

</xml_diff>

<commit_message>
Updated Excel sheet with slope compensation parameters.
</commit_message>
<xml_diff>
--- a/Excel/Boost Converter Design Params.xlsx
+++ b/Excel/Boost Converter Design Params.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\weiwi\OneDrive\Documents\GitHub\311\Excel\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{53354F8C-67C8-49BA-99E6-BFE737A9FF7B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{716A2018-3D68-4F68-9520-4E8D3019729C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-98" yWindow="-98" windowWidth="21795" windowHeight="12975" activeTab="1" xr2:uid="{0EA872C3-4804-43CB-9F0B-5F94DB7B4351}"/>
+    <workbookView xWindow="-98" yWindow="-98" windowWidth="21795" windowHeight="12975" xr2:uid="{0EA872C3-4804-43CB-9F0B-5F94DB7B4351}"/>
   </bookViews>
   <sheets>
     <sheet name="SS_Analysis" sheetId="1" r:id="rId1"/>
@@ -589,9 +589,6 @@
     <t>- To be done</t>
   </si>
   <si>
-    <t>fp = 1/2piRC @ 10kHz corner</t>
-  </si>
-  <si>
     <t>R21 = 37k, C12 = 3.3nF</t>
   </si>
   <si>
@@ -670,9 +667,6 @@
     <t>R7 limits current through IB/IC.</t>
   </si>
   <si>
-    <t>R7 = 200kOhms</t>
-  </si>
-  <si>
     <t>C13 = 10nF</t>
   </si>
   <si>
@@ -698,6 +692,12 @@
   </si>
   <si>
     <t xml:space="preserve">Limits current through IC. </t>
+  </si>
+  <si>
+    <t>fp = 1/2piRC @ 10MHz corner</t>
+  </si>
+  <si>
+    <t>R7 = 180kOhms</t>
   </si>
 </sst>
 </file>
@@ -3911,7 +3911,7 @@
         <v>39</v>
       </c>
       <c r="C89" s="18" t="s">
-        <v>191</v>
+        <v>190</v>
       </c>
     </row>
     <row r="90" spans="1:3">
@@ -3919,10 +3919,10 @@
         <v>130</v>
       </c>
       <c r="B90" s="16">
-        <v>140</v>
+        <v>150</v>
       </c>
       <c r="C90" s="18" t="s">
-        <v>192</v>
+        <v>191</v>
       </c>
     </row>
     <row r="91" spans="1:3">
@@ -4246,7 +4246,7 @@
       </c>
       <c r="G114" s="22"/>
       <c r="H114" s="22" t="s">
-        <v>185</v>
+        <v>184</v>
       </c>
     </row>
     <row r="115" spans="1:8">
@@ -4266,7 +4266,7 @@
       </c>
       <c r="G115" s="22"/>
       <c r="H115" s="22" t="s">
-        <v>185</v>
+        <v>184</v>
       </c>
     </row>
     <row r="116" spans="1:8">
@@ -4282,11 +4282,11 @@
       </c>
       <c r="E116" s="22"/>
       <c r="F116" s="22" t="s">
-        <v>183</v>
+        <v>218</v>
       </c>
       <c r="G116" s="22"/>
       <c r="H116" s="22" t="s">
-        <v>184</v>
+        <v>183</v>
       </c>
     </row>
     <row r="117" spans="1:8" ht="13.9" thickBot="1">
@@ -4311,91 +4311,91 @@
     </row>
     <row r="118" spans="1:8" ht="14.25" thickTop="1" thickBot="1">
       <c r="A118" s="85" t="s">
+        <v>185</v>
+      </c>
+      <c r="B118" s="100" t="s">
         <v>186</v>
-      </c>
-      <c r="B118" s="100" t="s">
-        <v>187</v>
       </c>
       <c r="C118" s="30"/>
       <c r="D118" s="30" t="s">
-        <v>188</v>
+        <v>187</v>
       </c>
       <c r="E118" s="30"/>
       <c r="F118" s="30" t="s">
-        <v>190</v>
+        <v>189</v>
       </c>
       <c r="G118" s="30"/>
       <c r="H118" s="30" t="s">
-        <v>189</v>
+        <v>188</v>
       </c>
     </row>
     <row r="119" spans="1:8" ht="13.9" thickTop="1"/>
     <row r="120" spans="1:8" ht="13.9">
       <c r="A120" s="131" t="s">
-        <v>214</v>
+        <v>212</v>
       </c>
     </row>
     <row r="121" spans="1:8">
       <c r="A121" s="132" t="s">
-        <v>207</v>
+        <v>206</v>
       </c>
       <c r="B121" t="s">
-        <v>204</v>
+        <v>203</v>
       </c>
     </row>
     <row r="122" spans="1:8">
       <c r="A122" s="132" t="s">
-        <v>206</v>
+        <v>205</v>
       </c>
     </row>
     <row r="123" spans="1:8">
       <c r="A123" s="132" t="s">
-        <v>208</v>
+        <v>207</v>
       </c>
       <c r="B123" t="s">
-        <v>205</v>
+        <v>204</v>
       </c>
     </row>
     <row r="124" spans="1:8">
       <c r="A124" s="132" t="s">
-        <v>210</v>
+        <v>219</v>
       </c>
       <c r="B124" t="s">
-        <v>209</v>
+        <v>208</v>
       </c>
     </row>
     <row r="125" spans="1:8" ht="13.9">
       <c r="A125" s="131" t="s">
-        <v>215</v>
+        <v>213</v>
       </c>
     </row>
     <row r="126" spans="1:8">
       <c r="A126" s="132" t="s">
+        <v>209</v>
+      </c>
+      <c r="B126" t="s">
         <v>211</v>
-      </c>
-      <c r="B126" t="s">
-        <v>213</v>
       </c>
     </row>
     <row r="127" spans="1:8">
       <c r="A127" s="132" t="s">
-        <v>212</v>
+        <v>210</v>
       </c>
     </row>
     <row r="128" spans="1:8">
       <c r="A128" s="132" t="s">
-        <v>216</v>
+        <v>214</v>
       </c>
       <c r="B128" t="s">
-        <v>217</v>
+        <v>215</v>
       </c>
     </row>
     <row r="129" spans="1:2">
       <c r="A129" s="132" t="s">
-        <v>218</v>
+        <v>216</v>
       </c>
       <c r="B129" t="s">
-        <v>219</v>
+        <v>217</v>
       </c>
     </row>
   </sheetData>
@@ -4677,7 +4677,7 @@
     </row>
     <row r="34" spans="1:7">
       <c r="A34" s="74" t="s">
-        <v>195</v>
+        <v>194</v>
       </c>
       <c r="B34" s="123">
         <f>ROUND(SQRT((2*B6*10^-6*B33*10^-3)/(B25*B19*10^-6)),0)</f>
@@ -4752,7 +4752,7 @@
     </row>
     <row r="40" spans="1:7">
       <c r="A40" s="81" t="s">
-        <v>194</v>
+        <v>193</v>
       </c>
       <c r="B40" s="80">
         <v>5</v>
@@ -4785,55 +4785,55 @@
     </row>
     <row r="43" spans="1:7" ht="13.9" thickTop="1">
       <c r="A43" s="125" t="s">
-        <v>198</v>
+        <v>197</v>
       </c>
       <c r="B43" s="126">
         <f>B35*10^3*SS_Analysis!F47/(2*B8)</f>
         <v>13.368479376977847</v>
       </c>
       <c r="C43" s="127" t="s">
-        <v>199</v>
+        <v>198</v>
       </c>
     </row>
     <row r="44" spans="1:7">
       <c r="A44" s="125" t="s">
-        <v>196</v>
+        <v>195</v>
       </c>
       <c r="B44" s="126">
         <f>1.71*10^-5*B11^1.12*B43^2.29</f>
         <v>1.1264811121722047</v>
       </c>
       <c r="C44" s="127" t="s">
-        <v>200</v>
+        <v>199</v>
       </c>
     </row>
     <row r="45" spans="1:7">
       <c r="A45" s="125" t="s">
-        <v>197</v>
+        <v>196</v>
       </c>
       <c r="B45" s="126">
         <f>(B44*10^3*B21*10^-9) + B42</f>
         <v>4.6890945111949675E-2</v>
       </c>
       <c r="C45" s="127" t="s">
-        <v>201</v>
+        <v>200</v>
       </c>
     </row>
     <row r="46" spans="1:7">
       <c r="A46" s="74" t="s">
-        <v>193</v>
+        <v>192</v>
       </c>
       <c r="B46" s="77">
         <f>B9/(B40*B39)</f>
         <v>2.0386837275999632</v>
       </c>
       <c r="C46" s="76" t="s">
-        <v>202</v>
+        <v>201</v>
       </c>
     </row>
     <row r="47" spans="1:7">
       <c r="A47" s="128" t="s">
-        <v>203</v>
+        <v>202</v>
       </c>
       <c r="B47" s="129">
         <f>B34*B40*B39/B27</f>

</xml_diff>

<commit_message>
Uploaded test values for breadboarding in open loop
</commit_message>
<xml_diff>
--- a/Excel/Boost Converter Design Params.xlsx
+++ b/Excel/Boost Converter Design Params.xlsx
@@ -1,20 +1,21 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="24334"/>
-  <workbookPr/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30430"/>
+  <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\weiwi\OneDrive\Documents\GitHub\311\Excel\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\tytom\Documents\GitHub\311\Excel\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{716A2018-3D68-4F68-9520-4E8D3019729C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8FA943A1-BAC0-4164-9636-0C29EC94EDB1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-98" yWindow="-98" windowWidth="21795" windowHeight="12975" xr2:uid="{0EA872C3-4804-43CB-9F0B-5F94DB7B4351}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="2" xr2:uid="{0EA872C3-4804-43CB-9F0B-5F94DB7B4351}"/>
   </bookViews>
   <sheets>
     <sheet name="SS_Analysis" sheetId="1" r:id="rId1"/>
     <sheet name="Inductor_Design" sheetId="2" r:id="rId2"/>
+    <sheet name="Testing_Openloop" sheetId="4" r:id="rId3"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -30,15 +31,12 @@
         <xcalcf:feature name="microsoft.com:LET_WF"/>
       </xcalcf:calcFeatures>
     </ext>
-    <ext xmlns:xlwcv="http://schemas.microsoft.com/office/spreadsheetml/2024/workbookCompatibilityVersion" uri="{D14903EA-33C4-47F7-8F05-3474C54BE107}">
-      <xlwcv:version setVersion="1"/>
-    </ext>
   </extLst>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="459" uniqueCount="220">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="527" uniqueCount="260">
   <si>
     <t>Parameter</t>
   </si>
@@ -698,6 +696,126 @@
   </si>
   <si>
     <t>R7 = 180kOhms</t>
+  </si>
+  <si>
+    <t>Testing with breadboard: E12 values</t>
+  </si>
+  <si>
+    <t>Rl values</t>
+  </si>
+  <si>
+    <t>Rl_E12 values</t>
+  </si>
+  <si>
+    <t>Testing Items for each:</t>
+  </si>
+  <si>
+    <t>Order list: breadboard testing</t>
+  </si>
+  <si>
+    <t>*</t>
+  </si>
+  <si>
+    <t>Output V</t>
+  </si>
+  <si>
+    <t>Breadboard</t>
+  </si>
+  <si>
+    <t>Current through inductor</t>
+  </si>
+  <si>
+    <t>5.6, 10, 22, 33, 47 ohm resistors</t>
+  </si>
+  <si>
+    <t>Current through shunt branch</t>
+  </si>
+  <si>
+    <t>47uH inductor</t>
+  </si>
+  <si>
+    <t>Schotty diode</t>
+  </si>
+  <si>
+    <t>^Note: Others were not measured</t>
+  </si>
+  <si>
+    <t xml:space="preserve">due to time constraints, and lack of </t>
+  </si>
+  <si>
+    <t>&gt; Input V given by DC power supply</t>
+  </si>
+  <si>
+    <t>0.1ohm shunt resistors available.</t>
+  </si>
+  <si>
+    <t>&gt;Switch operated using oscilloscope</t>
+  </si>
+  <si>
+    <t>Rl = 5.6</t>
+  </si>
+  <si>
+    <t>Real R: 5.58</t>
+  </si>
+  <si>
+    <t>Rl = 10</t>
+  </si>
+  <si>
+    <t>Real R: 10.07</t>
+  </si>
+  <si>
+    <t>Rl = 22</t>
+  </si>
+  <si>
+    <t>Real R: 22.08</t>
+  </si>
+  <si>
+    <t>Rl = 33</t>
+  </si>
+  <si>
+    <t>Real R: 32.89</t>
+  </si>
+  <si>
+    <t>Rl = 47</t>
+  </si>
+  <si>
+    <t>Real R: 47.13</t>
+  </si>
+  <si>
+    <t>Input V</t>
+  </si>
+  <si>
+    <t>Duty Cycle</t>
+  </si>
+  <si>
+    <t>3V</t>
+  </si>
+  <si>
+    <t>3.5V</t>
+  </si>
+  <si>
+    <t>3.8V</t>
+  </si>
+  <si>
+    <t>3.9V</t>
+  </si>
+  <si>
+    <t>3.4V</t>
+  </si>
+  <si>
+    <t>4V</t>
+  </si>
+  <si>
+    <t>4.1V</t>
+  </si>
+  <si>
+    <t>4.2V</t>
+  </si>
+  <si>
+    <t>4.26V</t>
+  </si>
+  <si>
+    <t>4.3V</t>
   </si>
 </sst>
 </file>
@@ -712,7 +830,7 @@
     <numFmt numFmtId="168" formatCode="0.0000000"/>
     <numFmt numFmtId="169" formatCode="0.0000"/>
   </numFmts>
-  <fonts count="10">
+  <fonts count="10" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -785,10 +903,11 @@
       <sz val="11"/>
       <color theme="1"/>
       <name val="Aptos Narrow"/>
+      <family val="2"/>
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="7">
+  <fills count="9">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -824,6 +943,18 @@
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="4" tint="0.59999389629810485"/>
+        <bgColor indexed="65"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="9" tint="0.79998168889431442"/>
+        <bgColor indexed="65"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="65">
     <border>
@@ -1730,13 +1861,15 @@
       <diagonal/>
     </border>
   </borders>
-  <cellStyleXfs count="4">
+  <cellStyleXfs count="6">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="1" applyNumberFormat="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="1" fillId="3" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="1" fillId="7" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="1" fillId="8" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="134">
+  <cellXfs count="136">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
@@ -1874,7 +2007,7 @@
     <xf numFmtId="49" fontId="8" fillId="0" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
     <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="169" fontId="0" fillId="0" borderId="49" xfId="0" applyNumberFormat="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="44" xfId="0" applyNumberFormat="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="44" xfId="0" applyBorder="1"/>
     <xf numFmtId="2" fontId="0" fillId="0" borderId="49" xfId="0" applyNumberFormat="1" applyBorder="1"/>
     <xf numFmtId="1" fontId="0" fillId="0" borderId="49" xfId="0" applyNumberFormat="1" applyBorder="1"/>
     <xf numFmtId="169" fontId="0" fillId="0" borderId="53" xfId="0" applyNumberFormat="1" applyBorder="1"/>
@@ -1882,17 +2015,21 @@
     <xf numFmtId="169" fontId="0" fillId="0" borderId="63" xfId="0" applyNumberFormat="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="64" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="1" fillId="3" borderId="0" xfId="2" applyBorder="1"/>
-    <xf numFmtId="166" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="64" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="2" applyFont="1" applyBorder="1"/>
     <xf numFmtId="167" fontId="0" fillId="0" borderId="34" xfId="0" applyNumberFormat="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="7" borderId="0" xfId="4"/>
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="0" xfId="2"/>
+    <xf numFmtId="0" fontId="1" fillId="8" borderId="0" xfId="5"/>
+    <xf numFmtId="9" fontId="1" fillId="8" borderId="0" xfId="5" applyNumberFormat="1"/>
   </cellXfs>
-  <cellStyles count="4">
+  <cellStyles count="6">
     <cellStyle name="20% - Accent1" xfId="2" builtinId="30"/>
+    <cellStyle name="20% - Accent6" xfId="5" builtinId="50"/>
+    <cellStyle name="40% - Accent1" xfId="4" builtinId="31"/>
     <cellStyle name="Check Cell" xfId="1" builtinId="23"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
-    <cellStyle name="Per cent" xfId="3" builtinId="5"/>
+    <cellStyle name="Percent" xfId="3" builtinId="5"/>
   </cellStyles>
   <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
@@ -2274,30 +2411,30 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E4C28CAE-7D6E-414C-9BF7-B54583CFEE9E}">
   <dimension ref="A1:N129"/>
-  <sheetFormatPr defaultColWidth="12" defaultRowHeight="13.5"/>
+  <sheetFormatPr defaultColWidth="12" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="20.4375" customWidth="1"/>
-    <col min="2" max="2" width="13.5625" customWidth="1"/>
-    <col min="3" max="3" width="13.3125" customWidth="1"/>
-    <col min="4" max="7" width="12.875" customWidth="1"/>
+    <col min="1" max="1" width="20.44140625" customWidth="1"/>
+    <col min="2" max="2" width="13.5546875" customWidth="1"/>
+    <col min="3" max="3" width="13.33203125" customWidth="1"/>
+    <col min="4" max="7" width="12.88671875" customWidth="1"/>
     <col min="8" max="8" width="22" customWidth="1"/>
-    <col min="9" max="11" width="12.875" customWidth="1"/>
-    <col min="12" max="12" width="17.4375" customWidth="1"/>
-    <col min="13" max="13" width="18.875" customWidth="1"/>
+    <col min="9" max="11" width="12.88671875" customWidth="1"/>
+    <col min="12" max="12" width="17.44140625" customWidth="1"/>
+    <col min="13" max="13" width="18.88671875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" ht="20.65">
+    <row r="1" spans="1:3" ht="21" x14ac:dyDescent="0.4">
       <c r="A1" s="1" t="s">
         <v>58</v>
       </c>
     </row>
-    <row r="3" spans="1:3" ht="17.649999999999999">
+    <row r="3" spans="1:3" ht="18" x14ac:dyDescent="0.35">
       <c r="A3" s="2" t="s">
         <v>137</v>
       </c>
     </row>
-    <row r="4" spans="1:3" ht="13.9" thickBot="1"/>
-    <row r="5" spans="1:3" ht="14.65" thickTop="1" thickBot="1">
+    <row r="4" spans="1:3" ht="15" thickBot="1" x14ac:dyDescent="0.35"/>
+    <row r="5" spans="1:3" ht="15.6" thickTop="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A5" s="3" t="s">
         <v>0</v>
       </c>
@@ -2308,7 +2445,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="6" spans="1:3" ht="13.9" thickTop="1">
+    <row r="6" spans="1:3" ht="15" thickTop="1" x14ac:dyDescent="0.3">
       <c r="A6" s="37" t="s">
         <v>36</v>
       </c>
@@ -2319,7 +2456,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="7" spans="1:3">
+    <row r="7" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A7" s="38" t="s">
         <v>37</v>
       </c>
@@ -2330,7 +2467,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="8" spans="1:3">
+    <row r="8" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A8" s="38" t="s">
         <v>38</v>
       </c>
@@ -2341,7 +2478,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="9" spans="1:3">
+    <row r="9" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A9" s="38" t="s">
         <v>56</v>
       </c>
@@ -2352,7 +2489,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="10" spans="1:3">
+    <row r="10" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A10" s="38" t="s">
         <v>57</v>
       </c>
@@ -2363,7 +2500,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="11" spans="1:3" ht="13.9" thickBot="1">
+    <row r="11" spans="1:3" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A11" s="10" t="s">
         <v>5</v>
       </c>
@@ -2374,16 +2511,16 @@
         <v>6</v>
       </c>
     </row>
-    <row r="12" spans="1:3" ht="15.4" thickTop="1">
+    <row r="12" spans="1:3" ht="16.2" thickTop="1" x14ac:dyDescent="0.3">
       <c r="A12" s="13"/>
     </row>
-    <row r="14" spans="1:3" ht="17.649999999999999">
+    <row r="14" spans="1:3" ht="18" x14ac:dyDescent="0.35">
       <c r="A14" s="2" t="s">
         <v>55</v>
       </c>
     </row>
-    <row r="15" spans="1:3" ht="13.9" thickBot="1"/>
-    <row r="16" spans="1:3" ht="14.65" thickTop="1" thickBot="1">
+    <row r="15" spans="1:3" ht="15" thickBot="1" x14ac:dyDescent="0.35"/>
+    <row r="16" spans="1:3" ht="15.6" thickTop="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A16" s="3" t="s">
         <v>0</v>
       </c>
@@ -2394,7 +2531,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="17" spans="1:3" ht="13.9" thickTop="1">
+    <row r="17" spans="1:3" ht="15" thickTop="1" x14ac:dyDescent="0.3">
       <c r="A17" s="45" t="s">
         <v>41</v>
       </c>
@@ -2406,7 +2543,7 @@
         <v>102</v>
       </c>
     </row>
-    <row r="18" spans="1:3">
+    <row r="18" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A18" s="47" t="s">
         <v>40</v>
       </c>
@@ -2418,7 +2555,7 @@
         <v>103</v>
       </c>
     </row>
-    <row r="19" spans="1:3">
+    <row r="19" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A19" s="56" t="s">
         <v>59</v>
       </c>
@@ -2430,7 +2567,7 @@
         <v>104</v>
       </c>
     </row>
-    <row r="20" spans="1:3">
+    <row r="20" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A20" s="49" t="s">
         <v>60</v>
       </c>
@@ -2442,7 +2579,7 @@
         <v>105</v>
       </c>
     </row>
-    <row r="21" spans="1:3">
+    <row r="21" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A21" s="52" t="s">
         <v>43</v>
       </c>
@@ -2454,7 +2591,7 @@
         <v>106</v>
       </c>
     </row>
-    <row r="22" spans="1:3">
+    <row r="22" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A22" s="52" t="s">
         <v>146</v>
       </c>
@@ -2466,7 +2603,7 @@
         <v>151</v>
       </c>
     </row>
-    <row r="23" spans="1:3">
+    <row r="23" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A23" s="52" t="s">
         <v>44</v>
       </c>
@@ -2478,7 +2615,7 @@
         <v>152</v>
       </c>
     </row>
-    <row r="24" spans="1:3">
+    <row r="24" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A24" s="93" t="s">
         <v>147</v>
       </c>
@@ -2490,7 +2627,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="25" spans="1:3" ht="13.9" thickBot="1">
+    <row r="25" spans="1:3" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A25" s="85" t="s">
         <v>101</v>
       </c>
@@ -2501,14 +2638,14 @@
         <v>8</v>
       </c>
     </row>
-    <row r="26" spans="1:3" ht="13.9" thickTop="1"/>
-    <row r="28" spans="1:3" ht="17.649999999999999">
+    <row r="26" spans="1:3" ht="15" thickTop="1" x14ac:dyDescent="0.3"/>
+    <row r="28" spans="1:3" ht="18" x14ac:dyDescent="0.35">
       <c r="A28" s="2" t="s">
         <v>9</v>
       </c>
     </row>
-    <row r="29" spans="1:3" ht="13.9" thickBot="1"/>
-    <row r="30" spans="1:3" ht="14.65" thickTop="1" thickBot="1">
+    <row r="29" spans="1:3" ht="15" thickBot="1" x14ac:dyDescent="0.35"/>
+    <row r="30" spans="1:3" ht="15.6" thickTop="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A30" s="3" t="s">
         <v>0</v>
       </c>
@@ -2519,7 +2656,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="31" spans="1:3" ht="13.9" thickTop="1">
+    <row r="31" spans="1:3" ht="15" thickTop="1" x14ac:dyDescent="0.3">
       <c r="A31" s="4" t="s">
         <v>10</v>
       </c>
@@ -2530,7 +2667,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="32" spans="1:3">
+    <row r="32" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A32" s="95" t="s">
         <v>148</v>
       </c>
@@ -2542,7 +2679,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="33" spans="1:11">
+    <row r="33" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A33" s="15" t="s">
         <v>11</v>
       </c>
@@ -2554,7 +2691,7 @@
         <v>150</v>
       </c>
     </row>
-    <row r="34" spans="1:11">
+    <row r="34" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A34" s="27" t="s">
         <v>149</v>
       </c>
@@ -2566,7 +2703,7 @@
         <v>107</v>
       </c>
     </row>
-    <row r="35" spans="1:11" ht="13.9" thickBot="1">
+    <row r="35" spans="1:11" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A35" s="10" t="s">
         <v>12</v>
       </c>
@@ -2577,14 +2714,14 @@
         <v>107</v>
       </c>
     </row>
-    <row r="36" spans="1:11" ht="13.9" thickTop="1"/>
-    <row r="38" spans="1:11" ht="17.649999999999999">
+    <row r="36" spans="1:11" ht="15" thickTop="1" x14ac:dyDescent="0.3"/>
+    <row r="38" spans="1:11" ht="18" x14ac:dyDescent="0.35">
       <c r="A38" s="2" t="s">
         <v>13</v>
       </c>
     </row>
-    <row r="39" spans="1:11" ht="13.9" thickBot="1"/>
-    <row r="40" spans="1:11" ht="14.65" thickTop="1" thickBot="1">
+    <row r="39" spans="1:11" ht="15" thickBot="1" x14ac:dyDescent="0.35"/>
+    <row r="40" spans="1:11" ht="15.6" thickTop="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A40" s="3" t="s">
         <v>0</v>
       </c>
@@ -2619,7 +2756,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="41" spans="1:11" ht="13.9" thickTop="1">
+    <row r="41" spans="1:11" ht="15" thickTop="1" x14ac:dyDescent="0.3">
       <c r="A41" s="4" t="s">
         <v>14</v>
       </c>
@@ -2654,7 +2791,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="42" spans="1:11">
+    <row r="42" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A42" s="44" t="s">
         <v>39</v>
       </c>
@@ -2689,7 +2826,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="43" spans="1:11">
+    <row r="43" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A43" s="7" t="s">
         <v>15</v>
       </c>
@@ -2725,7 +2862,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="44" spans="1:11">
+    <row r="44" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A44" s="7" t="s">
         <v>16</v>
       </c>
@@ -2765,7 +2902,7 @@
         <v>108</v>
       </c>
     </row>
-    <row r="45" spans="1:11">
+    <row r="45" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A45" s="7" t="s">
         <v>17</v>
       </c>
@@ -2805,7 +2942,7 @@
         <v>109</v>
       </c>
     </row>
-    <row r="46" spans="1:11">
+    <row r="46" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A46" s="38" t="s">
         <v>46</v>
       </c>
@@ -2845,7 +2982,7 @@
         <v>110</v>
       </c>
     </row>
-    <row r="47" spans="1:11">
+    <row r="47" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A47" s="38" t="s">
         <v>45</v>
       </c>
@@ -2885,7 +3022,7 @@
         <v>111</v>
       </c>
     </row>
-    <row r="48" spans="1:11">
+    <row r="48" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A48" s="7" t="s">
         <v>18</v>
       </c>
@@ -2915,7 +3052,7 @@
       </c>
       <c r="K48" s="23"/>
     </row>
-    <row r="49" spans="1:14">
+    <row r="49" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A49" s="7" t="s">
         <v>48</v>
       </c>
@@ -2955,7 +3092,7 @@
         <v>112</v>
       </c>
     </row>
-    <row r="50" spans="1:14">
+    <row r="50" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A50" s="7" t="s">
         <v>153</v>
       </c>
@@ -2995,7 +3132,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="51" spans="1:14">
+    <row r="51" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A51" s="7" t="s">
         <v>47</v>
       </c>
@@ -3035,7 +3172,7 @@
         <v>113</v>
       </c>
     </row>
-    <row r="52" spans="1:14">
+    <row r="52" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A52" s="27" t="s">
         <v>49</v>
       </c>
@@ -3075,7 +3212,7 @@
         <v>114</v>
       </c>
     </row>
-    <row r="53" spans="1:14">
+    <row r="53" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A53" s="27" t="s">
         <v>51</v>
       </c>
@@ -3115,7 +3252,7 @@
         <v>115</v>
       </c>
     </row>
-    <row r="54" spans="1:14">
+    <row r="54" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A54" s="27" t="s">
         <v>50</v>
       </c>
@@ -3155,7 +3292,7 @@
         <v>116</v>
       </c>
     </row>
-    <row r="55" spans="1:14">
+    <row r="55" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A55" s="7" t="s">
         <v>52</v>
       </c>
@@ -3190,7 +3327,7 @@
         <v>117</v>
       </c>
     </row>
-    <row r="56" spans="1:14">
+    <row r="56" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A56" s="27" t="s">
         <v>53</v>
       </c>
@@ -3234,7 +3371,7 @@
         <v>156</v>
       </c>
     </row>
-    <row r="57" spans="1:14" ht="13.9" thickBot="1">
+    <row r="57" spans="1:14" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A57" s="10" t="s">
         <v>54</v>
       </c>
@@ -3274,20 +3411,20 @@
         <v>119</v>
       </c>
     </row>
-    <row r="58" spans="1:14" ht="13.9" thickTop="1">
+    <row r="58" spans="1:14" ht="15" thickTop="1" x14ac:dyDescent="0.3">
       <c r="B58" s="32"/>
       <c r="C58" s="33"/>
     </row>
-    <row r="59" spans="1:14">
+    <row r="59" spans="1:14" x14ac:dyDescent="0.3">
       <c r="B59" s="32"/>
       <c r="C59" s="33"/>
     </row>
-    <row r="60" spans="1:14" ht="17.649999999999999">
+    <row r="60" spans="1:14" ht="18" x14ac:dyDescent="0.35">
       <c r="A60" s="2" t="s">
         <v>19</v>
       </c>
     </row>
-    <row r="62" spans="1:14" ht="14.25" thickBot="1">
+    <row r="62" spans="1:14" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A62" s="113" t="s">
         <v>0</v>
       </c>
@@ -3320,7 +3457,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="63" spans="1:14" ht="13.9" thickTop="1">
+    <row r="63" spans="1:14" ht="15" thickTop="1" x14ac:dyDescent="0.3">
       <c r="A63" s="7" t="s">
         <v>16</v>
       </c>
@@ -3360,7 +3497,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="64" spans="1:14">
+    <row r="64" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A64" s="7" t="s">
         <v>17</v>
       </c>
@@ -3390,7 +3527,7 @@
       </c>
       <c r="K64" s="23"/>
     </row>
-    <row r="65" spans="1:12">
+    <row r="65" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A65" s="38" t="s">
         <v>158</v>
       </c>
@@ -3425,7 +3562,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="66" spans="1:12">
+    <row r="66" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A66" s="38" t="s">
         <v>159</v>
       </c>
@@ -3460,7 +3597,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="67" spans="1:12">
+    <row r="67" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A67" s="7" t="s">
         <v>18</v>
       </c>
@@ -3485,7 +3622,7 @@
       </c>
       <c r="K67" s="23"/>
     </row>
-    <row r="68" spans="1:12">
+    <row r="68" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A68" s="38" t="s">
         <v>45</v>
       </c>
@@ -3525,7 +3662,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="69" spans="1:12">
+    <row r="69" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A69" s="7" t="s">
         <v>48</v>
       </c>
@@ -3560,7 +3697,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="70" spans="1:12">
+    <row r="70" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A70" s="7" t="s">
         <v>47</v>
       </c>
@@ -3596,7 +3733,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="71" spans="1:12">
+    <row r="71" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A71" s="27" t="s">
         <v>49</v>
       </c>
@@ -3631,7 +3768,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="72" spans="1:12">
+    <row r="72" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A72" s="27" t="s">
         <v>51</v>
       </c>
@@ -3666,7 +3803,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="73" spans="1:12">
+    <row r="73" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A73" s="27" t="s">
         <v>50</v>
       </c>
@@ -3702,7 +3839,7 @@
       </c>
       <c r="L73" s="106"/>
     </row>
-    <row r="74" spans="1:12">
+    <row r="74" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A74" s="7" t="s">
         <v>52</v>
       </c>
@@ -3737,7 +3874,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="75" spans="1:12">
+    <row r="75" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A75" s="27" t="s">
         <v>53</v>
       </c>
@@ -3772,7 +3909,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="76" spans="1:12" ht="13.9" thickBot="1">
+    <row r="76" spans="1:12" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A76" s="115" t="s">
         <v>54</v>
       </c>
@@ -3808,14 +3945,14 @@
         <v>160</v>
       </c>
     </row>
-    <row r="77" spans="1:12" ht="13.9" thickTop="1"/>
-    <row r="79" spans="1:12" ht="17.649999999999999">
+    <row r="77" spans="1:12" ht="15" thickTop="1" x14ac:dyDescent="0.3"/>
+    <row r="79" spans="1:12" ht="18" x14ac:dyDescent="0.35">
       <c r="A79" s="2" t="s">
         <v>22</v>
       </c>
     </row>
-    <row r="80" spans="1:12" ht="13.9" thickBot="1"/>
-    <row r="81" spans="1:3" ht="14.65" thickTop="1" thickBot="1">
+    <row r="80" spans="1:12" ht="15" thickBot="1" x14ac:dyDescent="0.35"/>
+    <row r="81" spans="1:3" ht="15.6" thickTop="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A81" s="3" t="s">
         <v>0</v>
       </c>
@@ -3826,7 +3963,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="82" spans="1:3" ht="13.9" thickTop="1">
+    <row r="82" spans="1:3" ht="15" thickTop="1" x14ac:dyDescent="0.3">
       <c r="A82" s="4" t="s">
         <v>122</v>
       </c>
@@ -3837,7 +3974,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="83" spans="1:3">
+    <row r="83" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A83" s="15" t="s">
         <v>123</v>
       </c>
@@ -3848,7 +3985,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="84" spans="1:3">
+    <row r="84" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A84" s="15" t="s">
         <v>23</v>
       </c>
@@ -3859,7 +3996,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="85" spans="1:3" ht="15">
+    <row r="85" spans="1:3" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A85" s="52" t="s">
         <v>128</v>
       </c>
@@ -3870,7 +4007,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="86" spans="1:3">
+    <row r="86" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A86" s="52" t="s">
         <v>127</v>
       </c>
@@ -3881,7 +4018,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="87" spans="1:3">
+    <row r="87" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A87" s="52" t="s">
         <v>126</v>
       </c>
@@ -3892,7 +4029,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="88" spans="1:3">
+    <row r="88" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A88" s="52" t="s">
         <v>125</v>
       </c>
@@ -3903,7 +4040,7 @@
         <v>132</v>
       </c>
     </row>
-    <row r="89" spans="1:3">
+    <row r="89" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A89" s="52" t="s">
         <v>129</v>
       </c>
@@ -3914,7 +4051,7 @@
         <v>190</v>
       </c>
     </row>
-    <row r="90" spans="1:3">
+    <row r="90" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A90" s="52" t="s">
         <v>130</v>
       </c>
@@ -3925,7 +4062,7 @@
         <v>191</v>
       </c>
     </row>
-    <row r="91" spans="1:3">
+    <row r="91" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A91" s="52" t="s">
         <v>131</v>
       </c>
@@ -3936,7 +4073,7 @@
         <v>133</v>
       </c>
     </row>
-    <row r="92" spans="1:3">
+    <row r="92" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A92" s="52" t="s">
         <v>27</v>
       </c>
@@ -3947,7 +4084,7 @@
         <v>134</v>
       </c>
     </row>
-    <row r="93" spans="1:3">
+    <row r="93" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A93" s="52" t="s">
         <v>28</v>
       </c>
@@ -3958,7 +4095,7 @@
         <v>135</v>
       </c>
     </row>
-    <row r="94" spans="1:3">
+    <row r="94" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A94" s="52" t="s">
         <v>124</v>
       </c>
@@ -3969,7 +4106,7 @@
         <v>136</v>
       </c>
     </row>
-    <row r="95" spans="1:3">
+    <row r="95" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A95" s="15" t="s">
         <v>120</v>
       </c>
@@ -3980,7 +4117,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="96" spans="1:3">
+    <row r="96" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A96" s="15" t="s">
         <v>121</v>
       </c>
@@ -3991,7 +4128,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="97" spans="1:11">
+    <row r="97" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A97" s="52" t="s">
         <v>163</v>
       </c>
@@ -4002,7 +4139,7 @@
         <v>162</v>
       </c>
     </row>
-    <row r="98" spans="1:11">
+    <row r="98" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A98" s="15" t="s">
         <v>30</v>
       </c>
@@ -4011,7 +4148,7 @@
       </c>
       <c r="C98" s="18"/>
     </row>
-    <row r="99" spans="1:11" ht="13.9" thickBot="1">
+    <row r="99" spans="1:11" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A99" s="10" t="s">
         <v>31</v>
       </c>
@@ -4020,14 +4157,14 @@
       </c>
       <c r="C99" s="19"/>
     </row>
-    <row r="100" spans="1:11" ht="13.9" thickTop="1"/>
-    <row r="102" spans="1:11" ht="17.649999999999999">
+    <row r="100" spans="1:11" ht="15" thickTop="1" x14ac:dyDescent="0.3"/>
+    <row r="102" spans="1:11" ht="18" x14ac:dyDescent="0.35">
       <c r="A102" s="2" t="s">
         <v>32</v>
       </c>
     </row>
-    <row r="103" spans="1:11" ht="13.9" thickBot="1"/>
-    <row r="104" spans="1:11" ht="14.65" thickTop="1" thickBot="1">
+    <row r="103" spans="1:11" ht="15" thickBot="1" x14ac:dyDescent="0.35"/>
+    <row r="104" spans="1:11" ht="15.6" thickTop="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A104" s="3" t="s">
         <v>0</v>
       </c>
@@ -4058,7 +4195,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="105" spans="1:11" ht="13.9" thickTop="1">
+    <row r="105" spans="1:11" ht="15" thickTop="1" x14ac:dyDescent="0.3">
       <c r="A105" s="7" t="s">
         <v>16</v>
       </c>
@@ -4097,7 +4234,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="106" spans="1:11">
+    <row r="106" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A106" s="7" t="s">
         <v>33</v>
       </c>
@@ -4132,7 +4269,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="107" spans="1:11">
+    <row r="107" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A107" s="38" t="s">
         <v>161</v>
       </c>
@@ -4167,7 +4304,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="108" spans="1:11" ht="13.9" thickBot="1">
+    <row r="108" spans="1:11" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A108" s="10" t="s">
         <v>34</v>
       </c>
@@ -4202,14 +4339,14 @@
         <v>35</v>
       </c>
     </row>
-    <row r="109" spans="1:11" ht="13.9" thickTop="1"/>
-    <row r="111" spans="1:11" ht="17.649999999999999">
+    <row r="109" spans="1:11" ht="15" thickTop="1" x14ac:dyDescent="0.3"/>
+    <row r="111" spans="1:11" ht="18" x14ac:dyDescent="0.35">
       <c r="A111" s="2" t="s">
         <v>164</v>
       </c>
     </row>
-    <row r="112" spans="1:11" ht="13.9" thickBot="1"/>
-    <row r="113" spans="1:8" ht="14.65" thickTop="1" thickBot="1">
+    <row r="112" spans="1:11" ht="15" thickBot="1" x14ac:dyDescent="0.35"/>
+    <row r="113" spans="1:8" ht="15.6" thickTop="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A113" s="3" t="s">
         <v>0</v>
       </c>
@@ -4229,7 +4366,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="114" spans="1:8" ht="13.9" thickTop="1">
+    <row r="114" spans="1:8" ht="15" thickTop="1" x14ac:dyDescent="0.3">
       <c r="A114" s="38" t="s">
         <v>165</v>
       </c>
@@ -4249,7 +4386,7 @@
         <v>184</v>
       </c>
     </row>
-    <row r="115" spans="1:8">
+    <row r="115" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A115" s="38" t="s">
         <v>172</v>
       </c>
@@ -4269,7 +4406,7 @@
         <v>184</v>
       </c>
     </row>
-    <row r="116" spans="1:8">
+    <row r="116" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A116" s="38" t="s">
         <v>178</v>
       </c>
@@ -4289,7 +4426,7 @@
         <v>183</v>
       </c>
     </row>
-    <row r="117" spans="1:8" ht="13.9" thickBot="1">
+    <row r="117" spans="1:8" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A117" s="85" t="s">
         <v>170</v>
       </c>
@@ -4309,7 +4446,7 @@
         <v>177</v>
       </c>
     </row>
-    <row r="118" spans="1:8" ht="14.25" thickTop="1" thickBot="1">
+    <row r="118" spans="1:8" ht="15.6" thickTop="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A118" s="85" t="s">
         <v>185</v>
       </c>
@@ -4329,69 +4466,69 @@
         <v>188</v>
       </c>
     </row>
-    <row r="119" spans="1:8" ht="13.9" thickTop="1"/>
-    <row r="120" spans="1:8" ht="13.9">
-      <c r="A120" s="131" t="s">
+    <row r="119" spans="1:8" ht="15" thickTop="1" x14ac:dyDescent="0.3"/>
+    <row r="120" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A120" s="129" t="s">
         <v>212</v>
       </c>
     </row>
-    <row r="121" spans="1:8">
-      <c r="A121" s="132" t="s">
+    <row r="121" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A121" s="130" t="s">
         <v>206</v>
       </c>
       <c r="B121" t="s">
         <v>203</v>
       </c>
     </row>
-    <row r="122" spans="1:8">
-      <c r="A122" s="132" t="s">
+    <row r="122" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A122" s="130" t="s">
         <v>205</v>
       </c>
     </row>
-    <row r="123" spans="1:8">
-      <c r="A123" s="132" t="s">
+    <row r="123" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A123" s="130" t="s">
         <v>207</v>
       </c>
       <c r="B123" t="s">
         <v>204</v>
       </c>
     </row>
-    <row r="124" spans="1:8">
-      <c r="A124" s="132" t="s">
+    <row r="124" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A124" s="130" t="s">
         <v>219</v>
       </c>
       <c r="B124" t="s">
         <v>208</v>
       </c>
     </row>
-    <row r="125" spans="1:8" ht="13.9">
-      <c r="A125" s="131" t="s">
+    <row r="125" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A125" s="129" t="s">
         <v>213</v>
       </c>
     </row>
-    <row r="126" spans="1:8">
-      <c r="A126" s="132" t="s">
+    <row r="126" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A126" s="130" t="s">
         <v>209</v>
       </c>
       <c r="B126" t="s">
         <v>211</v>
       </c>
     </row>
-    <row r="127" spans="1:8">
-      <c r="A127" s="132" t="s">
+    <row r="127" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A127" s="130" t="s">
         <v>210</v>
       </c>
     </row>
-    <row r="128" spans="1:8">
-      <c r="A128" s="132" t="s">
+    <row r="128" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A128" s="130" t="s">
         <v>214</v>
       </c>
       <c r="B128" t="s">
         <v>215</v>
       </c>
     </row>
-    <row r="129" spans="1:2">
-      <c r="A129" s="132" t="s">
+    <row r="129" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A129" s="130" t="s">
         <v>216</v>
       </c>
       <c r="B129" t="s">
@@ -4409,24 +4546,24 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{3F74A05D-7210-44AC-859D-2846F0884F7B}">
   <dimension ref="A1:G56"/>
-  <sheetFormatPr defaultColWidth="12" defaultRowHeight="13.5"/>
+  <sheetFormatPr defaultColWidth="12" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="24.4375" customWidth="1"/>
-    <col min="2" max="9" width="12.875" customWidth="1"/>
+    <col min="1" max="1" width="24.44140625" customWidth="1"/>
+    <col min="2" max="9" width="12.88671875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5" ht="20.65">
+    <row r="1" spans="1:5" ht="21" x14ac:dyDescent="0.4">
       <c r="A1" s="1" t="s">
         <v>90</v>
       </c>
     </row>
-    <row r="3" spans="1:5" ht="17.649999999999999">
+    <row r="3" spans="1:5" ht="18" x14ac:dyDescent="0.35">
       <c r="A3" s="2" t="s">
         <v>61</v>
       </c>
     </row>
-    <row r="4" spans="1:5" ht="13.9" thickBot="1"/>
-    <row r="5" spans="1:5" ht="14.65" thickTop="1" thickBot="1">
+    <row r="4" spans="1:5" ht="15" thickBot="1" x14ac:dyDescent="0.35"/>
+    <row r="5" spans="1:5" ht="15.6" thickTop="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A5" s="3" t="s">
         <v>0</v>
       </c>
@@ -4438,7 +4575,7 @@
       </c>
       <c r="E5" s="73"/>
     </row>
-    <row r="6" spans="1:5" ht="13.9" thickTop="1">
+    <row r="6" spans="1:5" ht="15" thickTop="1" x14ac:dyDescent="0.3">
       <c r="A6" s="37" t="s">
         <v>101</v>
       </c>
@@ -4450,7 +4587,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="7" spans="1:5">
+    <row r="7" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A7" s="38" t="s">
         <v>92</v>
       </c>
@@ -4462,7 +4599,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="8" spans="1:5">
+    <row r="8" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A8" s="38" t="s">
         <v>93</v>
       </c>
@@ -4474,7 +4611,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="9" spans="1:5">
+    <row r="9" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A9" s="38" t="s">
         <v>91</v>
       </c>
@@ -4486,7 +4623,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="10" spans="1:5">
+    <row r="10" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A10" s="7" t="s">
         <v>62</v>
       </c>
@@ -4497,7 +4634,7 @@
         <v>63</v>
       </c>
     </row>
-    <row r="11" spans="1:5" ht="13.9" thickBot="1">
+    <row r="11" spans="1:5" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A11" s="10" t="s">
         <v>5</v>
       </c>
@@ -4509,18 +4646,18 @@
         <v>6</v>
       </c>
     </row>
-    <row r="12" spans="1:5" ht="15.4" thickTop="1">
+    <row r="12" spans="1:5" ht="16.2" thickTop="1" x14ac:dyDescent="0.3">
       <c r="A12" s="13"/>
     </row>
-    <row r="14" spans="1:5" ht="17.649999999999999">
+    <row r="14" spans="1:5" ht="18" x14ac:dyDescent="0.35">
       <c r="A14" s="2" t="s">
         <v>64</v>
       </c>
     </row>
-    <row r="15" spans="1:5" ht="18" thickBot="1">
+    <row r="15" spans="1:5" ht="18.600000000000001" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A15" s="2"/>
     </row>
-    <row r="16" spans="1:5" ht="14.65" thickTop="1" thickBot="1">
+    <row r="16" spans="1:5" ht="15.6" thickTop="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A16" s="3" t="s">
         <v>0</v>
       </c>
@@ -4531,7 +4668,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="17" spans="1:3" ht="13.9" thickTop="1">
+    <row r="17" spans="1:3" ht="15" thickTop="1" x14ac:dyDescent="0.3">
       <c r="A17" s="59" t="s">
         <v>65</v>
       </c>
@@ -4540,7 +4677,7 @@
       </c>
       <c r="C17" s="61"/>
     </row>
-    <row r="18" spans="1:3">
+    <row r="18" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A18" s="62" t="s">
         <v>67</v>
       </c>
@@ -4549,7 +4686,7 @@
       </c>
       <c r="C18" s="64"/>
     </row>
-    <row r="19" spans="1:3">
+    <row r="19" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A19" s="62" t="s">
         <v>69</v>
       </c>
@@ -4560,7 +4697,7 @@
         <v>70</v>
       </c>
     </row>
-    <row r="20" spans="1:3">
+    <row r="20" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A20" s="62" t="s">
         <v>71</v>
       </c>
@@ -4571,7 +4708,7 @@
         <v>72</v>
       </c>
     </row>
-    <row r="21" spans="1:3">
+    <row r="21" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A21" s="62" t="s">
         <v>73</v>
       </c>
@@ -4582,7 +4719,7 @@
         <v>74</v>
       </c>
     </row>
-    <row r="22" spans="1:3">
+    <row r="22" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A22" s="62" t="s">
         <v>75</v>
       </c>
@@ -4593,7 +4730,7 @@
         <v>70</v>
       </c>
     </row>
-    <row r="23" spans="1:3">
+    <row r="23" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A23" s="62" t="s">
         <v>76</v>
       </c>
@@ -4604,7 +4741,7 @@
         <v>72</v>
       </c>
     </row>
-    <row r="24" spans="1:3">
+    <row r="24" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A24" s="62" t="s">
         <v>77</v>
       </c>
@@ -4616,7 +4753,7 @@
         <v>78</v>
       </c>
     </row>
-    <row r="25" spans="1:3">
+    <row r="25" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A25" s="62" t="s">
         <v>79</v>
       </c>
@@ -4628,7 +4765,7 @@
         <v>80</v>
       </c>
     </row>
-    <row r="26" spans="1:3">
+    <row r="26" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A26" s="67" t="s">
         <v>81</v>
       </c>
@@ -4636,7 +4773,7 @@
         <v>1510</v>
       </c>
     </row>
-    <row r="27" spans="1:3" ht="13.9" thickBot="1">
+    <row r="27" spans="1:3" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A27" s="68" t="s">
         <v>82</v>
       </c>
@@ -4645,14 +4782,14 @@
       </c>
       <c r="C27" s="70"/>
     </row>
-    <row r="28" spans="1:3" ht="13.9" thickTop="1"/>
-    <row r="30" spans="1:3" ht="17.649999999999999">
+    <row r="28" spans="1:3" ht="15" thickTop="1" x14ac:dyDescent="0.3"/>
+    <row r="30" spans="1:3" ht="18" x14ac:dyDescent="0.35">
       <c r="A30" s="2" t="s">
         <v>83</v>
       </c>
     </row>
-    <row r="31" spans="1:3" ht="13.9" thickBot="1"/>
-    <row r="32" spans="1:3" ht="14.65" thickTop="1" thickBot="1">
+    <row r="31" spans="1:3" ht="15" thickBot="1" x14ac:dyDescent="0.35"/>
+    <row r="32" spans="1:3" ht="15.6" thickTop="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A32" s="3" t="s">
         <v>0</v>
       </c>
@@ -4663,7 +4800,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="33" spans="1:7" ht="13.9" thickTop="1">
+    <row r="33" spans="1:7" ht="15" thickTop="1" x14ac:dyDescent="0.3">
       <c r="A33" s="59" t="s">
         <v>84</v>
       </c>
@@ -4675,7 +4812,7 @@
       </c>
       <c r="G33" s="73"/>
     </row>
-    <row r="34" spans="1:7">
+    <row r="34" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A34" s="74" t="s">
         <v>194</v>
       </c>
@@ -4688,7 +4825,7 @@
       </c>
       <c r="G34" s="73"/>
     </row>
-    <row r="35" spans="1:7">
+    <row r="35" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A35" s="74" t="s">
         <v>85</v>
       </c>
@@ -4702,7 +4839,7 @@
       <c r="F35" s="78"/>
       <c r="G35" s="73"/>
     </row>
-    <row r="36" spans="1:7" ht="15">
+    <row r="36" spans="1:7" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A36" s="74" t="s">
         <v>86</v>
       </c>
@@ -4715,7 +4852,7 @@
       <c r="F36" s="13"/>
       <c r="G36" s="13"/>
     </row>
-    <row r="37" spans="1:7">
+    <row r="37" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A37" s="74" t="s">
         <v>87</v>
       </c>
@@ -4727,7 +4864,7 @@
         <v>141</v>
       </c>
     </row>
-    <row r="38" spans="1:7">
+    <row r="38" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A38" s="81" t="s">
         <v>95</v>
       </c>
@@ -4738,7 +4875,7 @@
         <v>72</v>
       </c>
     </row>
-    <row r="39" spans="1:7">
+    <row r="39" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A39" s="81" t="s">
         <v>94</v>
       </c>
@@ -4750,7 +4887,7 @@
         <v>142</v>
       </c>
     </row>
-    <row r="40" spans="1:7">
+    <row r="40" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A40" s="81" t="s">
         <v>193</v>
       </c>
@@ -4759,7 +4896,7 @@
       </c>
       <c r="C40" s="76"/>
     </row>
-    <row r="41" spans="1:7">
+    <row r="41" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A41" s="81" t="s">
         <v>96</v>
       </c>
@@ -4771,7 +4908,7 @@
         <v>143</v>
       </c>
     </row>
-    <row r="42" spans="1:7" ht="13.9" thickBot="1">
+    <row r="42" spans="1:7" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A42" s="83" t="s">
         <v>88</v>
       </c>
@@ -4783,7 +4920,7 @@
         <v>144</v>
       </c>
     </row>
-    <row r="43" spans="1:7" ht="13.9" thickTop="1">
+    <row r="43" spans="1:7" ht="15" thickTop="1" x14ac:dyDescent="0.3">
       <c r="A43" s="125" t="s">
         <v>197</v>
       </c>
@@ -4795,7 +4932,7 @@
         <v>198</v>
       </c>
     </row>
-    <row r="44" spans="1:7">
+    <row r="44" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A44" s="125" t="s">
         <v>195</v>
       </c>
@@ -4807,7 +4944,7 @@
         <v>199</v>
       </c>
     </row>
-    <row r="45" spans="1:7">
+    <row r="45" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A45" s="125" t="s">
         <v>196</v>
       </c>
@@ -4819,7 +4956,7 @@
         <v>200</v>
       </c>
     </row>
-    <row r="46" spans="1:7">
+    <row r="46" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A46" s="74" t="s">
         <v>192</v>
       </c>
@@ -4831,25 +4968,25 @@
         <v>201</v>
       </c>
     </row>
-    <row r="47" spans="1:7">
+    <row r="47" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A47" s="128" t="s">
         <v>202</v>
       </c>
-      <c r="B47" s="129">
+      <c r="B47" s="114">
         <f>B34*B40*B39/B27</f>
         <v>24.166097335306102</v>
       </c>
-      <c r="C47" s="130" t="s">
+      <c r="C47" s="127" t="s">
         <v>70</v>
       </c>
     </row>
-    <row r="49" spans="1:3" ht="17.649999999999999">
+    <row r="49" spans="1:3" ht="18" x14ac:dyDescent="0.35">
       <c r="A49" s="2" t="s">
         <v>97</v>
       </c>
     </row>
-    <row r="50" spans="1:3" ht="13.9" thickBot="1"/>
-    <row r="51" spans="1:3" ht="14.65" thickTop="1" thickBot="1">
+    <row r="50" spans="1:3" ht="15" thickBot="1" x14ac:dyDescent="0.35"/>
+    <row r="51" spans="1:3" ht="15.6" thickTop="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A51" s="3" t="s">
         <v>0</v>
       </c>
@@ -4860,7 +4997,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="52" spans="1:3" ht="13.9" thickTop="1">
+    <row r="52" spans="1:3" ht="15" thickTop="1" x14ac:dyDescent="0.3">
       <c r="A52" s="81" t="s">
         <v>98</v>
       </c>
@@ -4871,11 +5008,11 @@
         <v>89</v>
       </c>
     </row>
-    <row r="53" spans="1:3">
+    <row r="53" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A53" s="74" t="s">
         <v>85</v>
       </c>
-      <c r="B53" s="133">
+      <c r="B53" s="131">
         <f>(B52*B8)/(B34*B19)</f>
         <v>0.20769450283115989</v>
       </c>
@@ -4883,7 +5020,7 @@
         <v>63</v>
       </c>
     </row>
-    <row r="54" spans="1:3">
+    <row r="54" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A54" s="81" t="s">
         <v>145</v>
       </c>
@@ -4894,7 +5031,7 @@
         <v>100</v>
       </c>
     </row>
-    <row r="55" spans="1:3" ht="13.9" thickBot="1">
+    <row r="55" spans="1:3" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A55" s="82" t="s">
         <v>99</v>
       </c>
@@ -4905,10 +5042,422 @@
         <v>100</v>
       </c>
     </row>
-    <row r="56" spans="1:3" ht="13.9" thickTop="1"/>
+    <row r="56" spans="1:3" ht="15" thickTop="1" x14ac:dyDescent="0.3"/>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{86BA37C4-8F32-417F-A8E4-D80C296F90D3}">
+  <dimension ref="B2:Y18"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetData>
+    <row r="2" spans="2:25" x14ac:dyDescent="0.3">
+      <c r="B2" s="129" t="s">
+        <v>220</v>
+      </c>
+    </row>
+    <row r="3" spans="2:25" x14ac:dyDescent="0.3">
+      <c r="B3" t="s">
+        <v>221</v>
+      </c>
+      <c r="D3" t="s">
+        <v>222</v>
+      </c>
+      <c r="G3" t="s">
+        <v>223</v>
+      </c>
+      <c r="K3" t="s">
+        <v>224</v>
+      </c>
+    </row>
+    <row r="4" spans="2:25" x14ac:dyDescent="0.3">
+      <c r="B4">
+        <v>5</v>
+      </c>
+      <c r="C4" t="s">
+        <v>225</v>
+      </c>
+      <c r="D4" s="129">
+        <v>5.6</v>
+      </c>
+      <c r="E4" t="s">
+        <v>225</v>
+      </c>
+      <c r="G4" s="129" t="s">
+        <v>226</v>
+      </c>
+      <c r="K4" t="s">
+        <v>227</v>
+      </c>
+    </row>
+    <row r="5" spans="2:25" x14ac:dyDescent="0.3">
+      <c r="B5">
+        <v>10</v>
+      </c>
+      <c r="C5" t="s">
+        <v>225</v>
+      </c>
+      <c r="D5" s="129">
+        <v>10</v>
+      </c>
+      <c r="E5" t="s">
+        <v>225</v>
+      </c>
+      <c r="G5" t="s">
+        <v>228</v>
+      </c>
+      <c r="K5" t="s">
+        <v>229</v>
+      </c>
+    </row>
+    <row r="6" spans="2:25" x14ac:dyDescent="0.3">
+      <c r="B6">
+        <v>15</v>
+      </c>
+      <c r="C6" t="s">
+        <v>225</v>
+      </c>
+      <c r="D6">
+        <v>15</v>
+      </c>
+      <c r="G6" t="s">
+        <v>230</v>
+      </c>
+      <c r="K6" t="s">
+        <v>231</v>
+      </c>
+    </row>
+    <row r="7" spans="2:25" x14ac:dyDescent="0.3">
+      <c r="B7">
+        <v>20</v>
+      </c>
+      <c r="D7" s="129">
+        <v>22</v>
+      </c>
+      <c r="E7" t="s">
+        <v>225</v>
+      </c>
+      <c r="K7" t="s">
+        <v>232</v>
+      </c>
+    </row>
+    <row r="8" spans="2:25" x14ac:dyDescent="0.3">
+      <c r="B8">
+        <v>25</v>
+      </c>
+      <c r="C8" t="s">
+        <v>225</v>
+      </c>
+      <c r="D8">
+        <v>27</v>
+      </c>
+      <c r="G8" t="s">
+        <v>233</v>
+      </c>
+    </row>
+    <row r="9" spans="2:25" x14ac:dyDescent="0.3">
+      <c r="B9">
+        <v>30</v>
+      </c>
+      <c r="C9" t="s">
+        <v>225</v>
+      </c>
+      <c r="D9">
+        <v>33</v>
+      </c>
+      <c r="G9" t="s">
+        <v>234</v>
+      </c>
+      <c r="K9" t="s">
+        <v>235</v>
+      </c>
+    </row>
+    <row r="10" spans="2:25" x14ac:dyDescent="0.3">
+      <c r="B10">
+        <v>35</v>
+      </c>
+      <c r="D10" s="129">
+        <v>33</v>
+      </c>
+      <c r="E10" t="s">
+        <v>225</v>
+      </c>
+      <c r="G10" t="s">
+        <v>236</v>
+      </c>
+      <c r="K10" t="s">
+        <v>237</v>
+      </c>
+    </row>
+    <row r="11" spans="2:25" x14ac:dyDescent="0.3">
+      <c r="B11">
+        <v>40</v>
+      </c>
+      <c r="C11" t="s">
+        <v>225</v>
+      </c>
+      <c r="D11">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="12" spans="2:25" x14ac:dyDescent="0.3">
+      <c r="B12">
+        <v>45</v>
+      </c>
+      <c r="C12" t="s">
+        <v>225</v>
+      </c>
+      <c r="D12">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="13" spans="2:25" x14ac:dyDescent="0.3">
+      <c r="B13">
+        <v>50</v>
+      </c>
+      <c r="C13" t="s">
+        <v>225</v>
+      </c>
+      <c r="D13" s="129">
+        <v>47</v>
+      </c>
+      <c r="E13" t="s">
+        <v>225</v>
+      </c>
+    </row>
+    <row r="15" spans="2:25" x14ac:dyDescent="0.3">
+      <c r="B15" s="132" t="s">
+        <v>238</v>
+      </c>
+      <c r="C15" s="132" t="s">
+        <v>239</v>
+      </c>
+      <c r="D15" s="132"/>
+      <c r="E15" s="132"/>
+      <c r="G15" s="132" t="s">
+        <v>240</v>
+      </c>
+      <c r="H15" s="132" t="s">
+        <v>241</v>
+      </c>
+      <c r="I15" s="132"/>
+      <c r="J15" s="132"/>
+      <c r="L15" s="132" t="s">
+        <v>242</v>
+      </c>
+      <c r="M15" s="132" t="s">
+        <v>243</v>
+      </c>
+      <c r="N15" s="132"/>
+      <c r="O15" s="132"/>
+      <c r="Q15" s="132" t="s">
+        <v>244</v>
+      </c>
+      <c r="R15" s="132" t="s">
+        <v>245</v>
+      </c>
+      <c r="S15" s="132"/>
+      <c r="T15" s="132"/>
+      <c r="V15" s="132" t="s">
+        <v>246</v>
+      </c>
+      <c r="W15" s="132" t="s">
+        <v>247</v>
+      </c>
+      <c r="X15" s="132"/>
+      <c r="Y15" s="132"/>
+    </row>
+    <row r="16" spans="2:25" x14ac:dyDescent="0.3">
+      <c r="B16" s="133" t="s">
+        <v>248</v>
+      </c>
+      <c r="C16" s="134">
+        <v>2.5</v>
+      </c>
+      <c r="D16" s="134">
+        <v>3</v>
+      </c>
+      <c r="E16" s="134">
+        <v>3.5</v>
+      </c>
+      <c r="G16" s="133" t="s">
+        <v>248</v>
+      </c>
+      <c r="H16" s="134">
+        <v>2.5</v>
+      </c>
+      <c r="I16" s="134">
+        <v>3</v>
+      </c>
+      <c r="J16" s="134">
+        <v>3.5</v>
+      </c>
+      <c r="L16" s="133" t="s">
+        <v>248</v>
+      </c>
+      <c r="M16" s="134">
+        <v>2.5</v>
+      </c>
+      <c r="N16" s="134">
+        <v>3</v>
+      </c>
+      <c r="O16" s="134">
+        <v>3.5</v>
+      </c>
+      <c r="Q16" s="133" t="s">
+        <v>248</v>
+      </c>
+      <c r="R16" s="134">
+        <v>2.5</v>
+      </c>
+      <c r="S16" s="134">
+        <v>3</v>
+      </c>
+      <c r="T16" s="134">
+        <v>3.5</v>
+      </c>
+      <c r="V16" s="133" t="s">
+        <v>248</v>
+      </c>
+      <c r="W16" s="134">
+        <v>2.5</v>
+      </c>
+      <c r="X16" s="134">
+        <v>3</v>
+      </c>
+      <c r="Y16" s="134">
+        <v>3.5</v>
+      </c>
+    </row>
+    <row r="17" spans="2:25" x14ac:dyDescent="0.3">
+      <c r="B17" s="133" t="s">
+        <v>249</v>
+      </c>
+      <c r="C17" s="135">
+        <v>0.5</v>
+      </c>
+      <c r="D17" s="135">
+        <v>0.4</v>
+      </c>
+      <c r="E17" s="135">
+        <v>0.3</v>
+      </c>
+      <c r="G17" s="133" t="s">
+        <v>249</v>
+      </c>
+      <c r="H17" s="135">
+        <v>0.5</v>
+      </c>
+      <c r="I17" s="135">
+        <v>0.4</v>
+      </c>
+      <c r="J17" s="135">
+        <v>0.3</v>
+      </c>
+      <c r="L17" s="133" t="s">
+        <v>249</v>
+      </c>
+      <c r="M17" s="135">
+        <v>0.5</v>
+      </c>
+      <c r="N17" s="135">
+        <v>0.4</v>
+      </c>
+      <c r="O17" s="135">
+        <v>0.3</v>
+      </c>
+      <c r="Q17" s="133" t="s">
+        <v>249</v>
+      </c>
+      <c r="R17" s="135">
+        <v>0.5</v>
+      </c>
+      <c r="S17" s="135">
+        <v>0.4</v>
+      </c>
+      <c r="T17" s="135">
+        <v>0.3</v>
+      </c>
+      <c r="V17" s="133" t="s">
+        <v>249</v>
+      </c>
+      <c r="W17" s="135">
+        <v>0.5</v>
+      </c>
+      <c r="X17" s="135">
+        <v>0.4</v>
+      </c>
+      <c r="Y17" s="135">
+        <v>0.3</v>
+      </c>
+    </row>
+    <row r="18" spans="2:25" x14ac:dyDescent="0.3">
+      <c r="B18" s="133" t="s">
+        <v>226</v>
+      </c>
+      <c r="C18" s="134" t="s">
+        <v>250</v>
+      </c>
+      <c r="D18" s="134">
+        <v>3.3</v>
+      </c>
+      <c r="E18" s="134">
+        <v>3.55</v>
+      </c>
+      <c r="G18" s="133" t="s">
+        <v>226</v>
+      </c>
+      <c r="H18" s="134" t="s">
+        <v>251</v>
+      </c>
+      <c r="I18" s="134" t="s">
+        <v>252</v>
+      </c>
+      <c r="J18" s="134" t="s">
+        <v>253</v>
+      </c>
+      <c r="L18" s="133" t="s">
+        <v>226</v>
+      </c>
+      <c r="M18" s="134" t="s">
+        <v>254</v>
+      </c>
+      <c r="N18" s="134" t="s">
+        <v>253</v>
+      </c>
+      <c r="O18" s="134" t="s">
+        <v>255</v>
+      </c>
+      <c r="Q18" s="133" t="s">
+        <v>226</v>
+      </c>
+      <c r="R18" s="134" t="s">
+        <v>255</v>
+      </c>
+      <c r="S18" s="134" t="s">
+        <v>256</v>
+      </c>
+      <c r="T18" s="134" t="s">
+        <v>257</v>
+      </c>
+      <c r="V18" s="133" t="s">
+        <v>226</v>
+      </c>
+      <c r="W18" s="134" t="s">
+        <v>257</v>
+      </c>
+      <c r="X18" s="134" t="s">
+        <v>258</v>
+      </c>
+      <c r="Y18" s="134" t="s">
+        <v>259</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
 

</xml_diff>

<commit_message>
Testing at ideal conditions on PCB in open loop completed for Output Voltage
</commit_message>
<xml_diff>
--- a/Excel/Boost Converter Design Params.xlsx
+++ b/Excel/Boost Converter Design Params.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\tytom\Documents\GitHub\311\Excel\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8FA943A1-BAC0-4164-9636-0C29EC94EDB1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{07F6AA57-F7B5-4DB7-BA1F-3183BF8002B4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="2" xr2:uid="{0EA872C3-4804-43CB-9F0B-5F94DB7B4351}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="527" uniqueCount="260">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="552" uniqueCount="266">
   <si>
     <t>Parameter</t>
   </si>
@@ -816,6 +816,24 @@
   </si>
   <si>
     <t>4.3V</t>
+  </si>
+  <si>
+    <t>Testing on PCB in Open Loop (Ideal Conditions)</t>
+  </si>
+  <si>
+    <t>Rl = 5</t>
+  </si>
+  <si>
+    <t>Rl = 20</t>
+  </si>
+  <si>
+    <t>Rl = 30</t>
+  </si>
+  <si>
+    <t>Rl = 40</t>
+  </si>
+  <si>
+    <t>Rl = 50</t>
   </si>
 </sst>
 </file>
@@ -907,7 +925,7 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="9">
+  <fills count="13">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -945,7 +963,30 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
+        <fgColor rgb="FFFFFFCC"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
         <fgColor theme="4" tint="0.59999389629810485"/>
+        <bgColor indexed="65"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="5" tint="0.59999389629810485"/>
+        <bgColor indexed="65"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="5" tint="0.39997558519241921"/>
+        <bgColor indexed="65"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="7" tint="0.59999389629810485"/>
         <bgColor indexed="65"/>
       </patternFill>
     </fill>
@@ -956,7 +997,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="65">
+  <borders count="66">
     <border>
       <left/>
       <right/>
@@ -1860,16 +1901,35 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color rgb="FFB2B2B2"/>
+      </left>
+      <right style="thin">
+        <color rgb="FFB2B2B2"/>
+      </right>
+      <top style="thin">
+        <color rgb="FFB2B2B2"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FFB2B2B2"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
-  <cellStyleXfs count="6">
+  <cellStyleXfs count="10">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="1" applyNumberFormat="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="1" fillId="3" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="1" fillId="7" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="1" fillId="7" borderId="65" applyNumberFormat="0" applyFont="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="1" fillId="8" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="1" fillId="9" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="1" fillId="10" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="1" fillId="11" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="1" fillId="12" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="136">
+  <cellXfs count="141">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
@@ -2018,17 +2078,26 @@
     <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="2" applyFont="1" applyBorder="1"/>
     <xf numFmtId="167" fontId="0" fillId="0" borderId="34" xfId="0" applyNumberFormat="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="1" fillId="7" borderId="0" xfId="4"/>
+    <xf numFmtId="0" fontId="1" fillId="8" borderId="0" xfId="5"/>
     <xf numFmtId="0" fontId="1" fillId="3" borderId="0" xfId="2"/>
-    <xf numFmtId="0" fontId="1" fillId="8" borderId="0" xfId="5"/>
-    <xf numFmtId="9" fontId="1" fillId="8" borderId="0" xfId="5" applyNumberFormat="1"/>
+    <xf numFmtId="0" fontId="1" fillId="12" borderId="0" xfId="9"/>
+    <xf numFmtId="9" fontId="1" fillId="12" borderId="0" xfId="9" applyNumberFormat="1"/>
+    <xf numFmtId="0" fontId="1" fillId="11" borderId="0" xfId="8"/>
+    <xf numFmtId="0" fontId="1" fillId="9" borderId="0" xfId="6"/>
+    <xf numFmtId="0" fontId="1" fillId="10" borderId="0" xfId="7"/>
+    <xf numFmtId="0" fontId="1" fillId="7" borderId="65" xfId="4"/>
+    <xf numFmtId="9" fontId="1" fillId="7" borderId="65" xfId="4" applyNumberFormat="1"/>
   </cellXfs>
-  <cellStyles count="6">
+  <cellStyles count="10">
     <cellStyle name="20% - Accent1" xfId="2" builtinId="30"/>
-    <cellStyle name="20% - Accent6" xfId="5" builtinId="50"/>
-    <cellStyle name="40% - Accent1" xfId="4" builtinId="31"/>
+    <cellStyle name="20% - Accent6" xfId="9" builtinId="50"/>
+    <cellStyle name="40% - Accent1" xfId="5" builtinId="31"/>
+    <cellStyle name="40% - Accent2" xfId="6" builtinId="35"/>
+    <cellStyle name="40% - Accent4" xfId="8" builtinId="43"/>
+    <cellStyle name="60% - Accent2" xfId="7" builtinId="36"/>
     <cellStyle name="Check Cell" xfId="1" builtinId="23"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
+    <cellStyle name="Note" xfId="4" builtinId="10"/>
     <cellStyle name="Percent" xfId="3" builtinId="5"/>
   </cellStyles>
   <dxfs count="0"/>
@@ -5051,13 +5120,16 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{86BA37C4-8F32-417F-A8E4-D80C296F90D3}">
-  <dimension ref="B2:Y18"/>
+  <dimension ref="B2:AD27"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <sheetData>
     <row r="2" spans="2:25" x14ac:dyDescent="0.3">
-      <c r="B2" s="129" t="s">
+      <c r="B2" s="136" t="s">
         <v>220</v>
       </c>
+      <c r="C2" s="136"/>
+      <c r="D2" s="136"/>
+      <c r="E2" s="136"/>
     </row>
     <row r="3" spans="2:25" x14ac:dyDescent="0.3">
       <c r="B3" t="s">
@@ -5332,7 +5404,7 @@
         <v>3.5</v>
       </c>
     </row>
-    <row r="17" spans="2:25" x14ac:dyDescent="0.3">
+    <row r="17" spans="2:30" x14ac:dyDescent="0.3">
       <c r="B17" s="133" t="s">
         <v>249</v>
       </c>
@@ -5394,7 +5466,7 @@
         <v>0.3</v>
       </c>
     </row>
-    <row r="18" spans="2:25" x14ac:dyDescent="0.3">
+    <row r="18" spans="2:30" x14ac:dyDescent="0.3">
       <c r="B18" s="133" t="s">
         <v>226</v>
       </c>
@@ -5454,6 +5526,275 @@
       </c>
       <c r="Y18" s="134" t="s">
         <v>259</v>
+      </c>
+    </row>
+    <row r="22" spans="2:30" x14ac:dyDescent="0.3">
+      <c r="B22" s="138" t="s">
+        <v>260</v>
+      </c>
+      <c r="C22" s="138"/>
+      <c r="D22" s="138"/>
+      <c r="E22" s="138"/>
+      <c r="F22" s="138"/>
+    </row>
+    <row r="24" spans="2:30" x14ac:dyDescent="0.3">
+      <c r="B24" s="138" t="s">
+        <v>261</v>
+      </c>
+      <c r="C24" s="138"/>
+      <c r="D24" s="138"/>
+      <c r="E24" s="138"/>
+      <c r="G24" s="138" t="s">
+        <v>240</v>
+      </c>
+      <c r="H24" s="138"/>
+      <c r="I24" s="138"/>
+      <c r="J24" s="138"/>
+      <c r="L24" s="138" t="s">
+        <v>262</v>
+      </c>
+      <c r="M24" s="138"/>
+      <c r="N24" s="138"/>
+      <c r="O24" s="138"/>
+      <c r="Q24" s="138" t="s">
+        <v>263</v>
+      </c>
+      <c r="R24" s="138"/>
+      <c r="S24" s="138"/>
+      <c r="T24" s="138"/>
+      <c r="V24" s="138" t="s">
+        <v>264</v>
+      </c>
+      <c r="W24" s="138"/>
+      <c r="X24" s="138"/>
+      <c r="Y24" s="138"/>
+      <c r="AA24" s="138" t="s">
+        <v>265</v>
+      </c>
+      <c r="AB24" s="138"/>
+      <c r="AC24" s="138"/>
+      <c r="AD24" s="138"/>
+    </row>
+    <row r="25" spans="2:30" x14ac:dyDescent="0.3">
+      <c r="B25" s="137" t="s">
+        <v>248</v>
+      </c>
+      <c r="C25" s="139">
+        <v>2.5</v>
+      </c>
+      <c r="D25" s="139">
+        <v>3</v>
+      </c>
+      <c r="E25" s="139">
+        <v>3.5</v>
+      </c>
+      <c r="G25" s="137" t="s">
+        <v>248</v>
+      </c>
+      <c r="H25" s="139">
+        <v>2.5</v>
+      </c>
+      <c r="I25" s="139">
+        <v>3</v>
+      </c>
+      <c r="J25" s="139">
+        <v>3.5</v>
+      </c>
+      <c r="L25" s="137" t="s">
+        <v>248</v>
+      </c>
+      <c r="M25" s="139">
+        <v>2.5</v>
+      </c>
+      <c r="N25" s="139">
+        <v>3</v>
+      </c>
+      <c r="O25" s="139">
+        <v>3.5</v>
+      </c>
+      <c r="Q25" s="137" t="s">
+        <v>248</v>
+      </c>
+      <c r="R25" s="139">
+        <v>2.5</v>
+      </c>
+      <c r="S25" s="139">
+        <v>3</v>
+      </c>
+      <c r="T25" s="139">
+        <v>3.5</v>
+      </c>
+      <c r="V25" s="137" t="s">
+        <v>248</v>
+      </c>
+      <c r="W25" s="139">
+        <v>2.5</v>
+      </c>
+      <c r="X25" s="139">
+        <v>3</v>
+      </c>
+      <c r="Y25" s="139">
+        <v>3.5</v>
+      </c>
+      <c r="AA25" s="137" t="s">
+        <v>248</v>
+      </c>
+      <c r="AB25" s="139">
+        <v>2.5</v>
+      </c>
+      <c r="AC25" s="139">
+        <v>3</v>
+      </c>
+      <c r="AD25" s="139">
+        <v>3.5</v>
+      </c>
+    </row>
+    <row r="26" spans="2:30" x14ac:dyDescent="0.3">
+      <c r="B26" s="137" t="s">
+        <v>249</v>
+      </c>
+      <c r="C26" s="140">
+        <v>0.5</v>
+      </c>
+      <c r="D26" s="140">
+        <v>0.4</v>
+      </c>
+      <c r="E26" s="140">
+        <v>0.3</v>
+      </c>
+      <c r="G26" s="137" t="s">
+        <v>249</v>
+      </c>
+      <c r="H26" s="140">
+        <v>0.5</v>
+      </c>
+      <c r="I26" s="140">
+        <v>0.4</v>
+      </c>
+      <c r="J26" s="140">
+        <v>0.3</v>
+      </c>
+      <c r="L26" s="137" t="s">
+        <v>249</v>
+      </c>
+      <c r="M26" s="140">
+        <v>0.5</v>
+      </c>
+      <c r="N26" s="140">
+        <v>0.4</v>
+      </c>
+      <c r="O26" s="140">
+        <v>0.3</v>
+      </c>
+      <c r="Q26" s="137" t="s">
+        <v>249</v>
+      </c>
+      <c r="R26" s="140">
+        <v>0.5</v>
+      </c>
+      <c r="S26" s="140">
+        <v>0.4</v>
+      </c>
+      <c r="T26" s="140">
+        <v>0.3</v>
+      </c>
+      <c r="V26" s="137" t="s">
+        <v>249</v>
+      </c>
+      <c r="W26" s="140">
+        <v>0.5</v>
+      </c>
+      <c r="X26" s="140">
+        <v>0.4</v>
+      </c>
+      <c r="Y26" s="140">
+        <v>0.3</v>
+      </c>
+      <c r="AA26" s="137" t="s">
+        <v>249</v>
+      </c>
+      <c r="AB26" s="140">
+        <v>0.5</v>
+      </c>
+      <c r="AC26" s="140">
+        <v>0.4</v>
+      </c>
+      <c r="AD26" s="140">
+        <v>0.3</v>
+      </c>
+    </row>
+    <row r="27" spans="2:30" x14ac:dyDescent="0.3">
+      <c r="B27" s="137" t="s">
+        <v>226</v>
+      </c>
+      <c r="C27" s="139">
+        <v>3.75</v>
+      </c>
+      <c r="D27" s="139">
+        <v>3.96</v>
+      </c>
+      <c r="E27" s="139">
+        <v>4.1100000000000003</v>
+      </c>
+      <c r="G27" s="137" t="s">
+        <v>226</v>
+      </c>
+      <c r="H27" s="139">
+        <v>4.16</v>
+      </c>
+      <c r="I27" s="139">
+        <v>4.28</v>
+      </c>
+      <c r="J27" s="139">
+        <v>4.3600000000000003</v>
+      </c>
+      <c r="L27" s="137" t="s">
+        <v>226</v>
+      </c>
+      <c r="M27" s="139">
+        <v>4.38</v>
+      </c>
+      <c r="N27" s="139">
+        <v>4.45</v>
+      </c>
+      <c r="O27" s="139">
+        <v>4.51</v>
+      </c>
+      <c r="Q27" s="137" t="s">
+        <v>226</v>
+      </c>
+      <c r="R27" s="139">
+        <v>4.46</v>
+      </c>
+      <c r="S27" s="139">
+        <v>4.53</v>
+      </c>
+      <c r="T27" s="139">
+        <v>4.5599999999999996</v>
+      </c>
+      <c r="V27" s="137" t="s">
+        <v>226</v>
+      </c>
+      <c r="W27" s="139">
+        <v>4.5199999999999996</v>
+      </c>
+      <c r="X27" s="139">
+        <v>4.5599999999999996</v>
+      </c>
+      <c r="Y27" s="139">
+        <v>4.6100000000000003</v>
+      </c>
+      <c r="AA27" s="137" t="s">
+        <v>226</v>
+      </c>
+      <c r="AB27" s="139">
+        <v>4.55</v>
+      </c>
+      <c r="AC27" s="139">
+        <v>4.5999999999999996</v>
+      </c>
+      <c r="AD27" s="139">
+        <v>4.63</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Duty cycle testing to find values that give us 5V vout, and redo of Open-Loop ideal testing using RT/CT instead of Vg pin for pulse signal input
</commit_message>
<xml_diff>
--- a/Excel/Boost Converter Design Params.xlsx
+++ b/Excel/Boost Converter Design Params.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\tytom\Documents\GitHub\311\Excel\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{07F6AA57-F7B5-4DB7-BA1F-3183BF8002B4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6E5D777D-C834-4A5F-B3C6-4E0724E2A737}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="2" xr2:uid="{0EA872C3-4804-43CB-9F0B-5F94DB7B4351}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="552" uniqueCount="266">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="571" uniqueCount="273">
   <si>
     <t>Parameter</t>
   </si>
@@ -834,6 +834,27 @@
   </si>
   <si>
     <t>Rl = 50</t>
+  </si>
+  <si>
+    <t>Efficiency</t>
+  </si>
+  <si>
+    <t>Pin</t>
+  </si>
+  <si>
+    <t>N/A  (PS Lim)</t>
+  </si>
+  <si>
+    <t>1 - 0.55</t>
+  </si>
+  <si>
+    <t>1 - 0.44</t>
+  </si>
+  <si>
+    <t>1 - 0.63</t>
+  </si>
+  <si>
+    <t>&gt;Testing duty cycle that gives Vout = 5V (less test cases)</t>
   </si>
 </sst>
 </file>
@@ -848,7 +869,7 @@
     <numFmt numFmtId="168" formatCode="0.0000000"/>
     <numFmt numFmtId="169" formatCode="0.0000"/>
   </numFmts>
-  <fonts count="10" x14ac:knownFonts="1">
+  <fonts count="11" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -924,8 +945,16 @@
       <family val="2"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color rgb="FFFA7D00"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
-  <fills count="13">
+  <fills count="14">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -959,6 +988,11 @@
       <patternFill patternType="solid">
         <fgColor theme="0"/>
         <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFF2F2F2"/>
       </patternFill>
     </fill>
     <fill>
@@ -997,7 +1031,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="66">
+  <borders count="67">
     <border>
       <left/>
       <right/>
@@ -1903,6 +1937,21 @@
     </border>
     <border>
       <left style="thin">
+        <color rgb="FF7F7F7F"/>
+      </left>
+      <right style="thin">
+        <color rgb="FF7F7F7F"/>
+      </right>
+      <top style="thin">
+        <color rgb="FF7F7F7F"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FF7F7F7F"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
         <color rgb="FFB2B2B2"/>
       </left>
       <right style="thin">
@@ -1917,19 +1966,20 @@
       <diagonal/>
     </border>
   </borders>
-  <cellStyleXfs count="10">
+  <cellStyleXfs count="11">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="1" applyNumberFormat="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="1" fillId="3" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="1" fillId="7" borderId="65" applyNumberFormat="0" applyFont="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="1" fillId="8" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="10" fillId="7" borderId="65" applyNumberFormat="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="1" fillId="8" borderId="66" applyNumberFormat="0" applyFont="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="1" fillId="9" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="1" fillId="10" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="1" fillId="11" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="1" fillId="12" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="1" fillId="13" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="141">
+  <cellXfs count="146">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
@@ -2078,26 +2128,32 @@
     <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="2" applyFont="1" applyBorder="1"/>
     <xf numFmtId="167" fontId="0" fillId="0" borderId="34" xfId="0" applyNumberFormat="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="1" fillId="8" borderId="0" xfId="5"/>
+    <xf numFmtId="0" fontId="1" fillId="9" borderId="0" xfId="6"/>
     <xf numFmtId="0" fontId="1" fillId="3" borderId="0" xfId="2"/>
+    <xf numFmtId="0" fontId="1" fillId="13" borderId="0" xfId="10"/>
+    <xf numFmtId="9" fontId="1" fillId="13" borderId="0" xfId="10" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="1" fillId="12" borderId="0" xfId="9"/>
-    <xf numFmtId="9" fontId="1" fillId="12" borderId="0" xfId="9" applyNumberFormat="1"/>
+    <xf numFmtId="0" fontId="1" fillId="10" borderId="0" xfId="7"/>
     <xf numFmtId="0" fontId="1" fillId="11" borderId="0" xfId="8"/>
-    <xf numFmtId="0" fontId="1" fillId="9" borderId="0" xfId="6"/>
-    <xf numFmtId="0" fontId="1" fillId="10" borderId="0" xfId="7"/>
-    <xf numFmtId="0" fontId="1" fillId="7" borderId="65" xfId="4"/>
-    <xf numFmtId="9" fontId="1" fillId="7" borderId="65" xfId="4" applyNumberFormat="1"/>
+    <xf numFmtId="0" fontId="1" fillId="8" borderId="66" xfId="5"/>
+    <xf numFmtId="9" fontId="1" fillId="8" borderId="66" xfId="5" applyNumberFormat="1"/>
+    <xf numFmtId="0" fontId="1" fillId="10" borderId="0" xfId="7" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="11" borderId="0" xfId="8" applyBorder="1"/>
+    <xf numFmtId="0" fontId="10" fillId="7" borderId="65" xfId="4"/>
+    <xf numFmtId="0" fontId="0" fillId="8" borderId="66" xfId="5" applyFont="1"/>
+    <xf numFmtId="9" fontId="0" fillId="8" borderId="66" xfId="5" applyNumberFormat="1" applyFont="1"/>
   </cellXfs>
-  <cellStyles count="10">
+  <cellStyles count="11">
     <cellStyle name="20% - Accent1" xfId="2" builtinId="30"/>
-    <cellStyle name="20% - Accent6" xfId="9" builtinId="50"/>
-    <cellStyle name="40% - Accent1" xfId="5" builtinId="31"/>
-    <cellStyle name="40% - Accent2" xfId="6" builtinId="35"/>
-    <cellStyle name="40% - Accent4" xfId="8" builtinId="43"/>
-    <cellStyle name="60% - Accent2" xfId="7" builtinId="36"/>
+    <cellStyle name="20% - Accent6" xfId="10" builtinId="50"/>
+    <cellStyle name="40% - Accent1" xfId="6" builtinId="31"/>
+    <cellStyle name="40% - Accent2" xfId="7" builtinId="35"/>
+    <cellStyle name="40% - Accent4" xfId="9" builtinId="43"/>
+    <cellStyle name="60% - Accent2" xfId="8" builtinId="36"/>
+    <cellStyle name="Calculation" xfId="4" builtinId="22"/>
     <cellStyle name="Check Cell" xfId="1" builtinId="23"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
-    <cellStyle name="Note" xfId="4" builtinId="10"/>
+    <cellStyle name="Note" xfId="5" builtinId="10"/>
     <cellStyle name="Percent" xfId="3" builtinId="5"/>
   </cellStyles>
   <dxfs count="0"/>
@@ -5120,7 +5176,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{86BA37C4-8F32-417F-A8E4-D80C296F90D3}">
-  <dimension ref="B2:AD27"/>
+  <dimension ref="B2:AD37"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <sheetData>
     <row r="2" spans="2:25" x14ac:dyDescent="0.3">
@@ -5728,10 +5784,10 @@
         <v>226</v>
       </c>
       <c r="C27" s="139">
-        <v>3.75</v>
+        <v>3.73</v>
       </c>
       <c r="D27" s="139">
-        <v>3.96</v>
+        <v>3.95</v>
       </c>
       <c r="E27" s="139">
         <v>4.1100000000000003</v>
@@ -5740,61 +5796,207 @@
         <v>226</v>
       </c>
       <c r="H27" s="139">
-        <v>4.16</v>
+        <v>4.09</v>
       </c>
       <c r="I27" s="139">
-        <v>4.28</v>
+        <v>4.22</v>
       </c>
       <c r="J27" s="139">
-        <v>4.3600000000000003</v>
+        <v>4.3</v>
       </c>
       <c r="L27" s="137" t="s">
         <v>226</v>
       </c>
       <c r="M27" s="139">
+        <v>4.28</v>
+      </c>
+      <c r="N27" s="139">
         <v>4.38</v>
       </c>
-      <c r="N27" s="139">
+      <c r="O27" s="139">
         <v>4.45</v>
-      </c>
-      <c r="O27" s="139">
-        <v>4.51</v>
       </c>
       <c r="Q27" s="137" t="s">
         <v>226</v>
       </c>
       <c r="R27" s="139">
-        <v>4.46</v>
+        <v>4.38</v>
       </c>
       <c r="S27" s="139">
-        <v>4.53</v>
+        <v>4.45</v>
       </c>
       <c r="T27" s="139">
-        <v>4.5599999999999996</v>
+        <v>4.51</v>
       </c>
       <c r="V27" s="137" t="s">
         <v>226</v>
       </c>
       <c r="W27" s="139">
-        <v>4.5199999999999996</v>
+        <v>4.42</v>
       </c>
       <c r="X27" s="139">
-        <v>4.5599999999999996</v>
+        <v>4.49</v>
       </c>
       <c r="Y27" s="139">
-        <v>4.6100000000000003</v>
+        <v>4.53</v>
       </c>
       <c r="AA27" s="137" t="s">
         <v>226</v>
       </c>
       <c r="AB27" s="139">
+        <v>4.47</v>
+      </c>
+      <c r="AC27" s="139">
+        <v>4.5</v>
+      </c>
+      <c r="AD27" s="139">
         <v>4.55</v>
       </c>
-      <c r="AC27" s="139">
-        <v>4.5999999999999996</v>
-      </c>
-      <c r="AD27" s="139">
-        <v>4.63</v>
+    </row>
+    <row r="29" spans="2:30" x14ac:dyDescent="0.3">
+      <c r="B29" s="142" t="s">
+        <v>272</v>
+      </c>
+      <c r="C29" s="138"/>
+      <c r="D29" s="138"/>
+      <c r="E29" s="138"/>
+      <c r="F29" s="138"/>
+      <c r="G29" s="138"/>
+    </row>
+    <row r="31" spans="2:30" x14ac:dyDescent="0.3">
+      <c r="B31" s="142" t="s">
+        <v>261</v>
+      </c>
+      <c r="C31" s="138"/>
+      <c r="D31" s="138"/>
+      <c r="F31" s="138" t="s">
+        <v>265</v>
+      </c>
+      <c r="G31" s="138"/>
+      <c r="H31" s="138"/>
+    </row>
+    <row r="32" spans="2:30" x14ac:dyDescent="0.3">
+      <c r="B32" s="137" t="s">
+        <v>248</v>
+      </c>
+      <c r="C32" s="143">
+        <v>2.5</v>
+      </c>
+      <c r="D32" s="143">
+        <v>3.5</v>
+      </c>
+      <c r="F32" s="137" t="s">
+        <v>248</v>
+      </c>
+      <c r="G32" s="143">
+        <v>2.5</v>
+      </c>
+      <c r="H32" s="143">
+        <v>3.5</v>
+      </c>
+    </row>
+    <row r="33" spans="2:8" x14ac:dyDescent="0.3">
+      <c r="B33" s="141" t="s">
+        <v>249</v>
+      </c>
+      <c r="C33" s="144" t="s">
+        <v>268</v>
+      </c>
+      <c r="D33" s="144" t="s">
+        <v>269</v>
+      </c>
+      <c r="F33" s="137" t="s">
+        <v>249</v>
+      </c>
+      <c r="G33" s="144" t="s">
+        <v>270</v>
+      </c>
+      <c r="H33" s="144" t="s">
+        <v>271</v>
+      </c>
+    </row>
+    <row r="34" spans="2:8" x14ac:dyDescent="0.3">
+      <c r="B34" s="137" t="s">
+        <v>226</v>
+      </c>
+      <c r="C34" s="144">
+        <v>4.7</v>
+      </c>
+      <c r="D34" s="144">
+        <v>4.97</v>
+      </c>
+      <c r="F34" s="137" t="s">
+        <v>226</v>
+      </c>
+      <c r="G34" s="144">
+        <v>5.05</v>
+      </c>
+      <c r="H34" s="144">
+        <v>5.03</v>
+      </c>
+    </row>
+    <row r="35" spans="2:8" x14ac:dyDescent="0.3">
+      <c r="B35" s="141" t="s">
+        <v>266</v>
+      </c>
+      <c r="C35" s="145">
+        <f>(C37/C36)</f>
+        <v>0.60606060606060608</v>
+      </c>
+      <c r="D35" s="145">
+        <f>D37/D36</f>
+        <v>0.82258064516129026</v>
+      </c>
+      <c r="F35" s="141" t="s">
+        <v>266</v>
+      </c>
+      <c r="G35" s="145">
+        <f>G37/G36</f>
+        <v>0.91228070175438603</v>
+      </c>
+      <c r="H35" s="145">
+        <f>H37/H36</f>
+        <v>0.9107142857142857</v>
+      </c>
+    </row>
+    <row r="36" spans="2:8" x14ac:dyDescent="0.3">
+      <c r="B36" s="141" t="s">
+        <v>267</v>
+      </c>
+      <c r="C36" s="144">
+        <v>7.26</v>
+      </c>
+      <c r="D36" s="144">
+        <v>6.2</v>
+      </c>
+      <c r="F36" s="141" t="s">
+        <v>267</v>
+      </c>
+      <c r="G36" s="144">
+        <v>0.56999999999999995</v>
+      </c>
+      <c r="H36" s="144">
+        <v>0.56000000000000005</v>
+      </c>
+    </row>
+    <row r="37" spans="2:8" x14ac:dyDescent="0.3">
+      <c r="B37" s="141" t="s">
+        <v>15</v>
+      </c>
+      <c r="C37" s="144">
+        <v>4.4000000000000004</v>
+      </c>
+      <c r="D37" s="144">
+        <v>5.0999999999999996</v>
+      </c>
+      <c r="F37" s="141" t="s">
+        <v>15</v>
+      </c>
+      <c r="G37" s="144">
+        <v>0.52</v>
+      </c>
+      <c r="H37" s="144">
+        <v>0.51</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Overvoltage values placed in
</commit_message>
<xml_diff>
--- a/Excel/Boost Converter Design Params.xlsx
+++ b/Excel/Boost Converter Design Params.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\tytom\Documents\GitHub\311\Excel\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6E5D777D-C834-4A5F-B3C6-4E0724E2A737}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B9EDA699-65E4-4ADE-BD55-265C6972D713}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="2" xr2:uid="{0EA872C3-4804-43CB-9F0B-5F94DB7B4351}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="571" uniqueCount="273">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="577" uniqueCount="279">
   <si>
     <t>Parameter</t>
   </si>
@@ -855,6 +855,24 @@
   </si>
   <si>
     <t>&gt;Testing duty cycle that gives Vout = 5V (less test cases)</t>
+  </si>
+  <si>
+    <t>At, 65% duty cycle it starts to limit</t>
+  </si>
+  <si>
+    <t>*Overvoltage cannot occur at 5ohms since</t>
+  </si>
+  <si>
+    <t>current is limited to 3A</t>
+  </si>
+  <si>
+    <t>*Overvoltage limits voltage to 5.99V at 3.5V Vin</t>
+  </si>
+  <si>
+    <t>At 65% duty cycle it starts to limit</t>
+  </si>
+  <si>
+    <t>*Overvoltage limits voltage to 5.97V at 2.5V Vin</t>
   </si>
 </sst>
 </file>
@@ -5874,6 +5892,9 @@
       </c>
       <c r="G31" s="138"/>
       <c r="H31" s="138"/>
+      <c r="J31" t="s">
+        <v>276</v>
+      </c>
     </row>
     <row r="32" spans="2:30" x14ac:dyDescent="0.3">
       <c r="B32" s="137" t="s">
@@ -5894,8 +5915,11 @@
       <c r="H32" s="143">
         <v>3.5</v>
       </c>
-    </row>
-    <row r="33" spans="2:8" x14ac:dyDescent="0.3">
+      <c r="J32" t="s">
+        <v>273</v>
+      </c>
+    </row>
+    <row r="33" spans="2:10" x14ac:dyDescent="0.3">
       <c r="B33" s="141" t="s">
         <v>249</v>
       </c>
@@ -5914,8 +5938,11 @@
       <c r="H33" s="144" t="s">
         <v>271</v>
       </c>
-    </row>
-    <row r="34" spans="2:8" x14ac:dyDescent="0.3">
+      <c r="J33" t="s">
+        <v>278</v>
+      </c>
+    </row>
+    <row r="34" spans="2:10" x14ac:dyDescent="0.3">
       <c r="B34" s="137" t="s">
         <v>226</v>
       </c>
@@ -5934,8 +5961,11 @@
       <c r="H34" s="144">
         <v>5.03</v>
       </c>
-    </row>
-    <row r="35" spans="2:8" x14ac:dyDescent="0.3">
+      <c r="J34" t="s">
+        <v>277</v>
+      </c>
+    </row>
+    <row r="35" spans="2:10" x14ac:dyDescent="0.3">
       <c r="B35" s="141" t="s">
         <v>266</v>
       </c>
@@ -5959,7 +5989,7 @@
         <v>0.9107142857142857</v>
       </c>
     </row>
-    <row r="36" spans="2:8" x14ac:dyDescent="0.3">
+    <row r="36" spans="2:10" x14ac:dyDescent="0.3">
       <c r="B36" s="141" t="s">
         <v>267</v>
       </c>
@@ -5978,8 +6008,11 @@
       <c r="H36" s="144">
         <v>0.56000000000000005</v>
       </c>
-    </row>
-    <row r="37" spans="2:8" x14ac:dyDescent="0.3">
+      <c r="J36" t="s">
+        <v>274</v>
+      </c>
+    </row>
+    <row r="37" spans="2:10" x14ac:dyDescent="0.3">
       <c r="B37" s="141" t="s">
         <v>15</v>
       </c>
@@ -5997,6 +6030,9 @@
       </c>
       <c r="H37" s="144">
         <v>0.51</v>
+      </c>
+      <c r="J37" t="s">
+        <v>275</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Matlab script for displaying CSV files created, and results uploaded to Boost Converter Design Params in Open Loop
</commit_message>
<xml_diff>
--- a/Excel/Boost Converter Design Params.xlsx
+++ b/Excel/Boost Converter Design Params.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\tytom\Documents\GitHub\311\Excel\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B9EDA699-65E4-4ADE-BD55-265C6972D713}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DF8CF42E-603F-4387-89D5-19831B881509}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="2" xr2:uid="{0EA872C3-4804-43CB-9F0B-5F94DB7B4351}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="577" uniqueCount="279">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="580" uniqueCount="281">
   <si>
     <t>Parameter</t>
   </si>
@@ -842,18 +842,6 @@
     <t>Pin</t>
   </si>
   <si>
-    <t>N/A  (PS Lim)</t>
-  </si>
-  <si>
-    <t>1 - 0.55</t>
-  </si>
-  <si>
-    <t>1 - 0.44</t>
-  </si>
-  <si>
-    <t>1 - 0.63</t>
-  </si>
-  <si>
     <t>&gt;Testing duty cycle that gives Vout = 5V (less test cases)</t>
   </si>
   <si>
@@ -873,6 +861,24 @@
   </si>
   <si>
     <t>*Overvoltage limits voltage to 5.97V at 2.5V Vin</t>
+  </si>
+  <si>
+    <t>1 - 0.35</t>
+  </si>
+  <si>
+    <t>V ripple</t>
+  </si>
+  <si>
+    <t>1 - 0.47</t>
+  </si>
+  <si>
+    <t>1 - 0.6</t>
+  </si>
+  <si>
+    <t>1 - 0.67</t>
+  </si>
+  <si>
+    <t>Output Voltages as displayed on Oscilloscope - (At boundary conditions - 2.5/3.5V, 5/50ohm)</t>
   </si>
 </sst>
 </file>
@@ -887,7 +893,7 @@
     <numFmt numFmtId="168" formatCode="0.0000000"/>
     <numFmt numFmtId="169" formatCode="0.0000"/>
   </numFmts>
-  <fonts count="11" x14ac:knownFonts="1">
+  <fonts count="11">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -1049,7 +1055,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="67">
+  <borders count="68">
     <border>
       <left/>
       <right/>
@@ -1981,6 +1987,17 @@
       <bottom style="thin">
         <color rgb="FFB2B2B2"/>
       </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="FFB2B2B2"/>
+      </left>
+      <right style="thin">
+        <color rgb="FFB2B2B2"/>
+      </right>
+      <top/>
+      <bottom/>
       <diagonal/>
     </border>
   </borders>
@@ -1997,7 +2014,7 @@
     <xf numFmtId="0" fontId="1" fillId="12" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="1" fillId="13" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="146">
+  <cellXfs count="147">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
@@ -2160,6 +2177,7 @@
     <xf numFmtId="0" fontId="10" fillId="7" borderId="65" xfId="4"/>
     <xf numFmtId="0" fontId="0" fillId="8" borderId="66" xfId="5" applyFont="1"/>
     <xf numFmtId="9" fontId="0" fillId="8" borderId="66" xfId="5" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="0" fontId="0" fillId="8" borderId="67" xfId="5" applyFont="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="11">
     <cellStyle name="20% - Accent1" xfId="2" builtinId="30"/>
@@ -2225,6 +2243,187 @@
         <a:xfrm>
           <a:off x="3352800" y="16101060"/>
           <a:ext cx="3362325" cy="3171825"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+</xdr:wsDr>
+</file>
+
+<file path=xl/drawings/drawing2.xml><?xml version="1.0" encoding="utf-8"?>
+<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>15</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>30</xdr:row>
+      <xdr:rowOff>1</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>26</xdr:col>
+      <xdr:colOff>138545</xdr:colOff>
+      <xdr:row>51</xdr:row>
+      <xdr:rowOff>101120</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="2" name="Picture 1">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{8B7EAD04-260A-155D-294C-837BBD2CBEB4}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId1"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="9144000" y="5403274"/>
+          <a:ext cx="6844145" cy="3883410"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>27</xdr:col>
+      <xdr:colOff>13856</xdr:colOff>
+      <xdr:row>30</xdr:row>
+      <xdr:rowOff>1</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>38</xdr:col>
+      <xdr:colOff>152400</xdr:colOff>
+      <xdr:row>51</xdr:row>
+      <xdr:rowOff>101145</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="3" name="Picture 2">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{81943837-512B-AE1D-34B4-B274ADB0136C}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId2"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="16473056" y="5403274"/>
+          <a:ext cx="6844144" cy="3883435"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>27</xdr:col>
+      <xdr:colOff>1</xdr:colOff>
+      <xdr:row>53</xdr:row>
+      <xdr:rowOff>1</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>38</xdr:col>
+      <xdr:colOff>180109</xdr:colOff>
+      <xdr:row>74</xdr:row>
+      <xdr:rowOff>123910</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="4" name="Picture 3">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{DE26C3D7-8ED7-B892-38C2-88CEB6142C7E}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId3"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="16459201" y="9545783"/>
+          <a:ext cx="6885708" cy="3906200"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>14</xdr:col>
+      <xdr:colOff>554182</xdr:colOff>
+      <xdr:row>53</xdr:row>
+      <xdr:rowOff>-1</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>26</xdr:col>
+      <xdr:colOff>166255</xdr:colOff>
+      <xdr:row>74</xdr:row>
+      <xdr:rowOff>148285</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="5" name="Picture 4">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{1567FB78-D5AF-7633-E768-577C29C1C699}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId4"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="9088582" y="9545781"/>
+          <a:ext cx="6927273" cy="3930577"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -2554,7 +2753,7 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E4C28CAE-7D6E-414C-9BF7-B54583CFEE9E}">
   <dimension ref="A1:N129"/>
-  <sheetFormatPr defaultColWidth="12" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultColWidth="12" defaultRowHeight="14.4"/>
   <cols>
     <col min="1" max="1" width="20.44140625" customWidth="1"/>
     <col min="2" max="2" width="13.5546875" customWidth="1"/>
@@ -2566,18 +2765,18 @@
     <col min="13" max="13" width="18.88671875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" ht="21" x14ac:dyDescent="0.4">
+    <row r="1" spans="1:3" ht="21">
       <c r="A1" s="1" t="s">
         <v>58</v>
       </c>
     </row>
-    <row r="3" spans="1:3" ht="18" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:3" ht="18">
       <c r="A3" s="2" t="s">
         <v>137</v>
       </c>
     </row>
-    <row r="4" spans="1:3" ht="15" thickBot="1" x14ac:dyDescent="0.35"/>
-    <row r="5" spans="1:3" ht="15.6" thickTop="1" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:3" ht="15" thickBot="1"/>
+    <row r="5" spans="1:3" ht="15.6" thickTop="1" thickBot="1">
       <c r="A5" s="3" t="s">
         <v>0</v>
       </c>
@@ -2588,7 +2787,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="6" spans="1:3" ht="15" thickTop="1" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:3" ht="15" thickTop="1">
       <c r="A6" s="37" t="s">
         <v>36</v>
       </c>
@@ -2599,7 +2798,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:3">
       <c r="A7" s="38" t="s">
         <v>37</v>
       </c>
@@ -2610,7 +2809,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="8" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:3">
       <c r="A8" s="38" t="s">
         <v>38</v>
       </c>
@@ -2621,7 +2820,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="9" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:3">
       <c r="A9" s="38" t="s">
         <v>56</v>
       </c>
@@ -2632,7 +2831,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="10" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:3">
       <c r="A10" s="38" t="s">
         <v>57</v>
       </c>
@@ -2643,7 +2842,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="11" spans="1:3" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:3" ht="15" thickBot="1">
       <c r="A11" s="10" t="s">
         <v>5</v>
       </c>
@@ -2654,16 +2853,16 @@
         <v>6</v>
       </c>
     </row>
-    <row r="12" spans="1:3" ht="16.2" thickTop="1" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:3" ht="16.2" thickTop="1">
       <c r="A12" s="13"/>
     </row>
-    <row r="14" spans="1:3" ht="18" x14ac:dyDescent="0.35">
+    <row r="14" spans="1:3" ht="18">
       <c r="A14" s="2" t="s">
         <v>55</v>
       </c>
     </row>
-    <row r="15" spans="1:3" ht="15" thickBot="1" x14ac:dyDescent="0.35"/>
-    <row r="16" spans="1:3" ht="15.6" thickTop="1" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="15" spans="1:3" ht="15" thickBot="1"/>
+    <row r="16" spans="1:3" ht="15.6" thickTop="1" thickBot="1">
       <c r="A16" s="3" t="s">
         <v>0</v>
       </c>
@@ -2674,7 +2873,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="17" spans="1:3" ht="15" thickTop="1" x14ac:dyDescent="0.3">
+    <row r="17" spans="1:3" ht="15" thickTop="1">
       <c r="A17" s="45" t="s">
         <v>41</v>
       </c>
@@ -2686,7 +2885,7 @@
         <v>102</v>
       </c>
     </row>
-    <row r="18" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="18" spans="1:3">
       <c r="A18" s="47" t="s">
         <v>40</v>
       </c>
@@ -2698,7 +2897,7 @@
         <v>103</v>
       </c>
     </row>
-    <row r="19" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="19" spans="1:3">
       <c r="A19" s="56" t="s">
         <v>59</v>
       </c>
@@ -2710,7 +2909,7 @@
         <v>104</v>
       </c>
     </row>
-    <row r="20" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="20" spans="1:3">
       <c r="A20" s="49" t="s">
         <v>60</v>
       </c>
@@ -2722,7 +2921,7 @@
         <v>105</v>
       </c>
     </row>
-    <row r="21" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="21" spans="1:3">
       <c r="A21" s="52" t="s">
         <v>43</v>
       </c>
@@ -2734,7 +2933,7 @@
         <v>106</v>
       </c>
     </row>
-    <row r="22" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="22" spans="1:3">
       <c r="A22" s="52" t="s">
         <v>146</v>
       </c>
@@ -2746,7 +2945,7 @@
         <v>151</v>
       </c>
     </row>
-    <row r="23" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="23" spans="1:3">
       <c r="A23" s="52" t="s">
         <v>44</v>
       </c>
@@ -2758,7 +2957,7 @@
         <v>152</v>
       </c>
     </row>
-    <row r="24" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="24" spans="1:3">
       <c r="A24" s="93" t="s">
         <v>147</v>
       </c>
@@ -2770,7 +2969,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="25" spans="1:3" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="25" spans="1:3" ht="15" thickBot="1">
       <c r="A25" s="85" t="s">
         <v>101</v>
       </c>
@@ -2781,14 +2980,14 @@
         <v>8</v>
       </c>
     </row>
-    <row r="26" spans="1:3" ht="15" thickTop="1" x14ac:dyDescent="0.3"/>
-    <row r="28" spans="1:3" ht="18" x14ac:dyDescent="0.35">
+    <row r="26" spans="1:3" ht="15" thickTop="1"/>
+    <row r="28" spans="1:3" ht="18">
       <c r="A28" s="2" t="s">
         <v>9</v>
       </c>
     </row>
-    <row r="29" spans="1:3" ht="15" thickBot="1" x14ac:dyDescent="0.35"/>
-    <row r="30" spans="1:3" ht="15.6" thickTop="1" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="29" spans="1:3" ht="15" thickBot="1"/>
+    <row r="30" spans="1:3" ht="15.6" thickTop="1" thickBot="1">
       <c r="A30" s="3" t="s">
         <v>0</v>
       </c>
@@ -2799,7 +2998,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="31" spans="1:3" ht="15" thickTop="1" x14ac:dyDescent="0.3">
+    <row r="31" spans="1:3" ht="15" thickTop="1">
       <c r="A31" s="4" t="s">
         <v>10</v>
       </c>
@@ -2810,7 +3009,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="32" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="32" spans="1:3">
       <c r="A32" s="95" t="s">
         <v>148</v>
       </c>
@@ -2822,7 +3021,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="33" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="33" spans="1:11">
       <c r="A33" s="15" t="s">
         <v>11</v>
       </c>
@@ -2834,7 +3033,7 @@
         <v>150</v>
       </c>
     </row>
-    <row r="34" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="34" spans="1:11">
       <c r="A34" s="27" t="s">
         <v>149</v>
       </c>
@@ -2846,7 +3045,7 @@
         <v>107</v>
       </c>
     </row>
-    <row r="35" spans="1:11" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="35" spans="1:11" ht="15" thickBot="1">
       <c r="A35" s="10" t="s">
         <v>12</v>
       </c>
@@ -2857,14 +3056,14 @@
         <v>107</v>
       </c>
     </row>
-    <row r="36" spans="1:11" ht="15" thickTop="1" x14ac:dyDescent="0.3"/>
-    <row r="38" spans="1:11" ht="18" x14ac:dyDescent="0.35">
+    <row r="36" spans="1:11" ht="15" thickTop="1"/>
+    <row r="38" spans="1:11" ht="18">
       <c r="A38" s="2" t="s">
         <v>13</v>
       </c>
     </row>
-    <row r="39" spans="1:11" ht="15" thickBot="1" x14ac:dyDescent="0.35"/>
-    <row r="40" spans="1:11" ht="15.6" thickTop="1" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="39" spans="1:11" ht="15" thickBot="1"/>
+    <row r="40" spans="1:11" ht="15.6" thickTop="1" thickBot="1">
       <c r="A40" s="3" t="s">
         <v>0</v>
       </c>
@@ -2899,7 +3098,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="41" spans="1:11" ht="15" thickTop="1" x14ac:dyDescent="0.3">
+    <row r="41" spans="1:11" ht="15" thickTop="1">
       <c r="A41" s="4" t="s">
         <v>14</v>
       </c>
@@ -2934,7 +3133,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="42" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="42" spans="1:11">
       <c r="A42" s="44" t="s">
         <v>39</v>
       </c>
@@ -2969,7 +3168,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="43" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="43" spans="1:11">
       <c r="A43" s="7" t="s">
         <v>15</v>
       </c>
@@ -3005,7 +3204,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="44" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="44" spans="1:11">
       <c r="A44" s="7" t="s">
         <v>16</v>
       </c>
@@ -3045,7 +3244,7 @@
         <v>108</v>
       </c>
     </row>
-    <row r="45" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="45" spans="1:11">
       <c r="A45" s="7" t="s">
         <v>17</v>
       </c>
@@ -3085,7 +3284,7 @@
         <v>109</v>
       </c>
     </row>
-    <row r="46" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="46" spans="1:11">
       <c r="A46" s="38" t="s">
         <v>46</v>
       </c>
@@ -3125,7 +3324,7 @@
         <v>110</v>
       </c>
     </row>
-    <row r="47" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="47" spans="1:11">
       <c r="A47" s="38" t="s">
         <v>45</v>
       </c>
@@ -3165,7 +3364,7 @@
         <v>111</v>
       </c>
     </row>
-    <row r="48" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="48" spans="1:11">
       <c r="A48" s="7" t="s">
         <v>18</v>
       </c>
@@ -3195,7 +3394,7 @@
       </c>
       <c r="K48" s="23"/>
     </row>
-    <row r="49" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="49" spans="1:14">
       <c r="A49" s="7" t="s">
         <v>48</v>
       </c>
@@ -3235,7 +3434,7 @@
         <v>112</v>
       </c>
     </row>
-    <row r="50" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="50" spans="1:14">
       <c r="A50" s="7" t="s">
         <v>153</v>
       </c>
@@ -3275,7 +3474,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="51" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="51" spans="1:14">
       <c r="A51" s="7" t="s">
         <v>47</v>
       </c>
@@ -3315,7 +3514,7 @@
         <v>113</v>
       </c>
     </row>
-    <row r="52" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="52" spans="1:14">
       <c r="A52" s="27" t="s">
         <v>49</v>
       </c>
@@ -3355,7 +3554,7 @@
         <v>114</v>
       </c>
     </row>
-    <row r="53" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="53" spans="1:14">
       <c r="A53" s="27" t="s">
         <v>51</v>
       </c>
@@ -3395,7 +3594,7 @@
         <v>115</v>
       </c>
     </row>
-    <row r="54" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="54" spans="1:14">
       <c r="A54" s="27" t="s">
         <v>50</v>
       </c>
@@ -3435,7 +3634,7 @@
         <v>116</v>
       </c>
     </row>
-    <row r="55" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="55" spans="1:14">
       <c r="A55" s="7" t="s">
         <v>52</v>
       </c>
@@ -3470,7 +3669,7 @@
         <v>117</v>
       </c>
     </row>
-    <row r="56" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="56" spans="1:14">
       <c r="A56" s="27" t="s">
         <v>53</v>
       </c>
@@ -3514,7 +3713,7 @@
         <v>156</v>
       </c>
     </row>
-    <row r="57" spans="1:14" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="57" spans="1:14" ht="15" thickBot="1">
       <c r="A57" s="10" t="s">
         <v>54</v>
       </c>
@@ -3554,20 +3753,20 @@
         <v>119</v>
       </c>
     </row>
-    <row r="58" spans="1:14" ht="15" thickTop="1" x14ac:dyDescent="0.3">
+    <row r="58" spans="1:14" ht="15" thickTop="1">
       <c r="B58" s="32"/>
       <c r="C58" s="33"/>
     </row>
-    <row r="59" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="59" spans="1:14">
       <c r="B59" s="32"/>
       <c r="C59" s="33"/>
     </row>
-    <row r="60" spans="1:14" ht="18" x14ac:dyDescent="0.35">
+    <row r="60" spans="1:14" ht="18">
       <c r="A60" s="2" t="s">
         <v>19</v>
       </c>
     </row>
-    <row r="62" spans="1:14" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="62" spans="1:14" ht="15" thickBot="1">
       <c r="A62" s="113" t="s">
         <v>0</v>
       </c>
@@ -3600,7 +3799,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="63" spans="1:14" ht="15" thickTop="1" x14ac:dyDescent="0.3">
+    <row r="63" spans="1:14" ht="15" thickTop="1">
       <c r="A63" s="7" t="s">
         <v>16</v>
       </c>
@@ -3640,7 +3839,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="64" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="64" spans="1:14">
       <c r="A64" s="7" t="s">
         <v>17</v>
       </c>
@@ -3670,7 +3869,7 @@
       </c>
       <c r="K64" s="23"/>
     </row>
-    <row r="65" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="65" spans="1:12">
       <c r="A65" s="38" t="s">
         <v>158</v>
       </c>
@@ -3705,7 +3904,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="66" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="66" spans="1:12">
       <c r="A66" s="38" t="s">
         <v>159</v>
       </c>
@@ -3740,7 +3939,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="67" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="67" spans="1:12">
       <c r="A67" s="7" t="s">
         <v>18</v>
       </c>
@@ -3765,7 +3964,7 @@
       </c>
       <c r="K67" s="23"/>
     </row>
-    <row r="68" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="68" spans="1:12">
       <c r="A68" s="38" t="s">
         <v>45</v>
       </c>
@@ -3805,7 +4004,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="69" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="69" spans="1:12">
       <c r="A69" s="7" t="s">
         <v>48</v>
       </c>
@@ -3840,7 +4039,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="70" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="70" spans="1:12">
       <c r="A70" s="7" t="s">
         <v>47</v>
       </c>
@@ -3876,7 +4075,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="71" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="71" spans="1:12">
       <c r="A71" s="27" t="s">
         <v>49</v>
       </c>
@@ -3911,7 +4110,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="72" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="72" spans="1:12">
       <c r="A72" s="27" t="s">
         <v>51</v>
       </c>
@@ -3946,7 +4145,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="73" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="73" spans="1:12">
       <c r="A73" s="27" t="s">
         <v>50</v>
       </c>
@@ -3982,7 +4181,7 @@
       </c>
       <c r="L73" s="106"/>
     </row>
-    <row r="74" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="74" spans="1:12">
       <c r="A74" s="7" t="s">
         <v>52</v>
       </c>
@@ -4017,7 +4216,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="75" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="75" spans="1:12">
       <c r="A75" s="27" t="s">
         <v>53</v>
       </c>
@@ -4052,7 +4251,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="76" spans="1:12" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="76" spans="1:12" ht="15" thickBot="1">
       <c r="A76" s="115" t="s">
         <v>54</v>
       </c>
@@ -4088,14 +4287,14 @@
         <v>160</v>
       </c>
     </row>
-    <row r="77" spans="1:12" ht="15" thickTop="1" x14ac:dyDescent="0.3"/>
-    <row r="79" spans="1:12" ht="18" x14ac:dyDescent="0.35">
+    <row r="77" spans="1:12" ht="15" thickTop="1"/>
+    <row r="79" spans="1:12" ht="18">
       <c r="A79" s="2" t="s">
         <v>22</v>
       </c>
     </row>
-    <row r="80" spans="1:12" ht="15" thickBot="1" x14ac:dyDescent="0.35"/>
-    <row r="81" spans="1:3" ht="15.6" thickTop="1" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="80" spans="1:12" ht="15" thickBot="1"/>
+    <row r="81" spans="1:3" ht="15.6" thickTop="1" thickBot="1">
       <c r="A81" s="3" t="s">
         <v>0</v>
       </c>
@@ -4106,7 +4305,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="82" spans="1:3" ht="15" thickTop="1" x14ac:dyDescent="0.3">
+    <row r="82" spans="1:3" ht="15" thickTop="1">
       <c r="A82" s="4" t="s">
         <v>122</v>
       </c>
@@ -4117,7 +4316,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="83" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="83" spans="1:3">
       <c r="A83" s="15" t="s">
         <v>123</v>
       </c>
@@ -4128,7 +4327,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="84" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="84" spans="1:3">
       <c r="A84" s="15" t="s">
         <v>23</v>
       </c>
@@ -4139,7 +4338,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="85" spans="1:3" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="85" spans="1:3" ht="15.6">
       <c r="A85" s="52" t="s">
         <v>128</v>
       </c>
@@ -4150,7 +4349,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="86" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="86" spans="1:3">
       <c r="A86" s="52" t="s">
         <v>127</v>
       </c>
@@ -4161,7 +4360,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="87" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="87" spans="1:3">
       <c r="A87" s="52" t="s">
         <v>126</v>
       </c>
@@ -4172,7 +4371,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="88" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="88" spans="1:3">
       <c r="A88" s="52" t="s">
         <v>125</v>
       </c>
@@ -4183,7 +4382,7 @@
         <v>132</v>
       </c>
     </row>
-    <row r="89" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="89" spans="1:3">
       <c r="A89" s="52" t="s">
         <v>129</v>
       </c>
@@ -4194,7 +4393,7 @@
         <v>190</v>
       </c>
     </row>
-    <row r="90" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="90" spans="1:3">
       <c r="A90" s="52" t="s">
         <v>130</v>
       </c>
@@ -4205,7 +4404,7 @@
         <v>191</v>
       </c>
     </row>
-    <row r="91" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="91" spans="1:3">
       <c r="A91" s="52" t="s">
         <v>131</v>
       </c>
@@ -4216,7 +4415,7 @@
         <v>133</v>
       </c>
     </row>
-    <row r="92" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="92" spans="1:3">
       <c r="A92" s="52" t="s">
         <v>27</v>
       </c>
@@ -4227,7 +4426,7 @@
         <v>134</v>
       </c>
     </row>
-    <row r="93" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="93" spans="1:3">
       <c r="A93" s="52" t="s">
         <v>28</v>
       </c>
@@ -4238,7 +4437,7 @@
         <v>135</v>
       </c>
     </row>
-    <row r="94" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="94" spans="1:3">
       <c r="A94" s="52" t="s">
         <v>124</v>
       </c>
@@ -4249,7 +4448,7 @@
         <v>136</v>
       </c>
     </row>
-    <row r="95" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="95" spans="1:3">
       <c r="A95" s="15" t="s">
         <v>120</v>
       </c>
@@ -4260,7 +4459,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="96" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="96" spans="1:3">
       <c r="A96" s="15" t="s">
         <v>121</v>
       </c>
@@ -4271,7 +4470,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="97" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="97" spans="1:11">
       <c r="A97" s="52" t="s">
         <v>163</v>
       </c>
@@ -4282,7 +4481,7 @@
         <v>162</v>
       </c>
     </row>
-    <row r="98" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="98" spans="1:11">
       <c r="A98" s="15" t="s">
         <v>30</v>
       </c>
@@ -4291,7 +4490,7 @@
       </c>
       <c r="C98" s="18"/>
     </row>
-    <row r="99" spans="1:11" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="99" spans="1:11" ht="15" thickBot="1">
       <c r="A99" s="10" t="s">
         <v>31</v>
       </c>
@@ -4300,14 +4499,14 @@
       </c>
       <c r="C99" s="19"/>
     </row>
-    <row r="100" spans="1:11" ht="15" thickTop="1" x14ac:dyDescent="0.3"/>
-    <row r="102" spans="1:11" ht="18" x14ac:dyDescent="0.35">
+    <row r="100" spans="1:11" ht="15" thickTop="1"/>
+    <row r="102" spans="1:11" ht="18">
       <c r="A102" s="2" t="s">
         <v>32</v>
       </c>
     </row>
-    <row r="103" spans="1:11" ht="15" thickBot="1" x14ac:dyDescent="0.35"/>
-    <row r="104" spans="1:11" ht="15.6" thickTop="1" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="103" spans="1:11" ht="15" thickBot="1"/>
+    <row r="104" spans="1:11" ht="15.6" thickTop="1" thickBot="1">
       <c r="A104" s="3" t="s">
         <v>0</v>
       </c>
@@ -4338,7 +4537,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="105" spans="1:11" ht="15" thickTop="1" x14ac:dyDescent="0.3">
+    <row r="105" spans="1:11" ht="15" thickTop="1">
       <c r="A105" s="7" t="s">
         <v>16</v>
       </c>
@@ -4377,7 +4576,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="106" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="106" spans="1:11">
       <c r="A106" s="7" t="s">
         <v>33</v>
       </c>
@@ -4412,7 +4611,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="107" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="107" spans="1:11">
       <c r="A107" s="38" t="s">
         <v>161</v>
       </c>
@@ -4447,7 +4646,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="108" spans="1:11" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="108" spans="1:11" ht="15" thickBot="1">
       <c r="A108" s="10" t="s">
         <v>34</v>
       </c>
@@ -4482,14 +4681,14 @@
         <v>35</v>
       </c>
     </row>
-    <row r="109" spans="1:11" ht="15" thickTop="1" x14ac:dyDescent="0.3"/>
-    <row r="111" spans="1:11" ht="18" x14ac:dyDescent="0.35">
+    <row r="109" spans="1:11" ht="15" thickTop="1"/>
+    <row r="111" spans="1:11" ht="18">
       <c r="A111" s="2" t="s">
         <v>164</v>
       </c>
     </row>
-    <row r="112" spans="1:11" ht="15" thickBot="1" x14ac:dyDescent="0.35"/>
-    <row r="113" spans="1:8" ht="15.6" thickTop="1" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="112" spans="1:11" ht="15" thickBot="1"/>
+    <row r="113" spans="1:8" ht="15.6" thickTop="1" thickBot="1">
       <c r="A113" s="3" t="s">
         <v>0</v>
       </c>
@@ -4509,7 +4708,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="114" spans="1:8" ht="15" thickTop="1" x14ac:dyDescent="0.3">
+    <row r="114" spans="1:8" ht="15" thickTop="1">
       <c r="A114" s="38" t="s">
         <v>165</v>
       </c>
@@ -4529,7 +4728,7 @@
         <v>184</v>
       </c>
     </row>
-    <row r="115" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="115" spans="1:8">
       <c r="A115" s="38" t="s">
         <v>172</v>
       </c>
@@ -4549,7 +4748,7 @@
         <v>184</v>
       </c>
     </row>
-    <row r="116" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="116" spans="1:8">
       <c r="A116" s="38" t="s">
         <v>178</v>
       </c>
@@ -4569,7 +4768,7 @@
         <v>183</v>
       </c>
     </row>
-    <row r="117" spans="1:8" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="117" spans="1:8" ht="15" thickBot="1">
       <c r="A117" s="85" t="s">
         <v>170</v>
       </c>
@@ -4589,7 +4788,7 @@
         <v>177</v>
       </c>
     </row>
-    <row r="118" spans="1:8" ht="15.6" thickTop="1" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="118" spans="1:8" ht="15.6" thickTop="1" thickBot="1">
       <c r="A118" s="85" t="s">
         <v>185</v>
       </c>
@@ -4609,13 +4808,13 @@
         <v>188</v>
       </c>
     </row>
-    <row r="119" spans="1:8" ht="15" thickTop="1" x14ac:dyDescent="0.3"/>
-    <row r="120" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="119" spans="1:8" ht="15" thickTop="1"/>
+    <row r="120" spans="1:8">
       <c r="A120" s="129" t="s">
         <v>212</v>
       </c>
     </row>
-    <row r="121" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="121" spans="1:8">
       <c r="A121" s="130" t="s">
         <v>206</v>
       </c>
@@ -4623,12 +4822,12 @@
         <v>203</v>
       </c>
     </row>
-    <row r="122" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="122" spans="1:8">
       <c r="A122" s="130" t="s">
         <v>205</v>
       </c>
     </row>
-    <row r="123" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="123" spans="1:8">
       <c r="A123" s="130" t="s">
         <v>207</v>
       </c>
@@ -4636,7 +4835,7 @@
         <v>204</v>
       </c>
     </row>
-    <row r="124" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="124" spans="1:8">
       <c r="A124" s="130" t="s">
         <v>219</v>
       </c>
@@ -4644,12 +4843,12 @@
         <v>208</v>
       </c>
     </row>
-    <row r="125" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="125" spans="1:8">
       <c r="A125" s="129" t="s">
         <v>213</v>
       </c>
     </row>
-    <row r="126" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="126" spans="1:8">
       <c r="A126" s="130" t="s">
         <v>209</v>
       </c>
@@ -4657,12 +4856,12 @@
         <v>211</v>
       </c>
     </row>
-    <row r="127" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="127" spans="1:8">
       <c r="A127" s="130" t="s">
         <v>210</v>
       </c>
     </row>
-    <row r="128" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="128" spans="1:8">
       <c r="A128" s="130" t="s">
         <v>214</v>
       </c>
@@ -4670,7 +4869,7 @@
         <v>215</v>
       </c>
     </row>
-    <row r="129" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="129" spans="1:2">
       <c r="A129" s="130" t="s">
         <v>216</v>
       </c>
@@ -4689,24 +4888,24 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{3F74A05D-7210-44AC-859D-2846F0884F7B}">
   <dimension ref="A1:G56"/>
-  <sheetFormatPr defaultColWidth="12" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultColWidth="12" defaultRowHeight="14.4"/>
   <cols>
     <col min="1" max="1" width="24.44140625" customWidth="1"/>
     <col min="2" max="9" width="12.88671875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5" ht="21" x14ac:dyDescent="0.4">
+    <row r="1" spans="1:5" ht="21">
       <c r="A1" s="1" t="s">
         <v>90</v>
       </c>
     </row>
-    <row r="3" spans="1:5" ht="18" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:5" ht="18">
       <c r="A3" s="2" t="s">
         <v>61</v>
       </c>
     </row>
-    <row r="4" spans="1:5" ht="15" thickBot="1" x14ac:dyDescent="0.35"/>
-    <row r="5" spans="1:5" ht="15.6" thickTop="1" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:5" ht="15" thickBot="1"/>
+    <row r="5" spans="1:5" ht="15.6" thickTop="1" thickBot="1">
       <c r="A5" s="3" t="s">
         <v>0</v>
       </c>
@@ -4718,7 +4917,7 @@
       </c>
       <c r="E5" s="73"/>
     </row>
-    <row r="6" spans="1:5" ht="15" thickTop="1" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:5" ht="15" thickTop="1">
       <c r="A6" s="37" t="s">
         <v>101</v>
       </c>
@@ -4730,7 +4929,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="7" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:5">
       <c r="A7" s="38" t="s">
         <v>92</v>
       </c>
@@ -4742,7 +4941,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="8" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:5">
       <c r="A8" s="38" t="s">
         <v>93</v>
       </c>
@@ -4754,7 +4953,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="9" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:5">
       <c r="A9" s="38" t="s">
         <v>91</v>
       </c>
@@ -4766,7 +4965,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="10" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:5">
       <c r="A10" s="7" t="s">
         <v>62</v>
       </c>
@@ -4777,7 +4976,7 @@
         <v>63</v>
       </c>
     </row>
-    <row r="11" spans="1:5" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:5" ht="15" thickBot="1">
       <c r="A11" s="10" t="s">
         <v>5</v>
       </c>
@@ -4789,18 +4988,18 @@
         <v>6</v>
       </c>
     </row>
-    <row r="12" spans="1:5" ht="16.2" thickTop="1" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:5" ht="16.2" thickTop="1">
       <c r="A12" s="13"/>
     </row>
-    <row r="14" spans="1:5" ht="18" x14ac:dyDescent="0.35">
+    <row r="14" spans="1:5" ht="18">
       <c r="A14" s="2" t="s">
         <v>64</v>
       </c>
     </row>
-    <row r="15" spans="1:5" ht="18.600000000000001" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="15" spans="1:5" ht="18.600000000000001" thickBot="1">
       <c r="A15" s="2"/>
     </row>
-    <row r="16" spans="1:5" ht="15.6" thickTop="1" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="16" spans="1:5" ht="15.6" thickTop="1" thickBot="1">
       <c r="A16" s="3" t="s">
         <v>0</v>
       </c>
@@ -4811,7 +5010,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="17" spans="1:3" ht="15" thickTop="1" x14ac:dyDescent="0.3">
+    <row r="17" spans="1:3" ht="15" thickTop="1">
       <c r="A17" s="59" t="s">
         <v>65</v>
       </c>
@@ -4820,7 +5019,7 @@
       </c>
       <c r="C17" s="61"/>
     </row>
-    <row r="18" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="18" spans="1:3">
       <c r="A18" s="62" t="s">
         <v>67</v>
       </c>
@@ -4829,7 +5028,7 @@
       </c>
       <c r="C18" s="64"/>
     </row>
-    <row r="19" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="19" spans="1:3">
       <c r="A19" s="62" t="s">
         <v>69</v>
       </c>
@@ -4840,7 +5039,7 @@
         <v>70</v>
       </c>
     </row>
-    <row r="20" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="20" spans="1:3">
       <c r="A20" s="62" t="s">
         <v>71</v>
       </c>
@@ -4851,7 +5050,7 @@
         <v>72</v>
       </c>
     </row>
-    <row r="21" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="21" spans="1:3">
       <c r="A21" s="62" t="s">
         <v>73</v>
       </c>
@@ -4862,7 +5061,7 @@
         <v>74</v>
       </c>
     </row>
-    <row r="22" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="22" spans="1:3">
       <c r="A22" s="62" t="s">
         <v>75</v>
       </c>
@@ -4873,7 +5072,7 @@
         <v>70</v>
       </c>
     </row>
-    <row r="23" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="23" spans="1:3">
       <c r="A23" s="62" t="s">
         <v>76</v>
       </c>
@@ -4884,7 +5083,7 @@
         <v>72</v>
       </c>
     </row>
-    <row r="24" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="24" spans="1:3">
       <c r="A24" s="62" t="s">
         <v>77</v>
       </c>
@@ -4896,7 +5095,7 @@
         <v>78</v>
       </c>
     </row>
-    <row r="25" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="25" spans="1:3">
       <c r="A25" s="62" t="s">
         <v>79</v>
       </c>
@@ -4908,7 +5107,7 @@
         <v>80</v>
       </c>
     </row>
-    <row r="26" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="26" spans="1:3">
       <c r="A26" s="67" t="s">
         <v>81</v>
       </c>
@@ -4916,7 +5115,7 @@
         <v>1510</v>
       </c>
     </row>
-    <row r="27" spans="1:3" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="27" spans="1:3" ht="15" thickBot="1">
       <c r="A27" s="68" t="s">
         <v>82</v>
       </c>
@@ -4925,14 +5124,14 @@
       </c>
       <c r="C27" s="70"/>
     </row>
-    <row r="28" spans="1:3" ht="15" thickTop="1" x14ac:dyDescent="0.3"/>
-    <row r="30" spans="1:3" ht="18" x14ac:dyDescent="0.35">
+    <row r="28" spans="1:3" ht="15" thickTop="1"/>
+    <row r="30" spans="1:3" ht="18">
       <c r="A30" s="2" t="s">
         <v>83</v>
       </c>
     </row>
-    <row r="31" spans="1:3" ht="15" thickBot="1" x14ac:dyDescent="0.35"/>
-    <row r="32" spans="1:3" ht="15.6" thickTop="1" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="31" spans="1:3" ht="15" thickBot="1"/>
+    <row r="32" spans="1:3" ht="15.6" thickTop="1" thickBot="1">
       <c r="A32" s="3" t="s">
         <v>0</v>
       </c>
@@ -4943,7 +5142,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="33" spans="1:7" ht="15" thickTop="1" x14ac:dyDescent="0.3">
+    <row r="33" spans="1:7" ht="15" thickTop="1">
       <c r="A33" s="59" t="s">
         <v>84</v>
       </c>
@@ -4955,7 +5154,7 @@
       </c>
       <c r="G33" s="73"/>
     </row>
-    <row r="34" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="34" spans="1:7">
       <c r="A34" s="74" t="s">
         <v>194</v>
       </c>
@@ -4968,7 +5167,7 @@
       </c>
       <c r="G34" s="73"/>
     </row>
-    <row r="35" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="35" spans="1:7">
       <c r="A35" s="74" t="s">
         <v>85</v>
       </c>
@@ -4982,7 +5181,7 @@
       <c r="F35" s="78"/>
       <c r="G35" s="73"/>
     </row>
-    <row r="36" spans="1:7" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="36" spans="1:7" ht="15.6">
       <c r="A36" s="74" t="s">
         <v>86</v>
       </c>
@@ -4995,7 +5194,7 @@
       <c r="F36" s="13"/>
       <c r="G36" s="13"/>
     </row>
-    <row r="37" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="37" spans="1:7">
       <c r="A37" s="74" t="s">
         <v>87</v>
       </c>
@@ -5007,7 +5206,7 @@
         <v>141</v>
       </c>
     </row>
-    <row r="38" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="38" spans="1:7">
       <c r="A38" s="81" t="s">
         <v>95</v>
       </c>
@@ -5018,7 +5217,7 @@
         <v>72</v>
       </c>
     </row>
-    <row r="39" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="39" spans="1:7">
       <c r="A39" s="81" t="s">
         <v>94</v>
       </c>
@@ -5030,7 +5229,7 @@
         <v>142</v>
       </c>
     </row>
-    <row r="40" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="40" spans="1:7">
       <c r="A40" s="81" t="s">
         <v>193</v>
       </c>
@@ -5039,7 +5238,7 @@
       </c>
       <c r="C40" s="76"/>
     </row>
-    <row r="41" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="41" spans="1:7">
       <c r="A41" s="81" t="s">
         <v>96</v>
       </c>
@@ -5051,7 +5250,7 @@
         <v>143</v>
       </c>
     </row>
-    <row r="42" spans="1:7" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="42" spans="1:7" ht="15" thickBot="1">
       <c r="A42" s="83" t="s">
         <v>88</v>
       </c>
@@ -5063,7 +5262,7 @@
         <v>144</v>
       </c>
     </row>
-    <row r="43" spans="1:7" ht="15" thickTop="1" x14ac:dyDescent="0.3">
+    <row r="43" spans="1:7" ht="15" thickTop="1">
       <c r="A43" s="125" t="s">
         <v>197</v>
       </c>
@@ -5075,7 +5274,7 @@
         <v>198</v>
       </c>
     </row>
-    <row r="44" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="44" spans="1:7">
       <c r="A44" s="125" t="s">
         <v>195</v>
       </c>
@@ -5087,7 +5286,7 @@
         <v>199</v>
       </c>
     </row>
-    <row r="45" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="45" spans="1:7">
       <c r="A45" s="125" t="s">
         <v>196</v>
       </c>
@@ -5099,7 +5298,7 @@
         <v>200</v>
       </c>
     </row>
-    <row r="46" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="46" spans="1:7">
       <c r="A46" s="74" t="s">
         <v>192</v>
       </c>
@@ -5111,7 +5310,7 @@
         <v>201</v>
       </c>
     </row>
-    <row r="47" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="47" spans="1:7">
       <c r="A47" s="128" t="s">
         <v>202</v>
       </c>
@@ -5123,13 +5322,13 @@
         <v>70</v>
       </c>
     </row>
-    <row r="49" spans="1:3" ht="18" x14ac:dyDescent="0.35">
+    <row r="49" spans="1:3" ht="18">
       <c r="A49" s="2" t="s">
         <v>97</v>
       </c>
     </row>
-    <row r="50" spans="1:3" ht="15" thickBot="1" x14ac:dyDescent="0.35"/>
-    <row r="51" spans="1:3" ht="15.6" thickTop="1" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="50" spans="1:3" ht="15" thickBot="1"/>
+    <row r="51" spans="1:3" ht="15.6" thickTop="1" thickBot="1">
       <c r="A51" s="3" t="s">
         <v>0</v>
       </c>
@@ -5140,7 +5339,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="52" spans="1:3" ht="15" thickTop="1" x14ac:dyDescent="0.3">
+    <row r="52" spans="1:3" ht="15" thickTop="1">
       <c r="A52" s="81" t="s">
         <v>98</v>
       </c>
@@ -5151,7 +5350,7 @@
         <v>89</v>
       </c>
     </row>
-    <row r="53" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="53" spans="1:3">
       <c r="A53" s="74" t="s">
         <v>85</v>
       </c>
@@ -5163,7 +5362,7 @@
         <v>63</v>
       </c>
     </row>
-    <row r="54" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="54" spans="1:3">
       <c r="A54" s="81" t="s">
         <v>145</v>
       </c>
@@ -5174,7 +5373,7 @@
         <v>100</v>
       </c>
     </row>
-    <row r="55" spans="1:3" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="55" spans="1:3" ht="15" thickBot="1">
       <c r="A55" s="82" t="s">
         <v>99</v>
       </c>
@@ -5185,7 +5384,7 @@
         <v>100</v>
       </c>
     </row>
-    <row r="56" spans="1:3" ht="15" thickTop="1" x14ac:dyDescent="0.3"/>
+    <row r="56" spans="1:3" ht="15" thickTop="1"/>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
@@ -5194,10 +5393,10 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{86BA37C4-8F32-417F-A8E4-D80C296F90D3}">
-  <dimension ref="B2:AD37"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <dimension ref="B2:AD38"/>
+  <sheetFormatPr defaultRowHeight="14.4"/>
   <sheetData>
-    <row r="2" spans="2:25" x14ac:dyDescent="0.3">
+    <row r="2" spans="2:25">
       <c r="B2" s="136" t="s">
         <v>220</v>
       </c>
@@ -5205,7 +5404,7 @@
       <c r="D2" s="136"/>
       <c r="E2" s="136"/>
     </row>
-    <row r="3" spans="2:25" x14ac:dyDescent="0.3">
+    <row r="3" spans="2:25">
       <c r="B3" t="s">
         <v>221</v>
       </c>
@@ -5219,7 +5418,7 @@
         <v>224</v>
       </c>
     </row>
-    <row r="4" spans="2:25" x14ac:dyDescent="0.3">
+    <row r="4" spans="2:25">
       <c r="B4">
         <v>5</v>
       </c>
@@ -5239,7 +5438,7 @@
         <v>227</v>
       </c>
     </row>
-    <row r="5" spans="2:25" x14ac:dyDescent="0.3">
+    <row r="5" spans="2:25">
       <c r="B5">
         <v>10</v>
       </c>
@@ -5259,7 +5458,7 @@
         <v>229</v>
       </c>
     </row>
-    <row r="6" spans="2:25" x14ac:dyDescent="0.3">
+    <row r="6" spans="2:25">
       <c r="B6">
         <v>15</v>
       </c>
@@ -5276,7 +5475,7 @@
         <v>231</v>
       </c>
     </row>
-    <row r="7" spans="2:25" x14ac:dyDescent="0.3">
+    <row r="7" spans="2:25">
       <c r="B7">
         <v>20</v>
       </c>
@@ -5290,7 +5489,7 @@
         <v>232</v>
       </c>
     </row>
-    <row r="8" spans="2:25" x14ac:dyDescent="0.3">
+    <row r="8" spans="2:25">
       <c r="B8">
         <v>25</v>
       </c>
@@ -5304,7 +5503,7 @@
         <v>233</v>
       </c>
     </row>
-    <row r="9" spans="2:25" x14ac:dyDescent="0.3">
+    <row r="9" spans="2:25">
       <c r="B9">
         <v>30</v>
       </c>
@@ -5321,7 +5520,7 @@
         <v>235</v>
       </c>
     </row>
-    <row r="10" spans="2:25" x14ac:dyDescent="0.3">
+    <row r="10" spans="2:25">
       <c r="B10">
         <v>35</v>
       </c>
@@ -5338,7 +5537,7 @@
         <v>237</v>
       </c>
     </row>
-    <row r="11" spans="2:25" x14ac:dyDescent="0.3">
+    <row r="11" spans="2:25">
       <c r="B11">
         <v>40</v>
       </c>
@@ -5349,7 +5548,7 @@
         <v>39</v>
       </c>
     </row>
-    <row r="12" spans="2:25" x14ac:dyDescent="0.3">
+    <row r="12" spans="2:25">
       <c r="B12">
         <v>45</v>
       </c>
@@ -5360,7 +5559,7 @@
         <v>47</v>
       </c>
     </row>
-    <row r="13" spans="2:25" x14ac:dyDescent="0.3">
+    <row r="13" spans="2:25">
       <c r="B13">
         <v>50</v>
       </c>
@@ -5374,7 +5573,7 @@
         <v>225</v>
       </c>
     </row>
-    <row r="15" spans="2:25" x14ac:dyDescent="0.3">
+    <row r="15" spans="2:25">
       <c r="B15" s="132" t="s">
         <v>238</v>
       </c>
@@ -5416,7 +5615,7 @@
       <c r="X15" s="132"/>
       <c r="Y15" s="132"/>
     </row>
-    <row r="16" spans="2:25" x14ac:dyDescent="0.3">
+    <row r="16" spans="2:25">
       <c r="B16" s="133" t="s">
         <v>248</v>
       </c>
@@ -5478,7 +5677,7 @@
         <v>3.5</v>
       </c>
     </row>
-    <row r="17" spans="2:30" x14ac:dyDescent="0.3">
+    <row r="17" spans="2:30">
       <c r="B17" s="133" t="s">
         <v>249</v>
       </c>
@@ -5540,7 +5739,7 @@
         <v>0.3</v>
       </c>
     </row>
-    <row r="18" spans="2:30" x14ac:dyDescent="0.3">
+    <row r="18" spans="2:30">
       <c r="B18" s="133" t="s">
         <v>226</v>
       </c>
@@ -5602,7 +5801,7 @@
         <v>259</v>
       </c>
     </row>
-    <row r="22" spans="2:30" x14ac:dyDescent="0.3">
+    <row r="22" spans="2:30">
       <c r="B22" s="138" t="s">
         <v>260</v>
       </c>
@@ -5611,7 +5810,7 @@
       <c r="E22" s="138"/>
       <c r="F22" s="138"/>
     </row>
-    <row r="24" spans="2:30" x14ac:dyDescent="0.3">
+    <row r="24" spans="2:30">
       <c r="B24" s="138" t="s">
         <v>261</v>
       </c>
@@ -5649,7 +5848,7 @@
       <c r="AC24" s="138"/>
       <c r="AD24" s="138"/>
     </row>
-    <row r="25" spans="2:30" x14ac:dyDescent="0.3">
+    <row r="25" spans="2:30">
       <c r="B25" s="137" t="s">
         <v>248</v>
       </c>
@@ -5723,7 +5922,7 @@
         <v>3.5</v>
       </c>
     </row>
-    <row r="26" spans="2:30" x14ac:dyDescent="0.3">
+    <row r="26" spans="2:30">
       <c r="B26" s="137" t="s">
         <v>249</v>
       </c>
@@ -5797,7 +5996,7 @@
         <v>0.3</v>
       </c>
     </row>
-    <row r="27" spans="2:30" x14ac:dyDescent="0.3">
+    <row r="27" spans="2:30">
       <c r="B27" s="137" t="s">
         <v>226</v>
       </c>
@@ -5871,17 +6070,29 @@
         <v>4.55</v>
       </c>
     </row>
-    <row r="29" spans="2:30" x14ac:dyDescent="0.3">
+    <row r="29" spans="2:30">
       <c r="B29" s="142" t="s">
-        <v>272</v>
+        <v>268</v>
       </c>
       <c r="C29" s="138"/>
       <c r="D29" s="138"/>
       <c r="E29" s="138"/>
       <c r="F29" s="138"/>
       <c r="G29" s="138"/>
-    </row>
-    <row r="31" spans="2:30" x14ac:dyDescent="0.3">
+      <c r="P29" s="138" t="s">
+        <v>280</v>
+      </c>
+      <c r="Q29" s="138"/>
+      <c r="R29" s="138"/>
+      <c r="S29" s="138"/>
+      <c r="T29" s="138"/>
+      <c r="U29" s="138"/>
+      <c r="V29" s="138"/>
+      <c r="W29" s="138"/>
+      <c r="X29" s="138"/>
+      <c r="Y29" s="138"/>
+    </row>
+    <row r="31" spans="2:30">
       <c r="B31" s="142" t="s">
         <v>261</v>
       </c>
@@ -5893,10 +6104,10 @@
       <c r="G31" s="138"/>
       <c r="H31" s="138"/>
       <c r="J31" t="s">
-        <v>276</v>
-      </c>
-    </row>
-    <row r="32" spans="2:30" x14ac:dyDescent="0.3">
+        <v>272</v>
+      </c>
+    </row>
+    <row r="32" spans="2:30">
       <c r="B32" s="137" t="s">
         <v>248</v>
       </c>
@@ -5916,127 +6127,148 @@
         <v>3.5</v>
       </c>
       <c r="J32" t="s">
-        <v>273</v>
-      </c>
-    </row>
-    <row r="33" spans="2:10" x14ac:dyDescent="0.3">
+        <v>269</v>
+      </c>
+    </row>
+    <row r="33" spans="2:10">
       <c r="B33" s="141" t="s">
         <v>249</v>
       </c>
       <c r="C33" s="144" t="s">
-        <v>268</v>
+        <v>275</v>
       </c>
       <c r="D33" s="144" t="s">
-        <v>269</v>
+        <v>278</v>
       </c>
       <c r="F33" s="137" t="s">
         <v>249</v>
       </c>
       <c r="G33" s="144" t="s">
-        <v>270</v>
+        <v>277</v>
       </c>
       <c r="H33" s="144" t="s">
-        <v>271</v>
+        <v>279</v>
       </c>
       <c r="J33" t="s">
-        <v>278</v>
-      </c>
-    </row>
-    <row r="34" spans="2:10" x14ac:dyDescent="0.3">
+        <v>274</v>
+      </c>
+    </row>
+    <row r="34" spans="2:10">
       <c r="B34" s="137" t="s">
         <v>226</v>
       </c>
       <c r="C34" s="144">
-        <v>4.7</v>
+        <v>5.04</v>
       </c>
       <c r="D34" s="144">
-        <v>4.97</v>
+        <v>5.05</v>
       </c>
       <c r="F34" s="137" t="s">
         <v>226</v>
       </c>
       <c r="G34" s="144">
-        <v>5.05</v>
+        <v>4.97</v>
       </c>
       <c r="H34" s="144">
-        <v>5.03</v>
+        <v>4.9800000000000004</v>
       </c>
       <c r="J34" t="s">
-        <v>277</v>
-      </c>
-    </row>
-    <row r="35" spans="2:10" x14ac:dyDescent="0.3">
+        <v>273</v>
+      </c>
+    </row>
+    <row r="35" spans="2:10">
       <c r="B35" s="141" t="s">
         <v>266</v>
       </c>
       <c r="C35" s="145">
         <f>(C37/C36)</f>
-        <v>0.60606060606060608</v>
+        <v>0.68319999999999992</v>
       </c>
       <c r="D35" s="145">
         <f>D37/D36</f>
-        <v>0.82258064516129026</v>
+        <v>0.78988326848249024</v>
       </c>
       <c r="F35" s="141" t="s">
         <v>266</v>
       </c>
       <c r="G35" s="145">
         <f>G37/G36</f>
-        <v>0.91228070175438603</v>
+        <v>0.86</v>
       </c>
       <c r="H35" s="145">
         <f>H37/H36</f>
-        <v>0.9107142857142857</v>
-      </c>
-    </row>
-    <row r="36" spans="2:10" x14ac:dyDescent="0.3">
+        <v>0.86</v>
+      </c>
+    </row>
+    <row r="36" spans="2:10">
       <c r="B36" s="141" t="s">
         <v>267</v>
       </c>
       <c r="C36" s="144">
-        <v>7.26</v>
+        <v>6.25</v>
       </c>
       <c r="D36" s="144">
-        <v>6.2</v>
+        <v>5.14</v>
       </c>
       <c r="F36" s="141" t="s">
         <v>267</v>
       </c>
       <c r="G36" s="144">
-        <v>0.56999999999999995</v>
+        <v>0.5</v>
       </c>
       <c r="H36" s="144">
-        <v>0.56000000000000005</v>
+        <v>0.5</v>
       </c>
       <c r="J36" t="s">
-        <v>274</v>
-      </c>
-    </row>
-    <row r="37" spans="2:10" x14ac:dyDescent="0.3">
+        <v>270</v>
+      </c>
+    </row>
+    <row r="37" spans="2:10">
       <c r="B37" s="141" t="s">
         <v>15</v>
       </c>
       <c r="C37" s="144">
-        <v>4.4000000000000004</v>
+        <v>4.2699999999999996</v>
       </c>
       <c r="D37" s="144">
-        <v>5.0999999999999996</v>
+        <v>4.0599999999999996</v>
       </c>
       <c r="F37" s="141" t="s">
         <v>15</v>
       </c>
       <c r="G37" s="144">
-        <v>0.52</v>
+        <v>0.43</v>
       </c>
       <c r="H37" s="144">
-        <v>0.51</v>
+        <v>0.43</v>
       </c>
       <c r="J37" t="s">
-        <v>275</v>
+        <v>271</v>
+      </c>
+    </row>
+    <row r="38" spans="2:10">
+      <c r="B38" s="141" t="s">
+        <v>276</v>
+      </c>
+      <c r="C38" s="146">
+        <v>3.9</v>
+      </c>
+      <c r="D38" s="146">
+        <v>4.04</v>
+      </c>
+      <c r="F38" s="141" t="s">
+        <v>276</v>
+      </c>
+      <c r="G38" s="146">
+        <v>2.88</v>
+      </c>
+      <c r="H38" s="146">
+        <v>2.56</v>
       </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <drawing r:id="rId1"/>
 </worksheet>
 </file>
 

</xml_diff>

<commit_message>
MATLAB files for progress review 3 and small explanation for OVP speed on excel changed
</commit_message>
<xml_diff>
--- a/Excel/Boost Converter Design Params.xlsx
+++ b/Excel/Boost Converter Design Params.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\tytom\Documents\GitHub\311\Excel\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DF8CF42E-603F-4387-89D5-19831B881509}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C64696F2-8FF6-4030-B3D5-6DFF6CFBDF88}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="2" xr2:uid="{0EA872C3-4804-43CB-9F0B-5F94DB7B4351}"/>
   </bookViews>
@@ -18,6 +18,7 @@
     <sheet name="Testing_Openloop" sheetId="4" r:id="rId3"/>
   </sheets>
   <calcPr calcId="191029"/>
+  <fileRecoveryPr repairLoad="1"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
@@ -36,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="580" uniqueCount="281">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="585" uniqueCount="286">
   <si>
     <t>Parameter</t>
   </si>
@@ -879,6 +880,21 @@
   </si>
   <si>
     <t>Output Voltages as displayed on Oscilloscope - (At boundary conditions - 2.5/3.5V, 5/50ohm)</t>
+  </si>
+  <si>
+    <t>Over Voltage Protection (OVP)</t>
+  </si>
+  <si>
+    <t>From putting a 7v signal through the 5v pin on the pcb, then measuring Vout and capturing the time it takes</t>
+  </si>
+  <si>
+    <t>to go high  (set to 6V)</t>
+  </si>
+  <si>
+    <t>Speed: 286.4ns</t>
+  </si>
+  <si>
+    <t>OverVoltage threshold is 6.1, will lower in future</t>
   </si>
 </sst>
 </file>
@@ -893,7 +909,7 @@
     <numFmt numFmtId="168" formatCode="0.0000000"/>
     <numFmt numFmtId="169" formatCode="0.0000"/>
   </numFmts>
-  <fonts count="11">
+  <fonts count="12">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -977,8 +993,15 @@
       <family val="2"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF9C5700"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
-  <fills count="14">
+  <fills count="15">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -1054,6 +1077,11 @@
         <bgColor indexed="65"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFEB9C"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="68">
     <border>
@@ -2001,7 +2029,7 @@
       <diagonal/>
     </border>
   </borders>
-  <cellStyleXfs count="11">
+  <cellStyleXfs count="12">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="1" applyNumberFormat="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="1" fillId="3" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
@@ -2013,8 +2041,9 @@
     <xf numFmtId="0" fontId="1" fillId="11" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="1" fillId="12" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="1" fillId="13" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="11" fillId="14" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="147">
+  <cellXfs count="149">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
@@ -2178,8 +2207,10 @@
     <xf numFmtId="0" fontId="0" fillId="8" borderId="66" xfId="5" applyFont="1"/>
     <xf numFmtId="9" fontId="0" fillId="8" borderId="66" xfId="5" applyNumberFormat="1" applyFont="1"/>
     <xf numFmtId="0" fontId="0" fillId="8" borderId="67" xfId="5" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="11" fillId="14" borderId="0" xfId="11" applyBorder="1"/>
+    <xf numFmtId="0" fontId="11" fillId="14" borderId="0" xfId="11"/>
   </cellXfs>
-  <cellStyles count="11">
+  <cellStyles count="12">
     <cellStyle name="20% - Accent1" xfId="2" builtinId="30"/>
     <cellStyle name="20% - Accent6" xfId="10" builtinId="50"/>
     <cellStyle name="40% - Accent1" xfId="6" builtinId="31"/>
@@ -2188,6 +2219,7 @@
     <cellStyle name="60% - Accent2" xfId="8" builtinId="36"/>
     <cellStyle name="Calculation" xfId="4" builtinId="22"/>
     <cellStyle name="Check Cell" xfId="1" builtinId="23"/>
+    <cellStyle name="Neutral" xfId="11" builtinId="28"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
     <cellStyle name="Note" xfId="5" builtinId="10"/>
     <cellStyle name="Percent" xfId="3" builtinId="5"/>
@@ -5393,7 +5425,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{86BA37C4-8F32-417F-A8E4-D80C296F90D3}">
-  <dimension ref="B2:AD38"/>
+  <dimension ref="B2:AD47"/>
   <sheetFormatPr defaultRowHeight="14.4"/>
   <sheetData>
     <row r="2" spans="2:25">
@@ -5809,6 +5841,7 @@
       <c r="D22" s="138"/>
       <c r="E22" s="138"/>
       <c r="F22" s="138"/>
+      <c r="G22" s="138"/>
     </row>
     <row r="24" spans="2:30">
       <c r="B24" s="138" t="s">
@@ -6130,7 +6163,7 @@
         <v>269</v>
       </c>
     </row>
-    <row r="33" spans="2:10">
+    <row r="33" spans="2:13">
       <c r="B33" s="141" t="s">
         <v>249</v>
       </c>
@@ -6153,7 +6186,7 @@
         <v>274</v>
       </c>
     </row>
-    <row r="34" spans="2:10">
+    <row r="34" spans="2:13">
       <c r="B34" s="137" t="s">
         <v>226</v>
       </c>
@@ -6176,7 +6209,7 @@
         <v>273</v>
       </c>
     </row>
-    <row r="35" spans="2:10">
+    <row r="35" spans="2:13">
       <c r="B35" s="141" t="s">
         <v>266</v>
       </c>
@@ -6200,7 +6233,7 @@
         <v>0.86</v>
       </c>
     </row>
-    <row r="36" spans="2:10">
+    <row r="36" spans="2:13">
       <c r="B36" s="141" t="s">
         <v>267</v>
       </c>
@@ -6223,7 +6256,7 @@
         <v>270</v>
       </c>
     </row>
-    <row r="37" spans="2:10">
+    <row r="37" spans="2:13">
       <c r="B37" s="141" t="s">
         <v>15</v>
       </c>
@@ -6246,7 +6279,7 @@
         <v>271</v>
       </c>
     </row>
-    <row r="38" spans="2:10">
+    <row r="38" spans="2:13">
       <c r="B38" s="141" t="s">
         <v>276</v>
       </c>
@@ -6266,9 +6299,107 @@
         <v>2.56</v>
       </c>
     </row>
+    <row r="40" spans="2:13">
+      <c r="B40" s="141" t="s">
+        <v>281</v>
+      </c>
+    </row>
+    <row r="42" spans="2:13">
+      <c r="B42" s="147" t="s">
+        <v>284</v>
+      </c>
+      <c r="C42" s="148"/>
+      <c r="D42" s="148"/>
+      <c r="E42" s="148"/>
+      <c r="F42" s="148"/>
+      <c r="G42" s="148"/>
+      <c r="H42" s="148"/>
+      <c r="I42" s="148"/>
+      <c r="J42" s="148"/>
+      <c r="K42" s="148"/>
+      <c r="L42" s="148"/>
+      <c r="M42" s="148"/>
+    </row>
+    <row r="43" spans="2:13">
+      <c r="B43" s="148" t="s">
+        <v>282</v>
+      </c>
+      <c r="C43" s="148"/>
+      <c r="D43" s="148"/>
+      <c r="E43" s="148"/>
+      <c r="F43" s="148"/>
+      <c r="G43" s="148"/>
+      <c r="H43" s="148"/>
+      <c r="I43" s="148"/>
+      <c r="J43" s="148"/>
+      <c r="K43" s="148"/>
+      <c r="L43" s="148"/>
+      <c r="M43" s="148"/>
+    </row>
+    <row r="44" spans="2:13">
+      <c r="B44" s="147" t="s">
+        <v>283</v>
+      </c>
+      <c r="C44" s="148"/>
+      <c r="D44" s="148"/>
+      <c r="E44" s="148"/>
+      <c r="F44" s="148"/>
+      <c r="G44" s="148"/>
+      <c r="H44" s="148"/>
+      <c r="I44" s="148"/>
+      <c r="J44" s="148"/>
+      <c r="K44" s="148"/>
+      <c r="L44" s="148"/>
+      <c r="M44" s="148"/>
+    </row>
+    <row r="45" spans="2:13">
+      <c r="B45" s="148"/>
+      <c r="C45" s="148"/>
+      <c r="D45" s="148"/>
+      <c r="E45" s="148"/>
+      <c r="F45" s="148"/>
+      <c r="G45" s="148"/>
+      <c r="H45" s="148"/>
+      <c r="I45" s="148"/>
+      <c r="J45" s="148"/>
+      <c r="K45" s="148"/>
+      <c r="L45" s="148"/>
+      <c r="M45" s="148"/>
+    </row>
+    <row r="46" spans="2:13">
+      <c r="B46" s="147" t="s">
+        <v>285</v>
+      </c>
+      <c r="C46" s="148"/>
+      <c r="D46" s="148"/>
+      <c r="E46" s="148"/>
+      <c r="F46" s="148"/>
+      <c r="G46" s="148"/>
+      <c r="H46" s="148"/>
+      <c r="I46" s="148"/>
+      <c r="J46" s="148"/>
+      <c r="K46" s="148"/>
+      <c r="L46" s="148"/>
+      <c r="M46" s="148"/>
+    </row>
+    <row r="47" spans="2:13">
+      <c r="B47" s="148"/>
+      <c r="C47" s="148"/>
+      <c r="D47" s="148"/>
+      <c r="E47" s="148"/>
+      <c r="F47" s="148"/>
+      <c r="G47" s="148"/>
+      <c r="H47" s="148"/>
+      <c r="I47" s="148"/>
+      <c r="J47" s="148"/>
+      <c r="K47" s="148"/>
+      <c r="L47" s="148"/>
+      <c r="M47" s="148"/>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <drawing r:id="rId1"/>
+  <pageSetup orientation="portrait" r:id="rId1"/>
+  <drawing r:id="rId2"/>
 </worksheet>
 </file>
 

</xml_diff>

<commit_message>
Current sense testing completed, ran on MATLAB, and displayed on excel
</commit_message>
<xml_diff>
--- a/Excel/Boost Converter Design Params.xlsx
+++ b/Excel/Boost Converter Design Params.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\tytom\Documents\GitHub\311\Excel\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C64696F2-8FF6-4030-B3D5-6DFF6CFBDF88}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{390D13BA-2610-43F0-8D19-D74055A957CF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="2" xr2:uid="{0EA872C3-4804-43CB-9F0B-5F94DB7B4351}"/>
   </bookViews>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="585" uniqueCount="286">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="624" uniqueCount="313">
   <si>
     <t>Parameter</t>
   </si>
@@ -882,19 +882,100 @@
     <t>Output Voltages as displayed on Oscilloscope - (At boundary conditions - 2.5/3.5V, 5/50ohm)</t>
   </si>
   <si>
-    <t>Over Voltage Protection (OVP)</t>
-  </si>
-  <si>
-    <t>From putting a 7v signal through the 5v pin on the pcb, then measuring Vout and capturing the time it takes</t>
-  </si>
-  <si>
-    <t>to go high  (set to 6V)</t>
-  </si>
-  <si>
     <t>Speed: 286.4ns</t>
   </si>
   <si>
-    <t>OverVoltage threshold is 6.1, will lower in future</t>
+    <t>Over Voltage Protection (OVP) testing</t>
+  </si>
+  <si>
+    <t>Current feedback testing - (IFB is input, IFBF is output)</t>
+  </si>
+  <si>
+    <t>IFB(mean) (mV)</t>
+  </si>
+  <si>
+    <t>IFB(peak) (mV)</t>
+  </si>
+  <si>
+    <t>IFBF(mean) (mV)</t>
+  </si>
+  <si>
+    <t>IFBF(peak) (mV)</t>
+  </si>
+  <si>
+    <t>Voltage divider check:</t>
+  </si>
+  <si>
+    <t>Duty cycle</t>
+  </si>
+  <si>
+    <t>VFB(mean) (V)</t>
+  </si>
+  <si>
+    <t>VFBF(mean) (V)</t>
+  </si>
+  <si>
+    <t>VFB(pk-pk amplitude) (V)</t>
+  </si>
+  <si>
+    <t>VFBF(pk-pk amplitude) (V)</t>
+  </si>
+  <si>
+    <t>Filename (output/IFBF)</t>
+  </si>
+  <si>
+    <t>Filename (input/IFB)</t>
+  </si>
+  <si>
+    <t>5_25_O</t>
+  </si>
+  <si>
+    <t>5_25_I</t>
+  </si>
+  <si>
+    <t>C1</t>
+  </si>
+  <si>
+    <t>C2</t>
+  </si>
+  <si>
+    <t>50_25_I2</t>
+  </si>
+  <si>
+    <t>50_25_O</t>
+  </si>
+  <si>
+    <t>5_35_I</t>
+  </si>
+  <si>
+    <t>50_35_I</t>
+  </si>
+  <si>
+    <t>50_35_O</t>
+  </si>
+  <si>
+    <t>5_35_O</t>
+  </si>
+  <si>
+    <t>VDIV_I</t>
+  </si>
+  <si>
+    <t>VDIV_O</t>
+  </si>
+  <si>
+    <t>Current sense input &amp; output values as displayed on Oscilloscope</t>
+  </si>
+  <si>
+    <t>OverVoltage threshold is 6.1, which was found (+detailed in report) by incrementing in 0.1V intervals to the</t>
+  </si>
+  <si>
+    <t>input of the OVP comparator</t>
+  </si>
+  <si>
+    <t xml:space="preserve">From putting a 7v signal through the 5v pin on the pcb, then measuring Vout and capturing the time it takes on a rising </t>
+  </si>
+  <si>
+    <t>edge to go high  (set to 6V)</t>
   </si>
 </sst>
 </file>
@@ -1001,7 +1082,7 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="15">
+  <fills count="18">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -1082,6 +1163,24 @@
         <fgColor rgb="FFFFEB9C"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="8" tint="0.79998168889431442"/>
+        <bgColor indexed="65"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="8" tint="0.59999389629810485"/>
+        <bgColor indexed="65"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="8" tint="0.39997558519241921"/>
+        <bgColor indexed="65"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="68">
     <border>
@@ -2029,7 +2128,7 @@
       <diagonal/>
     </border>
   </borders>
-  <cellStyleXfs count="12">
+  <cellStyleXfs count="15">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="1" applyNumberFormat="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="1" fillId="3" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
@@ -2042,8 +2141,11 @@
     <xf numFmtId="0" fontId="1" fillId="12" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="1" fillId="13" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="11" fillId="14" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="1" fillId="15" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="1" fillId="16" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="1" fillId="17" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="149">
+  <cellXfs count="166">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
@@ -2205,18 +2307,46 @@
     <xf numFmtId="0" fontId="1" fillId="11" borderId="0" xfId="8" applyBorder="1"/>
     <xf numFmtId="0" fontId="10" fillId="7" borderId="65" xfId="4"/>
     <xf numFmtId="0" fontId="0" fillId="8" borderId="66" xfId="5" applyFont="1"/>
-    <xf numFmtId="9" fontId="0" fillId="8" borderId="66" xfId="5" applyNumberFormat="1" applyFont="1"/>
     <xf numFmtId="0" fontId="0" fillId="8" borderId="67" xfId="5" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="11" fillId="14" borderId="0" xfId="11" applyBorder="1"/>
     <xf numFmtId="0" fontId="11" fillId="14" borderId="0" xfId="11"/>
+    <xf numFmtId="0" fontId="1" fillId="17" borderId="0" xfId="14" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="17" borderId="0" xfId="14"/>
+    <xf numFmtId="0" fontId="1" fillId="16" borderId="0" xfId="13"/>
+    <xf numFmtId="0" fontId="1" fillId="16" borderId="0" xfId="13" applyBorder="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="1" fillId="15" borderId="66" xfId="12" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="15" borderId="66" xfId="12" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="15" borderId="66" xfId="12" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="15" borderId="66" xfId="12" applyNumberFormat="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="16" borderId="0" xfId="13" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="15" borderId="66" xfId="12" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="9" fillId="16" borderId="0" xfId="13" applyFont="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="16" borderId="0" xfId="13" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="15" borderId="0" xfId="12"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="10" borderId="0" xfId="7" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="9" fillId="8" borderId="66" xfId="5" applyFont="1"/>
+    <xf numFmtId="0" fontId="9" fillId="10" borderId="0" xfId="7" applyFont="1"/>
+    <xf numFmtId="9" fontId="9" fillId="8" borderId="66" xfId="5" applyNumberFormat="1" applyFont="1"/>
   </cellXfs>
-  <cellStyles count="12">
+  <cellStyles count="15">
     <cellStyle name="20% - Accent1" xfId="2" builtinId="30"/>
+    <cellStyle name="20% - Accent5" xfId="12" builtinId="46"/>
     <cellStyle name="20% - Accent6" xfId="10" builtinId="50"/>
     <cellStyle name="40% - Accent1" xfId="6" builtinId="31"/>
     <cellStyle name="40% - Accent2" xfId="7" builtinId="35"/>
     <cellStyle name="40% - Accent4" xfId="9" builtinId="43"/>
+    <cellStyle name="40% - Accent5" xfId="13" builtinId="47"/>
     <cellStyle name="60% - Accent2" xfId="8" builtinId="36"/>
+    <cellStyle name="60% - Accent5" xfId="14" builtinId="48"/>
     <cellStyle name="Calculation" xfId="4" builtinId="22"/>
     <cellStyle name="Check Cell" xfId="1" builtinId="23"/>
     <cellStyle name="Neutral" xfId="11" builtinId="28"/>
@@ -2291,15 +2421,15 @@
   <xdr:twoCellAnchor editAs="oneCell">
     <xdr:from>
       <xdr:col>15</xdr:col>
-      <xdr:colOff>0</xdr:colOff>
+      <xdr:colOff>13857</xdr:colOff>
       <xdr:row>30</xdr:row>
-      <xdr:rowOff>1</xdr:rowOff>
+      <xdr:rowOff>2</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>26</xdr:col>
-      <xdr:colOff>138545</xdr:colOff>
-      <xdr:row>51</xdr:row>
-      <xdr:rowOff>101120</xdr:rowOff>
+      <xdr:col>21</xdr:col>
+      <xdr:colOff>346364</xdr:colOff>
+      <xdr:row>42</xdr:row>
+      <xdr:rowOff>102704</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -2322,8 +2452,8 @@
       </xdr:blipFill>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="9144000" y="5403274"/>
-          <a:ext cx="6844145" cy="3883410"/>
+          <a:off x="9157857" y="5403275"/>
+          <a:ext cx="3990107" cy="2264011"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -2334,16 +2464,16 @@
   </xdr:twoCellAnchor>
   <xdr:twoCellAnchor editAs="oneCell">
     <xdr:from>
-      <xdr:col>27</xdr:col>
-      <xdr:colOff>13856</xdr:colOff>
-      <xdr:row>30</xdr:row>
-      <xdr:rowOff>1</xdr:rowOff>
+      <xdr:col>21</xdr:col>
+      <xdr:colOff>554184</xdr:colOff>
+      <xdr:row>29</xdr:row>
+      <xdr:rowOff>166256</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>38</xdr:col>
-      <xdr:colOff>152400</xdr:colOff>
-      <xdr:row>51</xdr:row>
-      <xdr:rowOff>101145</xdr:rowOff>
+      <xdr:col>28</xdr:col>
+      <xdr:colOff>341394</xdr:colOff>
+      <xdr:row>42</xdr:row>
+      <xdr:rowOff>125506</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -2366,8 +2496,8 @@
       </xdr:blipFill>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="16473056" y="5403274"/>
-          <a:ext cx="6844144" cy="3883435"/>
+          <a:off x="13355784" y="5365785"/>
+          <a:ext cx="4054410" cy="2290074"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -2378,16 +2508,16 @@
   </xdr:twoCellAnchor>
   <xdr:twoCellAnchor editAs="oneCell">
     <xdr:from>
-      <xdr:col>27</xdr:col>
-      <xdr:colOff>1</xdr:colOff>
-      <xdr:row>53</xdr:row>
-      <xdr:rowOff>1</xdr:rowOff>
+      <xdr:col>21</xdr:col>
+      <xdr:colOff>367555</xdr:colOff>
+      <xdr:row>42</xdr:row>
+      <xdr:rowOff>62754</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>38</xdr:col>
-      <xdr:colOff>180109</xdr:colOff>
-      <xdr:row>74</xdr:row>
-      <xdr:rowOff>123910</xdr:rowOff>
+      <xdr:col>28</xdr:col>
+      <xdr:colOff>332509</xdr:colOff>
+      <xdr:row>55</xdr:row>
+      <xdr:rowOff>103650</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -2410,8 +2540,8 @@
       </xdr:blipFill>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="16459201" y="9545783"/>
-          <a:ext cx="6885708" cy="3906200"/>
+          <a:off x="13169155" y="7627336"/>
+          <a:ext cx="4232154" cy="2401364"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -2423,15 +2553,15 @@
   <xdr:twoCellAnchor editAs="oneCell">
     <xdr:from>
       <xdr:col>14</xdr:col>
-      <xdr:colOff>554182</xdr:colOff>
-      <xdr:row>53</xdr:row>
-      <xdr:rowOff>-1</xdr:rowOff>
+      <xdr:colOff>428677</xdr:colOff>
+      <xdr:row>42</xdr:row>
+      <xdr:rowOff>161363</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>26</xdr:col>
-      <xdr:colOff>166255</xdr:colOff>
-      <xdr:row>74</xdr:row>
-      <xdr:rowOff>148285</xdr:rowOff>
+      <xdr:col>21</xdr:col>
+      <xdr:colOff>358588</xdr:colOff>
+      <xdr:row>55</xdr:row>
+      <xdr:rowOff>179603</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -2454,8 +2584,228 @@
       </xdr:blipFill>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="9088582" y="9545781"/>
-          <a:ext cx="6927273" cy="3930577"/>
+          <a:off x="8963077" y="7691716"/>
+          <a:ext cx="4197111" cy="2371097"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>15</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>59</xdr:row>
+      <xdr:rowOff>55433</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>21</xdr:col>
+      <xdr:colOff>461044</xdr:colOff>
+      <xdr:row>65</xdr:row>
+      <xdr:rowOff>322133</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="6" name="Picture 5">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{72AC9D6A-FF01-2638-2013-51024D0218FE}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId5"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="9144000" y="10681869"/>
+          <a:ext cx="4118644" cy="2261755"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>15</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>65</xdr:row>
+      <xdr:rowOff>415650</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>21</xdr:col>
+      <xdr:colOff>458551</xdr:colOff>
+      <xdr:row>72</xdr:row>
+      <xdr:rowOff>124704</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="7" name="Picture 6">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{C0279119-940B-3080-557F-91F9B7126003}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId6"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="9144000" y="13037141"/>
+          <a:ext cx="4116151" cy="2272145"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>22</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>59</xdr:row>
+      <xdr:rowOff>55433</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>28</xdr:col>
+      <xdr:colOff>422084</xdr:colOff>
+      <xdr:row>65</xdr:row>
+      <xdr:rowOff>346378</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="8" name="Picture 7">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{2F311C41-6F3D-F739-94B3-9028510B5699}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId7"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="13411200" y="10681869"/>
+          <a:ext cx="4079684" cy="2286000"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>22</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>65</xdr:row>
+      <xdr:rowOff>443358</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>28</xdr:col>
+      <xdr:colOff>443345</xdr:colOff>
+      <xdr:row>72</xdr:row>
+      <xdr:rowOff>178180</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="9" name="Picture 8">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{5AAE0149-09E0-4295-9A2E-053E48C567E2}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId8"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="13411200" y="13064849"/>
+          <a:ext cx="4100945" cy="2297913"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>29</xdr:col>
+      <xdr:colOff>41564</xdr:colOff>
+      <xdr:row>62</xdr:row>
+      <xdr:rowOff>249381</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>36</xdr:col>
+      <xdr:colOff>512619</xdr:colOff>
+      <xdr:row>66</xdr:row>
+      <xdr:rowOff>429636</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="10" name="Picture 9">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{8FF3397F-D6DE-5A90-7A9B-430A6D8DF197}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId9"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="17719964" y="11416145"/>
+          <a:ext cx="4738255" cy="2369273"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -5425,7 +5775,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{86BA37C4-8F32-417F-A8E4-D80C296F90D3}">
-  <dimension ref="B2:AD47"/>
+  <dimension ref="A2:AD68"/>
   <sheetFormatPr defaultRowHeight="14.4"/>
   <sheetData>
     <row r="2" spans="2:25">
@@ -6163,30 +6513,30 @@
         <v>269</v>
       </c>
     </row>
-    <row r="33" spans="2:13">
-      <c r="B33" s="141" t="s">
+    <row r="33" spans="2:14">
+      <c r="B33" s="162" t="s">
         <v>249</v>
       </c>
-      <c r="C33" s="144" t="s">
+      <c r="C33" s="163" t="s">
         <v>275</v>
       </c>
-      <c r="D33" s="144" t="s">
+      <c r="D33" s="163" t="s">
         <v>278</v>
       </c>
-      <c r="F33" s="137" t="s">
+      <c r="F33" s="164" t="s">
         <v>249</v>
       </c>
-      <c r="G33" s="144" t="s">
+      <c r="G33" s="163" t="s">
         <v>277</v>
       </c>
-      <c r="H33" s="144" t="s">
+      <c r="H33" s="163" t="s">
         <v>279</v>
       </c>
       <c r="J33" t="s">
         <v>274</v>
       </c>
     </row>
-    <row r="34" spans="2:13">
+    <row r="34" spans="2:14">
       <c r="B34" s="137" t="s">
         <v>226</v>
       </c>
@@ -6209,31 +6559,31 @@
         <v>273</v>
       </c>
     </row>
-    <row r="35" spans="2:13">
-      <c r="B35" s="141" t="s">
+    <row r="35" spans="2:14">
+      <c r="B35" s="162" t="s">
         <v>266</v>
       </c>
-      <c r="C35" s="145">
+      <c r="C35" s="165">
         <f>(C37/C36)</f>
         <v>0.68319999999999992</v>
       </c>
-      <c r="D35" s="145">
+      <c r="D35" s="165">
         <f>D37/D36</f>
         <v>0.78988326848249024</v>
       </c>
-      <c r="F35" s="141" t="s">
+      <c r="F35" s="162" t="s">
         <v>266</v>
       </c>
-      <c r="G35" s="145">
+      <c r="G35" s="165">
         <f>G37/G36</f>
         <v>0.86</v>
       </c>
-      <c r="H35" s="145">
+      <c r="H35" s="165">
         <f>H37/H36</f>
         <v>0.86</v>
       </c>
     </row>
-    <row r="36" spans="2:13">
+    <row r="36" spans="2:14">
       <c r="B36" s="141" t="s">
         <v>267</v>
       </c>
@@ -6256,7 +6606,7 @@
         <v>270</v>
       </c>
     </row>
-    <row r="37" spans="2:13">
+    <row r="37" spans="2:14">
       <c r="B37" s="141" t="s">
         <v>15</v>
       </c>
@@ -6279,122 +6629,385 @@
         <v>271</v>
       </c>
     </row>
-    <row r="38" spans="2:13">
+    <row r="38" spans="2:14">
       <c r="B38" s="141" t="s">
         <v>276</v>
       </c>
-      <c r="C38" s="146">
+      <c r="C38" s="145">
         <v>3.9</v>
       </c>
-      <c r="D38" s="146">
+      <c r="D38" s="145">
         <v>4.04</v>
       </c>
       <c r="F38" s="141" t="s">
         <v>276</v>
       </c>
-      <c r="G38" s="146">
+      <c r="G38" s="145">
         <v>2.88</v>
       </c>
-      <c r="H38" s="146">
+      <c r="H38" s="145">
         <v>2.56</v>
       </c>
     </row>
-    <row r="40" spans="2:13">
-      <c r="B40" s="141" t="s">
+    <row r="45" spans="2:14">
+      <c r="B45" s="146" t="s">
+        <v>282</v>
+      </c>
+      <c r="C45" s="147"/>
+      <c r="D45" s="147"/>
+      <c r="E45" s="147"/>
+    </row>
+    <row r="47" spans="2:14">
+      <c r="B47" s="146" t="s">
         <v>281</v>
       </c>
-    </row>
-    <row r="42" spans="2:13">
-      <c r="B42" s="147" t="s">
+      <c r="C47" s="147"/>
+      <c r="D47" s="147"/>
+      <c r="E47" s="147"/>
+      <c r="F47" s="147"/>
+      <c r="G47" s="147"/>
+      <c r="H47" s="147"/>
+      <c r="I47" s="147"/>
+      <c r="J47" s="147"/>
+      <c r="K47" s="147"/>
+      <c r="L47" s="147"/>
+      <c r="M47" s="147"/>
+      <c r="N47" s="147"/>
+    </row>
+    <row r="48" spans="2:14">
+      <c r="B48" s="147" t="s">
+        <v>311</v>
+      </c>
+      <c r="C48" s="147"/>
+      <c r="D48" s="147"/>
+      <c r="E48" s="147"/>
+      <c r="F48" s="147"/>
+      <c r="G48" s="147"/>
+      <c r="H48" s="147"/>
+      <c r="I48" s="147"/>
+      <c r="J48" s="147"/>
+      <c r="K48" s="147"/>
+      <c r="L48" s="147"/>
+      <c r="M48" s="147"/>
+      <c r="N48" s="147"/>
+    </row>
+    <row r="49" spans="1:22">
+      <c r="B49" s="146" t="s">
+        <v>312</v>
+      </c>
+      <c r="C49" s="147"/>
+      <c r="D49" s="147"/>
+      <c r="E49" s="147"/>
+      <c r="F49" s="147"/>
+      <c r="G49" s="147"/>
+      <c r="H49" s="147"/>
+      <c r="I49" s="147"/>
+      <c r="J49" s="147"/>
+      <c r="K49" s="147"/>
+      <c r="L49" s="147"/>
+      <c r="M49" s="147"/>
+      <c r="N49" s="147"/>
+    </row>
+    <row r="50" spans="1:22">
+      <c r="B50" s="147"/>
+      <c r="C50" s="147"/>
+      <c r="D50" s="147"/>
+      <c r="E50" s="147"/>
+      <c r="F50" s="147"/>
+      <c r="G50" s="147"/>
+      <c r="H50" s="147"/>
+      <c r="I50" s="147"/>
+      <c r="J50" s="147"/>
+      <c r="K50" s="147"/>
+      <c r="L50" s="147"/>
+      <c r="M50" s="147"/>
+      <c r="N50" s="147"/>
+    </row>
+    <row r="51" spans="1:22">
+      <c r="B51" s="146" t="s">
+        <v>309</v>
+      </c>
+      <c r="C51" s="147"/>
+      <c r="D51" s="147"/>
+      <c r="E51" s="147"/>
+      <c r="F51" s="147"/>
+      <c r="G51" s="147"/>
+      <c r="H51" s="147"/>
+      <c r="I51" s="147"/>
+      <c r="J51" s="147"/>
+      <c r="K51" s="147"/>
+      <c r="L51" s="147"/>
+      <c r="M51" s="147"/>
+      <c r="N51" s="147"/>
+    </row>
+    <row r="52" spans="1:22">
+      <c r="B52" s="147" t="s">
+        <v>310</v>
+      </c>
+      <c r="C52" s="147"/>
+      <c r="D52" s="147"/>
+      <c r="E52" s="147"/>
+      <c r="F52" s="147"/>
+      <c r="G52" s="147"/>
+      <c r="H52" s="147"/>
+      <c r="I52" s="147"/>
+      <c r="J52" s="147"/>
+      <c r="K52" s="147"/>
+      <c r="L52" s="147"/>
+      <c r="M52" s="147"/>
+      <c r="N52" s="147"/>
+    </row>
+    <row r="54" spans="1:22">
+      <c r="A54" t="s">
+        <v>299</v>
+      </c>
+    </row>
+    <row r="56" spans="1:22">
+      <c r="A56" t="s">
+        <v>298</v>
+      </c>
+    </row>
+    <row r="58" spans="1:22">
+      <c r="B58" s="149" t="s">
+        <v>283</v>
+      </c>
+      <c r="C58" s="149"/>
+      <c r="D58" s="149"/>
+      <c r="E58" s="149"/>
+      <c r="F58" s="149"/>
+      <c r="J58" s="149" t="s">
+        <v>288</v>
+      </c>
+      <c r="K58" s="149"/>
+      <c r="P58" s="149" t="s">
+        <v>308</v>
+      </c>
+      <c r="Q58" s="149"/>
+      <c r="R58" s="149"/>
+      <c r="S58" s="149"/>
+      <c r="T58" s="149"/>
+      <c r="U58" s="149"/>
+      <c r="V58" s="149"/>
+    </row>
+    <row r="60" spans="1:22">
+      <c r="B60" s="148" t="s">
+        <v>261</v>
+      </c>
+      <c r="C60" s="149"/>
+      <c r="D60" s="149"/>
+      <c r="F60" s="148" t="s">
+        <v>265</v>
+      </c>
+      <c r="G60" s="149"/>
+      <c r="H60" s="149"/>
+      <c r="J60" s="149" t="s">
+        <v>261</v>
+      </c>
+      <c r="K60" s="149"/>
+    </row>
+    <row r="61" spans="1:22">
+      <c r="B61" s="150" t="s">
+        <v>248</v>
+      </c>
+      <c r="C61" s="143">
+        <v>2.5</v>
+      </c>
+      <c r="D61" s="143">
+        <v>3.5</v>
+      </c>
+      <c r="F61" s="150" t="s">
+        <v>248</v>
+      </c>
+      <c r="G61" s="143">
+        <v>2.5</v>
+      </c>
+      <c r="H61" s="143">
+        <v>3.5</v>
+      </c>
+      <c r="J61" s="150" t="s">
+        <v>248</v>
+      </c>
+      <c r="K61" s="160">
+        <v>2.5</v>
+      </c>
+    </row>
+    <row r="62" spans="1:22">
+      <c r="B62" s="151" t="s">
+        <v>249</v>
+      </c>
+      <c r="C62" s="152">
+        <v>0.5</v>
+      </c>
+      <c r="D62" s="152">
+        <v>0.3</v>
+      </c>
+      <c r="F62" s="151" t="s">
+        <v>249</v>
+      </c>
+      <c r="G62" s="152">
+        <v>0.5</v>
+      </c>
+      <c r="H62" s="152">
+        <v>0.3</v>
+      </c>
+      <c r="J62" s="150" t="s">
+        <v>289</v>
+      </c>
+      <c r="K62" s="160">
+        <v>0.5</v>
+      </c>
+    </row>
+    <row r="63" spans="1:22" ht="28.8">
+      <c r="B63" s="158" t="s">
         <v>284</v>
       </c>
-      <c r="C42" s="148"/>
-      <c r="D42" s="148"/>
-      <c r="E42" s="148"/>
-      <c r="F42" s="148"/>
-      <c r="G42" s="148"/>
-      <c r="H42" s="148"/>
-      <c r="I42" s="148"/>
-      <c r="J42" s="148"/>
-      <c r="K42" s="148"/>
-      <c r="L42" s="148"/>
-      <c r="M42" s="148"/>
-    </row>
-    <row r="43" spans="2:13">
-      <c r="B43" s="148" t="s">
-        <v>282</v>
-      </c>
-      <c r="C43" s="148"/>
-      <c r="D43" s="148"/>
-      <c r="E43" s="148"/>
-      <c r="F43" s="148"/>
-      <c r="G43" s="148"/>
-      <c r="H43" s="148"/>
-      <c r="I43" s="148"/>
-      <c r="J43" s="148"/>
-      <c r="K43" s="148"/>
-      <c r="L43" s="148"/>
-      <c r="M43" s="148"/>
-    </row>
-    <row r="44" spans="2:13">
-      <c r="B44" s="147" t="s">
-        <v>283</v>
-      </c>
-      <c r="C44" s="148"/>
-      <c r="D44" s="148"/>
-      <c r="E44" s="148"/>
-      <c r="F44" s="148"/>
-      <c r="G44" s="148"/>
-      <c r="H44" s="148"/>
-      <c r="I44" s="148"/>
-      <c r="J44" s="148"/>
-      <c r="K44" s="148"/>
-      <c r="L44" s="148"/>
-      <c r="M44" s="148"/>
-    </row>
-    <row r="45" spans="2:13">
-      <c r="B45" s="148"/>
-      <c r="C45" s="148"/>
-      <c r="D45" s="148"/>
-      <c r="E45" s="148"/>
-      <c r="F45" s="148"/>
-      <c r="G45" s="148"/>
-      <c r="H45" s="148"/>
-      <c r="I45" s="148"/>
-      <c r="J45" s="148"/>
-      <c r="K45" s="148"/>
-      <c r="L45" s="148"/>
-      <c r="M45" s="148"/>
-    </row>
-    <row r="46" spans="2:13">
-      <c r="B46" s="147" t="s">
+      <c r="C63" s="157">
+        <v>73</v>
+      </c>
+      <c r="D63" s="157">
+        <v>35.700000000000003</v>
+      </c>
+      <c r="F63" s="158" t="s">
+        <v>284</v>
+      </c>
+      <c r="G63" s="157">
+        <v>8.8000000000000007</v>
+      </c>
+      <c r="H63" s="157">
+        <v>3.9</v>
+      </c>
+      <c r="J63" s="158" t="s">
+        <v>290</v>
+      </c>
+      <c r="K63" s="157">
+        <v>1.85</v>
+      </c>
+    </row>
+    <row r="64" spans="1:22" ht="57.6">
+      <c r="B64" s="156" t="s">
         <v>285</v>
       </c>
-      <c r="C46" s="148"/>
-      <c r="D46" s="148"/>
-      <c r="E46" s="148"/>
-      <c r="F46" s="148"/>
-      <c r="G46" s="148"/>
-      <c r="H46" s="148"/>
-      <c r="I46" s="148"/>
-      <c r="J46" s="148"/>
-      <c r="K46" s="148"/>
-      <c r="L46" s="148"/>
-      <c r="M46" s="148"/>
-    </row>
-    <row r="47" spans="2:13">
-      <c r="B47" s="148"/>
-      <c r="C47" s="148"/>
-      <c r="D47" s="148"/>
-      <c r="E47" s="148"/>
-      <c r="F47" s="148"/>
-      <c r="G47" s="148"/>
-      <c r="H47" s="148"/>
-      <c r="I47" s="148"/>
-      <c r="J47" s="148"/>
-      <c r="K47" s="148"/>
-      <c r="L47" s="148"/>
-      <c r="M47" s="148"/>
+      <c r="C64" s="154">
+        <v>612</v>
+      </c>
+      <c r="D64" s="154">
+        <v>592.9</v>
+      </c>
+      <c r="F64" s="156" t="s">
+        <v>285</v>
+      </c>
+      <c r="G64" s="154">
+        <v>250</v>
+      </c>
+      <c r="H64" s="155">
+        <v>231.3</v>
+      </c>
+      <c r="J64" s="156" t="s">
+        <v>292</v>
+      </c>
+      <c r="K64" s="154">
+        <v>0.42</v>
+      </c>
+    </row>
+    <row r="65" spans="2:11" ht="28.8">
+      <c r="B65" s="159" t="s">
+        <v>286</v>
+      </c>
+      <c r="C65" s="157">
+        <v>277.89999999999998</v>
+      </c>
+      <c r="D65" s="157">
+        <v>131.4</v>
+      </c>
+      <c r="F65" s="159" t="s">
+        <v>286</v>
+      </c>
+      <c r="G65" s="157">
+        <v>39.6</v>
+      </c>
+      <c r="H65" s="157">
+        <v>19.8</v>
+      </c>
+      <c r="J65" s="159" t="s">
+        <v>291</v>
+      </c>
+      <c r="K65" s="157">
+        <v>3.66</v>
+      </c>
+    </row>
+    <row r="66" spans="2:11" ht="57.6">
+      <c r="B66" s="156" t="s">
+        <v>287</v>
+      </c>
+      <c r="C66" s="153">
+        <v>749.7</v>
+      </c>
+      <c r="D66" s="152">
+        <v>558.6</v>
+      </c>
+      <c r="F66" s="156" t="s">
+        <v>287</v>
+      </c>
+      <c r="G66" s="153">
+        <v>211.7</v>
+      </c>
+      <c r="H66" s="152">
+        <v>181.8</v>
+      </c>
+      <c r="J66" s="156" t="s">
+        <v>293</v>
+      </c>
+      <c r="K66" s="153">
+        <v>2.99</v>
+      </c>
+    </row>
+    <row r="67" spans="2:11" ht="43.2">
+      <c r="B67" s="161" t="s">
+        <v>295</v>
+      </c>
+      <c r="C67" s="161" t="s">
+        <v>297</v>
+      </c>
+      <c r="D67" s="161" t="s">
+        <v>302</v>
+      </c>
+      <c r="E67" s="161"/>
+      <c r="F67" s="161"/>
+      <c r="G67" s="161" t="s">
+        <v>300</v>
+      </c>
+      <c r="H67" s="161" t="s">
+        <v>303</v>
+      </c>
+      <c r="I67" s="161"/>
+      <c r="J67" s="161"/>
+      <c r="K67" s="161" t="s">
+        <v>306</v>
+      </c>
+    </row>
+    <row r="68" spans="2:11" ht="43.2">
+      <c r="B68" s="161" t="s">
+        <v>294</v>
+      </c>
+      <c r="C68" s="161" t="s">
+        <v>296</v>
+      </c>
+      <c r="D68" s="161" t="s">
+        <v>305</v>
+      </c>
+      <c r="E68" s="161"/>
+      <c r="F68" s="161"/>
+      <c r="G68" s="161" t="s">
+        <v>301</v>
+      </c>
+      <c r="H68" s="161" t="s">
+        <v>304</v>
+      </c>
+      <c r="I68" s="161"/>
+      <c r="J68" s="161"/>
+      <c r="K68" s="161" t="s">
+        <v>307</v>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
OVP Voltage graphs and values formatted onto excel sheet
</commit_message>
<xml_diff>
--- a/Excel/Boost Converter Design Params.xlsx
+++ b/Excel/Boost Converter Design Params.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\tytom\Documents\GitHub\311\Excel\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{390D13BA-2610-43F0-8D19-D74055A957CF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B3FEB86E-84E6-4867-A586-20C85CEDADEA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="2" xr2:uid="{0EA872C3-4804-43CB-9F0B-5F94DB7B4351}"/>
   </bookViews>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="624" uniqueCount="313">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="625" uniqueCount="314">
   <si>
     <t>Parameter</t>
   </si>
@@ -976,6 +976,9 @@
   </si>
   <si>
     <t>edge to go high  (set to 6V)</t>
+  </si>
+  <si>
+    <t>OVP testing results as displayed on Oscilloscope</t>
   </si>
 </sst>
 </file>
@@ -2560,8 +2563,8 @@
     <xdr:to>
       <xdr:col>21</xdr:col>
       <xdr:colOff>358588</xdr:colOff>
-      <xdr:row>55</xdr:row>
-      <xdr:rowOff>179603</xdr:rowOff>
+      <xdr:row>56</xdr:row>
+      <xdr:rowOff>6421</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -2736,8 +2739,8 @@
     <xdr:to>
       <xdr:col>28</xdr:col>
       <xdr:colOff>443345</xdr:colOff>
-      <xdr:row>72</xdr:row>
-      <xdr:rowOff>178180</xdr:rowOff>
+      <xdr:row>73</xdr:row>
+      <xdr:rowOff>4998</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -2806,6 +2809,138 @@
         <a:xfrm>
           <a:off x="17719964" y="11416145"/>
           <a:ext cx="4738255" cy="2369273"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>15</xdr:col>
+      <xdr:colOff>2</xdr:colOff>
+      <xdr:row>77</xdr:row>
+      <xdr:rowOff>167642</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>21</xdr:col>
+      <xdr:colOff>526473</xdr:colOff>
+      <xdr:row>91</xdr:row>
+      <xdr:rowOff>27584</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="15" name="Picture 14">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{0FE9A0F2-AC83-3E70-C6CB-52B04BEE39CA}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId10"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="9144002" y="16443962"/>
+          <a:ext cx="4184071" cy="2420262"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>15</xdr:col>
+      <xdr:colOff>13854</xdr:colOff>
+      <xdr:row>92</xdr:row>
+      <xdr:rowOff>38793</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>21</xdr:col>
+      <xdr:colOff>538119</xdr:colOff>
+      <xdr:row>105</xdr:row>
+      <xdr:rowOff>80357</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="16" name="Picture 15">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{3B5EAF27-7FAF-4190-A59B-190FC83C90E9}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId11"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="9157854" y="19058313"/>
+          <a:ext cx="4181865" cy="2419004"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>22</xdr:col>
+      <xdr:colOff>136238</xdr:colOff>
+      <xdr:row>85</xdr:row>
+      <xdr:rowOff>11611</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>28</xdr:col>
+      <xdr:colOff>522761</xdr:colOff>
+      <xdr:row>97</xdr:row>
+      <xdr:rowOff>66039</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="17" name="Picture 16">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{E1FD7901-490C-9F8C-EDB2-7F3626BACAB7}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId12"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="13547438" y="17750971"/>
+          <a:ext cx="4044123" cy="2248988"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -5775,7 +5910,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{86BA37C4-8F32-417F-A8E4-D80C296F90D3}">
-  <dimension ref="A2:AD68"/>
+  <dimension ref="A2:AD83"/>
   <sheetFormatPr defaultRowHeight="14.4"/>
   <sheetData>
     <row r="2" spans="2:25">
@@ -6513,7 +6648,7 @@
         <v>269</v>
       </c>
     </row>
-    <row r="33" spans="2:14">
+    <row r="33" spans="2:10">
       <c r="B33" s="162" t="s">
         <v>249</v>
       </c>
@@ -6536,7 +6671,7 @@
         <v>274</v>
       </c>
     </row>
-    <row r="34" spans="2:14">
+    <row r="34" spans="2:10">
       <c r="B34" s="137" t="s">
         <v>226</v>
       </c>
@@ -6559,7 +6694,7 @@
         <v>273</v>
       </c>
     </row>
-    <row r="35" spans="2:14">
+    <row r="35" spans="2:10">
       <c r="B35" s="162" t="s">
         <v>266</v>
       </c>
@@ -6583,7 +6718,7 @@
         <v>0.86</v>
       </c>
     </row>
-    <row r="36" spans="2:14">
+    <row r="36" spans="2:10">
       <c r="B36" s="141" t="s">
         <v>267</v>
       </c>
@@ -6606,7 +6741,7 @@
         <v>270</v>
       </c>
     </row>
-    <row r="37" spans="2:14">
+    <row r="37" spans="2:10">
       <c r="B37" s="141" t="s">
         <v>15</v>
       </c>
@@ -6629,7 +6764,7 @@
         <v>271</v>
       </c>
     </row>
-    <row r="38" spans="2:14">
+    <row r="38" spans="2:10">
       <c r="B38" s="141" t="s">
         <v>276</v>
       </c>
@@ -6648,114 +6783,6 @@
       <c r="H38" s="145">
         <v>2.56</v>
       </c>
-    </row>
-    <row r="45" spans="2:14">
-      <c r="B45" s="146" t="s">
-        <v>282</v>
-      </c>
-      <c r="C45" s="147"/>
-      <c r="D45" s="147"/>
-      <c r="E45" s="147"/>
-    </row>
-    <row r="47" spans="2:14">
-      <c r="B47" s="146" t="s">
-        <v>281</v>
-      </c>
-      <c r="C47" s="147"/>
-      <c r="D47" s="147"/>
-      <c r="E47" s="147"/>
-      <c r="F47" s="147"/>
-      <c r="G47" s="147"/>
-      <c r="H47" s="147"/>
-      <c r="I47" s="147"/>
-      <c r="J47" s="147"/>
-      <c r="K47" s="147"/>
-      <c r="L47" s="147"/>
-      <c r="M47" s="147"/>
-      <c r="N47" s="147"/>
-    </row>
-    <row r="48" spans="2:14">
-      <c r="B48" s="147" t="s">
-        <v>311</v>
-      </c>
-      <c r="C48" s="147"/>
-      <c r="D48" s="147"/>
-      <c r="E48" s="147"/>
-      <c r="F48" s="147"/>
-      <c r="G48" s="147"/>
-      <c r="H48" s="147"/>
-      <c r="I48" s="147"/>
-      <c r="J48" s="147"/>
-      <c r="K48" s="147"/>
-      <c r="L48" s="147"/>
-      <c r="M48" s="147"/>
-      <c r="N48" s="147"/>
-    </row>
-    <row r="49" spans="1:22">
-      <c r="B49" s="146" t="s">
-        <v>312</v>
-      </c>
-      <c r="C49" s="147"/>
-      <c r="D49" s="147"/>
-      <c r="E49" s="147"/>
-      <c r="F49" s="147"/>
-      <c r="G49" s="147"/>
-      <c r="H49" s="147"/>
-      <c r="I49" s="147"/>
-      <c r="J49" s="147"/>
-      <c r="K49" s="147"/>
-      <c r="L49" s="147"/>
-      <c r="M49" s="147"/>
-      <c r="N49" s="147"/>
-    </row>
-    <row r="50" spans="1:22">
-      <c r="B50" s="147"/>
-      <c r="C50" s="147"/>
-      <c r="D50" s="147"/>
-      <c r="E50" s="147"/>
-      <c r="F50" s="147"/>
-      <c r="G50" s="147"/>
-      <c r="H50" s="147"/>
-      <c r="I50" s="147"/>
-      <c r="J50" s="147"/>
-      <c r="K50" s="147"/>
-      <c r="L50" s="147"/>
-      <c r="M50" s="147"/>
-      <c r="N50" s="147"/>
-    </row>
-    <row r="51" spans="1:22">
-      <c r="B51" s="146" t="s">
-        <v>309</v>
-      </c>
-      <c r="C51" s="147"/>
-      <c r="D51" s="147"/>
-      <c r="E51" s="147"/>
-      <c r="F51" s="147"/>
-      <c r="G51" s="147"/>
-      <c r="H51" s="147"/>
-      <c r="I51" s="147"/>
-      <c r="J51" s="147"/>
-      <c r="K51" s="147"/>
-      <c r="L51" s="147"/>
-      <c r="M51" s="147"/>
-      <c r="N51" s="147"/>
-    </row>
-    <row r="52" spans="1:22">
-      <c r="B52" s="147" t="s">
-        <v>310</v>
-      </c>
-      <c r="C52" s="147"/>
-      <c r="D52" s="147"/>
-      <c r="E52" s="147"/>
-      <c r="F52" s="147"/>
-      <c r="G52" s="147"/>
-      <c r="H52" s="147"/>
-      <c r="I52" s="147"/>
-      <c r="J52" s="147"/>
-      <c r="K52" s="147"/>
-      <c r="L52" s="147"/>
-      <c r="M52" s="147"/>
-      <c r="N52" s="147"/>
     </row>
     <row r="54" spans="1:22">
       <c r="A54" t="s">
@@ -6909,7 +6936,7 @@
         <v>0.42</v>
       </c>
     </row>
-    <row r="65" spans="2:11" ht="28.8">
+    <row r="65" spans="2:20" ht="28.8">
       <c r="B65" s="159" t="s">
         <v>286</v>
       </c>
@@ -6935,7 +6962,7 @@
         <v>3.66</v>
       </c>
     </row>
-    <row r="66" spans="2:11" ht="57.6">
+    <row r="66" spans="2:20" ht="57.6">
       <c r="B66" s="156" t="s">
         <v>287</v>
       </c>
@@ -6961,7 +6988,7 @@
         <v>2.99</v>
       </c>
     </row>
-    <row r="67" spans="2:11" ht="43.2">
+    <row r="67" spans="2:20" ht="43.2">
       <c r="B67" s="161" t="s">
         <v>295</v>
       </c>
@@ -6985,7 +7012,7 @@
         <v>306</v>
       </c>
     </row>
-    <row r="68" spans="2:11" ht="43.2">
+    <row r="68" spans="2:20" ht="43.2">
       <c r="B68" s="161" t="s">
         <v>294</v>
       </c>
@@ -7008,6 +7035,121 @@
       <c r="K68" s="161" t="s">
         <v>307</v>
       </c>
+    </row>
+    <row r="76" spans="2:20">
+      <c r="B76" s="146" t="s">
+        <v>282</v>
+      </c>
+      <c r="C76" s="147"/>
+      <c r="D76" s="147"/>
+      <c r="E76" s="147"/>
+      <c r="P76" s="147" t="s">
+        <v>313</v>
+      </c>
+      <c r="Q76" s="147"/>
+      <c r="R76" s="147"/>
+      <c r="S76" s="147"/>
+      <c r="T76" s="147"/>
+    </row>
+    <row r="78" spans="2:20">
+      <c r="B78" s="146" t="s">
+        <v>281</v>
+      </c>
+      <c r="C78" s="147"/>
+      <c r="D78" s="147"/>
+      <c r="E78" s="147"/>
+      <c r="F78" s="147"/>
+      <c r="G78" s="147"/>
+      <c r="H78" s="147"/>
+      <c r="I78" s="147"/>
+      <c r="J78" s="147"/>
+      <c r="K78" s="147"/>
+      <c r="L78" s="147"/>
+      <c r="M78" s="147"/>
+      <c r="N78" s="147"/>
+    </row>
+    <row r="79" spans="2:20">
+      <c r="B79" s="147" t="s">
+        <v>311</v>
+      </c>
+      <c r="C79" s="147"/>
+      <c r="D79" s="147"/>
+      <c r="E79" s="147"/>
+      <c r="F79" s="147"/>
+      <c r="G79" s="147"/>
+      <c r="H79" s="147"/>
+      <c r="I79" s="147"/>
+      <c r="J79" s="147"/>
+      <c r="K79" s="147"/>
+      <c r="L79" s="147"/>
+      <c r="M79" s="147"/>
+      <c r="N79" s="147"/>
+    </row>
+    <row r="80" spans="2:20">
+      <c r="B80" s="146" t="s">
+        <v>312</v>
+      </c>
+      <c r="C80" s="147"/>
+      <c r="D80" s="147"/>
+      <c r="E80" s="147"/>
+      <c r="F80" s="147"/>
+      <c r="G80" s="147"/>
+      <c r="H80" s="147"/>
+      <c r="I80" s="147"/>
+      <c r="J80" s="147"/>
+      <c r="K80" s="147"/>
+      <c r="L80" s="147"/>
+      <c r="M80" s="147"/>
+      <c r="N80" s="147"/>
+    </row>
+    <row r="81" spans="2:14">
+      <c r="B81" s="147"/>
+      <c r="C81" s="147"/>
+      <c r="D81" s="147"/>
+      <c r="E81" s="147"/>
+      <c r="F81" s="147"/>
+      <c r="G81" s="147"/>
+      <c r="H81" s="147"/>
+      <c r="I81" s="147"/>
+      <c r="J81" s="147"/>
+      <c r="K81" s="147"/>
+      <c r="L81" s="147"/>
+      <c r="M81" s="147"/>
+      <c r="N81" s="147"/>
+    </row>
+    <row r="82" spans="2:14">
+      <c r="B82" s="146" t="s">
+        <v>309</v>
+      </c>
+      <c r="C82" s="147"/>
+      <c r="D82" s="147"/>
+      <c r="E82" s="147"/>
+      <c r="F82" s="147"/>
+      <c r="G82" s="147"/>
+      <c r="H82" s="147"/>
+      <c r="I82" s="147"/>
+      <c r="J82" s="147"/>
+      <c r="K82" s="147"/>
+      <c r="L82" s="147"/>
+      <c r="M82" s="147"/>
+      <c r="N82" s="147"/>
+    </row>
+    <row r="83" spans="2:14">
+      <c r="B83" s="147" t="s">
+        <v>310</v>
+      </c>
+      <c r="C83" s="147"/>
+      <c r="D83" s="147"/>
+      <c r="E83" s="147"/>
+      <c r="F83" s="147"/>
+      <c r="G83" s="147"/>
+      <c r="H83" s="147"/>
+      <c r="I83" s="147"/>
+      <c r="J83" s="147"/>
+      <c r="K83" s="147"/>
+      <c r="L83" s="147"/>
+      <c r="M83" s="147"/>
+      <c r="N83" s="147"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
MCU_VFB added to testing loop
</commit_message>
<xml_diff>
--- a/Excel/Boost Converter Design Params.xlsx
+++ b/Excel/Boost Converter Design Params.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\tytom\Documents\GitHub\311\Excel\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B3FEB86E-84E6-4867-A586-20C85CEDADEA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4A94C463-2E29-47D2-95EE-DD776DA90086}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="2" xr2:uid="{0EA872C3-4804-43CB-9F0B-5F94DB7B4351}"/>
   </bookViews>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="625" uniqueCount="314">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="631" uniqueCount="315">
   <si>
     <t>Parameter</t>
   </si>
@@ -979,6 +979,9 @@
   </si>
   <si>
     <t>OVP testing results as displayed on Oscilloscope</t>
+  </si>
+  <si>
+    <t>MCU_VFB</t>
   </si>
 </sst>
 </file>
@@ -2425,13 +2428,13 @@
     <xdr:from>
       <xdr:col>15</xdr:col>
       <xdr:colOff>13857</xdr:colOff>
-      <xdr:row>30</xdr:row>
+      <xdr:row>31</xdr:row>
       <xdr:rowOff>2</xdr:rowOff>
     </xdr:from>
     <xdr:to>
       <xdr:col>21</xdr:col>
       <xdr:colOff>346364</xdr:colOff>
-      <xdr:row>42</xdr:row>
+      <xdr:row>43</xdr:row>
       <xdr:rowOff>102704</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
@@ -2468,15 +2471,15 @@
   <xdr:twoCellAnchor editAs="oneCell">
     <xdr:from>
       <xdr:col>21</xdr:col>
-      <xdr:colOff>554184</xdr:colOff>
-      <xdr:row>29</xdr:row>
-      <xdr:rowOff>166256</xdr:rowOff>
+      <xdr:colOff>472248</xdr:colOff>
+      <xdr:row>31</xdr:row>
+      <xdr:rowOff>100707</xdr:rowOff>
     </xdr:from>
     <xdr:to>
       <xdr:col>28</xdr:col>
-      <xdr:colOff>341394</xdr:colOff>
-      <xdr:row>42</xdr:row>
-      <xdr:rowOff>125506</xdr:rowOff>
+      <xdr:colOff>259458</xdr:colOff>
+      <xdr:row>44</xdr:row>
+      <xdr:rowOff>59957</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -2499,8 +2502,8 @@
       </xdr:blipFill>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="13355784" y="5365785"/>
-          <a:ext cx="4054410" cy="2290074"/>
+          <a:off x="13205022" y="5688707"/>
+          <a:ext cx="4031468" cy="2302605"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -2513,13 +2516,13 @@
     <xdr:from>
       <xdr:col>21</xdr:col>
       <xdr:colOff>367555</xdr:colOff>
-      <xdr:row>42</xdr:row>
+      <xdr:row>43</xdr:row>
       <xdr:rowOff>62754</xdr:rowOff>
     </xdr:from>
     <xdr:to>
       <xdr:col>28</xdr:col>
       <xdr:colOff>332509</xdr:colOff>
-      <xdr:row>55</xdr:row>
+      <xdr:row>56</xdr:row>
       <xdr:rowOff>103650</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
@@ -2557,13 +2560,13 @@
     <xdr:from>
       <xdr:col>14</xdr:col>
       <xdr:colOff>428677</xdr:colOff>
-      <xdr:row>42</xdr:row>
+      <xdr:row>43</xdr:row>
       <xdr:rowOff>161363</xdr:rowOff>
     </xdr:from>
     <xdr:to>
       <xdr:col>21</xdr:col>
       <xdr:colOff>358588</xdr:colOff>
-      <xdr:row>56</xdr:row>
+      <xdr:row>57</xdr:row>
       <xdr:rowOff>6421</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
@@ -2601,13 +2604,13 @@
     <xdr:from>
       <xdr:col>15</xdr:col>
       <xdr:colOff>0</xdr:colOff>
-      <xdr:row>59</xdr:row>
+      <xdr:row>60</xdr:row>
       <xdr:rowOff>55433</xdr:rowOff>
     </xdr:from>
     <xdr:to>
       <xdr:col>21</xdr:col>
       <xdr:colOff>461044</xdr:colOff>
-      <xdr:row>65</xdr:row>
+      <xdr:row>66</xdr:row>
       <xdr:rowOff>322133</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
@@ -2645,13 +2648,13 @@
     <xdr:from>
       <xdr:col>15</xdr:col>
       <xdr:colOff>0</xdr:colOff>
-      <xdr:row>65</xdr:row>
+      <xdr:row>66</xdr:row>
       <xdr:rowOff>415650</xdr:rowOff>
     </xdr:from>
     <xdr:to>
       <xdr:col>21</xdr:col>
       <xdr:colOff>458551</xdr:colOff>
-      <xdr:row>72</xdr:row>
+      <xdr:row>73</xdr:row>
       <xdr:rowOff>124704</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
@@ -2689,13 +2692,13 @@
     <xdr:from>
       <xdr:col>22</xdr:col>
       <xdr:colOff>0</xdr:colOff>
-      <xdr:row>59</xdr:row>
+      <xdr:row>60</xdr:row>
       <xdr:rowOff>55433</xdr:rowOff>
     </xdr:from>
     <xdr:to>
       <xdr:col>28</xdr:col>
       <xdr:colOff>422084</xdr:colOff>
-      <xdr:row>65</xdr:row>
+      <xdr:row>66</xdr:row>
       <xdr:rowOff>346378</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
@@ -2733,13 +2736,13 @@
     <xdr:from>
       <xdr:col>22</xdr:col>
       <xdr:colOff>0</xdr:colOff>
-      <xdr:row>65</xdr:row>
+      <xdr:row>66</xdr:row>
       <xdr:rowOff>443358</xdr:rowOff>
     </xdr:from>
     <xdr:to>
       <xdr:col>28</xdr:col>
       <xdr:colOff>443345</xdr:colOff>
-      <xdr:row>73</xdr:row>
+      <xdr:row>74</xdr:row>
       <xdr:rowOff>4998</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
@@ -2777,13 +2780,13 @@
     <xdr:from>
       <xdr:col>29</xdr:col>
       <xdr:colOff>41564</xdr:colOff>
-      <xdr:row>62</xdr:row>
+      <xdr:row>63</xdr:row>
       <xdr:rowOff>249381</xdr:rowOff>
     </xdr:from>
     <xdr:to>
       <xdr:col>36</xdr:col>
       <xdr:colOff>512619</xdr:colOff>
-      <xdr:row>66</xdr:row>
+      <xdr:row>67</xdr:row>
       <xdr:rowOff>429636</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
@@ -2821,13 +2824,13 @@
     <xdr:from>
       <xdr:col>15</xdr:col>
       <xdr:colOff>2</xdr:colOff>
-      <xdr:row>77</xdr:row>
+      <xdr:row>78</xdr:row>
       <xdr:rowOff>167642</xdr:rowOff>
     </xdr:from>
     <xdr:to>
       <xdr:col>21</xdr:col>
       <xdr:colOff>526473</xdr:colOff>
-      <xdr:row>91</xdr:row>
+      <xdr:row>92</xdr:row>
       <xdr:rowOff>27584</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
@@ -2865,13 +2868,13 @@
     <xdr:from>
       <xdr:col>15</xdr:col>
       <xdr:colOff>13854</xdr:colOff>
-      <xdr:row>92</xdr:row>
+      <xdr:row>93</xdr:row>
       <xdr:rowOff>38793</xdr:rowOff>
     </xdr:from>
     <xdr:to>
       <xdr:col>21</xdr:col>
       <xdr:colOff>538119</xdr:colOff>
-      <xdr:row>105</xdr:row>
+      <xdr:row>106</xdr:row>
       <xdr:rowOff>80357</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
@@ -2909,13 +2912,13 @@
     <xdr:from>
       <xdr:col>22</xdr:col>
       <xdr:colOff>136238</xdr:colOff>
-      <xdr:row>85</xdr:row>
+      <xdr:row>86</xdr:row>
       <xdr:rowOff>11611</xdr:rowOff>
     </xdr:from>
     <xdr:to>
       <xdr:col>28</xdr:col>
       <xdr:colOff>522761</xdr:colOff>
-      <xdr:row>97</xdr:row>
+      <xdr:row>98</xdr:row>
       <xdr:rowOff>66039</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
@@ -5910,7 +5913,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{86BA37C4-8F32-417F-A8E4-D80C296F90D3}">
-  <dimension ref="A2:AD83"/>
+  <dimension ref="A2:AD84"/>
   <sheetFormatPr defaultRowHeight="14.4"/>
   <sheetData>
     <row r="2" spans="2:25">
@@ -6588,199 +6591,291 @@
         <v>4.55</v>
       </c>
     </row>
-    <row r="29" spans="2:30">
-      <c r="B29" s="142" t="s">
+    <row r="28" spans="2:30">
+      <c r="B28" s="141" t="s">
+        <v>314</v>
+      </c>
+      <c r="C28" s="144">
+        <f>C27/2</f>
+        <v>1.865</v>
+      </c>
+      <c r="D28" s="144">
+        <f>D27/2</f>
+        <v>1.9750000000000001</v>
+      </c>
+      <c r="E28" s="144">
+        <f>E27/2</f>
+        <v>2.0550000000000002</v>
+      </c>
+      <c r="G28" s="141" t="s">
+        <v>314</v>
+      </c>
+      <c r="H28" s="144">
+        <f t="shared" ref="F28:O28" si="0">H27/2</f>
+        <v>2.0449999999999999</v>
+      </c>
+      <c r="I28" s="144">
+        <f t="shared" si="0"/>
+        <v>2.11</v>
+      </c>
+      <c r="J28" s="144">
+        <f t="shared" si="0"/>
+        <v>2.15</v>
+      </c>
+      <c r="L28" s="141" t="s">
+        <v>314</v>
+      </c>
+      <c r="M28" s="144">
+        <f t="shared" si="0"/>
+        <v>2.14</v>
+      </c>
+      <c r="N28" s="144">
+        <f t="shared" si="0"/>
+        <v>2.19</v>
+      </c>
+      <c r="O28" s="144">
+        <f t="shared" si="0"/>
+        <v>2.2250000000000001</v>
+      </c>
+      <c r="Q28" s="141" t="s">
+        <v>314</v>
+      </c>
+      <c r="R28" s="144">
+        <f t="shared" ref="R28" si="1">R27/2</f>
+        <v>2.19</v>
+      </c>
+      <c r="S28" s="144">
+        <f t="shared" ref="S28" si="2">S27/2</f>
+        <v>2.2250000000000001</v>
+      </c>
+      <c r="T28" s="144">
+        <f t="shared" ref="T28" si="3">T27/2</f>
+        <v>2.2549999999999999</v>
+      </c>
+      <c r="V28" s="141" t="s">
+        <v>314</v>
+      </c>
+      <c r="W28" s="144">
+        <f t="shared" ref="W28" si="4">W27/2</f>
+        <v>2.21</v>
+      </c>
+      <c r="X28" s="144">
+        <f t="shared" ref="X28" si="5">X27/2</f>
+        <v>2.2450000000000001</v>
+      </c>
+      <c r="Y28" s="144">
+        <f t="shared" ref="Y28" si="6">Y27/2</f>
+        <v>2.2650000000000001</v>
+      </c>
+      <c r="AA28" s="141" t="s">
+        <v>314</v>
+      </c>
+      <c r="AB28" s="144">
+        <f t="shared" ref="AB28" si="7">AB27/2</f>
+        <v>2.2349999999999999</v>
+      </c>
+      <c r="AC28" s="144">
+        <f t="shared" ref="AC28" si="8">AC27/2</f>
+        <v>2.25</v>
+      </c>
+      <c r="AD28" s="144">
+        <f t="shared" ref="AD28" si="9">AD27/2</f>
+        <v>2.2749999999999999</v>
+      </c>
+    </row>
+    <row r="30" spans="2:30">
+      <c r="B30" s="142" t="s">
         <v>268</v>
       </c>
-      <c r="C29" s="138"/>
-      <c r="D29" s="138"/>
-      <c r="E29" s="138"/>
-      <c r="F29" s="138"/>
-      <c r="G29" s="138"/>
-      <c r="P29" s="138" t="s">
+      <c r="C30" s="138"/>
+      <c r="D30" s="138"/>
+      <c r="E30" s="138"/>
+      <c r="F30" s="138"/>
+      <c r="G30" s="138"/>
+      <c r="P30" s="138" t="s">
         <v>280</v>
       </c>
-      <c r="Q29" s="138"/>
-      <c r="R29" s="138"/>
-      <c r="S29" s="138"/>
-      <c r="T29" s="138"/>
-      <c r="U29" s="138"/>
-      <c r="V29" s="138"/>
-      <c r="W29" s="138"/>
-      <c r="X29" s="138"/>
-      <c r="Y29" s="138"/>
-    </row>
-    <row r="31" spans="2:30">
-      <c r="B31" s="142" t="s">
+      <c r="Q30" s="138"/>
+      <c r="R30" s="138"/>
+      <c r="S30" s="138"/>
+      <c r="T30" s="138"/>
+      <c r="U30" s="138"/>
+      <c r="V30" s="138"/>
+      <c r="W30" s="138"/>
+      <c r="X30" s="138"/>
+      <c r="Y30" s="138"/>
+    </row>
+    <row r="32" spans="2:30">
+      <c r="B32" s="142" t="s">
         <v>261</v>
       </c>
-      <c r="C31" s="138"/>
-      <c r="D31" s="138"/>
-      <c r="F31" s="138" t="s">
+      <c r="C32" s="138"/>
+      <c r="D32" s="138"/>
+      <c r="F32" s="138" t="s">
         <v>265</v>
       </c>
-      <c r="G31" s="138"/>
-      <c r="H31" s="138"/>
-      <c r="J31" t="s">
+      <c r="G32" s="138"/>
+      <c r="H32" s="138"/>
+      <c r="J32" t="s">
         <v>272</v>
       </c>
     </row>
-    <row r="32" spans="2:30">
-      <c r="B32" s="137" t="s">
+    <row r="33" spans="2:10">
+      <c r="B33" s="137" t="s">
         <v>248</v>
       </c>
-      <c r="C32" s="143">
+      <c r="C33" s="143">
         <v>2.5</v>
       </c>
-      <c r="D32" s="143">
+      <c r="D33" s="143">
         <v>3.5</v>
       </c>
-      <c r="F32" s="137" t="s">
+      <c r="F33" s="137" t="s">
         <v>248</v>
       </c>
-      <c r="G32" s="143">
+      <c r="G33" s="143">
         <v>2.5</v>
       </c>
-      <c r="H32" s="143">
+      <c r="H33" s="143">
         <v>3.5</v>
       </c>
-      <c r="J32" t="s">
+      <c r="J33" t="s">
         <v>269</v>
       </c>
     </row>
-    <row r="33" spans="2:10">
-      <c r="B33" s="162" t="s">
+    <row r="34" spans="2:10">
+      <c r="B34" s="162" t="s">
         <v>249</v>
       </c>
-      <c r="C33" s="163" t="s">
+      <c r="C34" s="163" t="s">
         <v>275</v>
       </c>
-      <c r="D33" s="163" t="s">
+      <c r="D34" s="163" t="s">
         <v>278</v>
       </c>
-      <c r="F33" s="164" t="s">
+      <c r="F34" s="164" t="s">
         <v>249</v>
       </c>
-      <c r="G33" s="163" t="s">
+      <c r="G34" s="163" t="s">
         <v>277</v>
       </c>
-      <c r="H33" s="163" t="s">
+      <c r="H34" s="163" t="s">
         <v>279</v>
       </c>
-      <c r="J33" t="s">
+      <c r="J34" t="s">
         <v>274</v>
       </c>
     </row>
-    <row r="34" spans="2:10">
-      <c r="B34" s="137" t="s">
+    <row r="35" spans="2:10">
+      <c r="B35" s="137" t="s">
         <v>226</v>
       </c>
-      <c r="C34" s="144">
+      <c r="C35" s="144">
         <v>5.04</v>
       </c>
-      <c r="D34" s="144">
+      <c r="D35" s="144">
         <v>5.05</v>
       </c>
-      <c r="F34" s="137" t="s">
+      <c r="F35" s="137" t="s">
         <v>226</v>
       </c>
-      <c r="G34" s="144">
+      <c r="G35" s="144">
         <v>4.97</v>
       </c>
-      <c r="H34" s="144">
+      <c r="H35" s="144">
         <v>4.9800000000000004</v>
       </c>
-      <c r="J34" t="s">
+      <c r="J35" t="s">
         <v>273</v>
       </c>
     </row>
-    <row r="35" spans="2:10">
-      <c r="B35" s="162" t="s">
+    <row r="36" spans="2:10">
+      <c r="B36" s="162" t="s">
         <v>266</v>
       </c>
-      <c r="C35" s="165">
-        <f>(C37/C36)</f>
+      <c r="C36" s="165">
+        <f>(C38/C37)</f>
         <v>0.68319999999999992</v>
       </c>
-      <c r="D35" s="165">
-        <f>D37/D36</f>
+      <c r="D36" s="165">
+        <f>D38/D37</f>
         <v>0.78988326848249024</v>
       </c>
-      <c r="F35" s="162" t="s">
+      <c r="F36" s="162" t="s">
         <v>266</v>
       </c>
-      <c r="G35" s="165">
-        <f>G37/G36</f>
+      <c r="G36" s="165">
+        <f>G38/G37</f>
         <v>0.86</v>
       </c>
-      <c r="H35" s="165">
-        <f>H37/H36</f>
+      <c r="H36" s="165">
+        <f>H38/H37</f>
         <v>0.86</v>
-      </c>
-    </row>
-    <row r="36" spans="2:10">
-      <c r="B36" s="141" t="s">
-        <v>267</v>
-      </c>
-      <c r="C36" s="144">
-        <v>6.25</v>
-      </c>
-      <c r="D36" s="144">
-        <v>5.14</v>
-      </c>
-      <c r="F36" s="141" t="s">
-        <v>267</v>
-      </c>
-      <c r="G36" s="144">
-        <v>0.5</v>
-      </c>
-      <c r="H36" s="144">
-        <v>0.5</v>
-      </c>
-      <c r="J36" t="s">
-        <v>270</v>
       </c>
     </row>
     <row r="37" spans="2:10">
       <c r="B37" s="141" t="s">
-        <v>15</v>
+        <v>267</v>
       </c>
       <c r="C37" s="144">
-        <v>4.2699999999999996</v>
+        <v>6.25</v>
       </c>
       <c r="D37" s="144">
-        <v>4.0599999999999996</v>
+        <v>5.14</v>
       </c>
       <c r="F37" s="141" t="s">
-        <v>15</v>
+        <v>267</v>
       </c>
       <c r="G37" s="144">
-        <v>0.43</v>
+        <v>0.5</v>
       </c>
       <c r="H37" s="144">
-        <v>0.43</v>
+        <v>0.5</v>
       </c>
       <c r="J37" t="s">
-        <v>271</v>
+        <v>270</v>
       </c>
     </row>
     <row r="38" spans="2:10">
       <c r="B38" s="141" t="s">
+        <v>15</v>
+      </c>
+      <c r="C38" s="144">
+        <v>4.2699999999999996</v>
+      </c>
+      <c r="D38" s="144">
+        <v>4.0599999999999996</v>
+      </c>
+      <c r="F38" s="141" t="s">
+        <v>15</v>
+      </c>
+      <c r="G38" s="144">
+        <v>0.43</v>
+      </c>
+      <c r="H38" s="144">
+        <v>0.43</v>
+      </c>
+      <c r="J38" t="s">
+        <v>271</v>
+      </c>
+    </row>
+    <row r="39" spans="2:10">
+      <c r="B39" s="141" t="s">
         <v>276</v>
       </c>
-      <c r="C38" s="145">
+      <c r="C39" s="145">
         <v>3.9</v>
       </c>
-      <c r="D38" s="145">
+      <c r="D39" s="145">
         <v>4.04</v>
       </c>
-      <c r="F38" s="141" t="s">
+      <c r="F39" s="141" t="s">
         <v>276</v>
       </c>
-      <c r="G38" s="145">
+      <c r="G39" s="145">
         <v>2.88</v>
       </c>
-      <c r="H38" s="145">
+      <c r="H39" s="145">
         <v>2.56</v>
       </c>
     </row>
@@ -6794,283 +6889,266 @@
         <v>298</v>
       </c>
     </row>
-    <row r="58" spans="1:22">
-      <c r="B58" s="149" t="s">
+    <row r="59" spans="1:22">
+      <c r="B59" s="149" t="s">
         <v>283</v>
       </c>
-      <c r="C58" s="149"/>
-      <c r="D58" s="149"/>
-      <c r="E58" s="149"/>
-      <c r="F58" s="149"/>
-      <c r="J58" s="149" t="s">
+      <c r="C59" s="149"/>
+      <c r="D59" s="149"/>
+      <c r="E59" s="149"/>
+      <c r="F59" s="149"/>
+      <c r="J59" s="149" t="s">
         <v>288</v>
       </c>
-      <c r="K58" s="149"/>
-      <c r="P58" s="149" t="s">
+      <c r="K59" s="149"/>
+      <c r="P59" s="149" t="s">
         <v>308</v>
       </c>
-      <c r="Q58" s="149"/>
-      <c r="R58" s="149"/>
-      <c r="S58" s="149"/>
-      <c r="T58" s="149"/>
-      <c r="U58" s="149"/>
-      <c r="V58" s="149"/>
-    </row>
-    <row r="60" spans="1:22">
-      <c r="B60" s="148" t="s">
+      <c r="Q59" s="149"/>
+      <c r="R59" s="149"/>
+      <c r="S59" s="149"/>
+      <c r="T59" s="149"/>
+      <c r="U59" s="149"/>
+      <c r="V59" s="149"/>
+    </row>
+    <row r="61" spans="1:22">
+      <c r="B61" s="148" t="s">
         <v>261</v>
       </c>
-      <c r="C60" s="149"/>
-      <c r="D60" s="149"/>
-      <c r="F60" s="148" t="s">
+      <c r="C61" s="149"/>
+      <c r="D61" s="149"/>
+      <c r="F61" s="148" t="s">
         <v>265</v>
       </c>
-      <c r="G60" s="149"/>
-      <c r="H60" s="149"/>
-      <c r="J60" s="149" t="s">
+      <c r="G61" s="149"/>
+      <c r="H61" s="149"/>
+      <c r="J61" s="149" t="s">
         <v>261</v>
       </c>
-      <c r="K60" s="149"/>
-    </row>
-    <row r="61" spans="1:22">
-      <c r="B61" s="150" t="s">
+      <c r="K61" s="149"/>
+    </row>
+    <row r="62" spans="1:22">
+      <c r="B62" s="150" t="s">
         <v>248</v>
       </c>
-      <c r="C61" s="143">
+      <c r="C62" s="143">
         <v>2.5</v>
       </c>
-      <c r="D61" s="143">
+      <c r="D62" s="143">
         <v>3.5</v>
       </c>
-      <c r="F61" s="150" t="s">
+      <c r="F62" s="150" t="s">
         <v>248</v>
       </c>
-      <c r="G61" s="143">
+      <c r="G62" s="143">
         <v>2.5</v>
       </c>
-      <c r="H61" s="143">
+      <c r="H62" s="143">
         <v>3.5</v>
       </c>
-      <c r="J61" s="150" t="s">
+      <c r="J62" s="150" t="s">
         <v>248</v>
       </c>
-      <c r="K61" s="160">
+      <c r="K62" s="160">
         <v>2.5</v>
       </c>
     </row>
-    <row r="62" spans="1:22">
-      <c r="B62" s="151" t="s">
+    <row r="63" spans="1:22">
+      <c r="B63" s="151" t="s">
         <v>249</v>
       </c>
-      <c r="C62" s="152">
+      <c r="C63" s="152">
         <v>0.5</v>
       </c>
-      <c r="D62" s="152">
+      <c r="D63" s="152">
         <v>0.3</v>
       </c>
-      <c r="F62" s="151" t="s">
+      <c r="F63" s="151" t="s">
         <v>249</v>
       </c>
-      <c r="G62" s="152">
+      <c r="G63" s="152">
         <v>0.5</v>
       </c>
-      <c r="H62" s="152">
+      <c r="H63" s="152">
         <v>0.3</v>
       </c>
-      <c r="J62" s="150" t="s">
+      <c r="J63" s="150" t="s">
         <v>289</v>
       </c>
-      <c r="K62" s="160">
+      <c r="K63" s="160">
         <v>0.5</v>
       </c>
     </row>
-    <row r="63" spans="1:22" ht="28.8">
-      <c r="B63" s="158" t="s">
+    <row r="64" spans="1:22" ht="28.8">
+      <c r="B64" s="158" t="s">
         <v>284</v>
       </c>
-      <c r="C63" s="157">
+      <c r="C64" s="157">
         <v>73</v>
       </c>
-      <c r="D63" s="157">
+      <c r="D64" s="157">
         <v>35.700000000000003</v>
       </c>
-      <c r="F63" s="158" t="s">
+      <c r="F64" s="158" t="s">
         <v>284</v>
       </c>
-      <c r="G63" s="157">
+      <c r="G64" s="157">
         <v>8.8000000000000007</v>
       </c>
-      <c r="H63" s="157">
+      <c r="H64" s="157">
         <v>3.9</v>
       </c>
-      <c r="J63" s="158" t="s">
+      <c r="J64" s="158" t="s">
         <v>290</v>
       </c>
-      <c r="K63" s="157">
+      <c r="K64" s="157">
         <v>1.85</v>
       </c>
     </row>
-    <row r="64" spans="1:22" ht="57.6">
-      <c r="B64" s="156" t="s">
+    <row r="65" spans="2:20" ht="57.6">
+      <c r="B65" s="156" t="s">
         <v>285</v>
       </c>
-      <c r="C64" s="154">
+      <c r="C65" s="154">
         <v>612</v>
       </c>
-      <c r="D64" s="154">
+      <c r="D65" s="154">
         <v>592.9</v>
       </c>
-      <c r="F64" s="156" t="s">
+      <c r="F65" s="156" t="s">
         <v>285</v>
       </c>
-      <c r="G64" s="154">
+      <c r="G65" s="154">
         <v>250</v>
       </c>
-      <c r="H64" s="155">
+      <c r="H65" s="155">
         <v>231.3</v>
       </c>
-      <c r="J64" s="156" t="s">
+      <c r="J65" s="156" t="s">
         <v>292</v>
       </c>
-      <c r="K64" s="154">
+      <c r="K65" s="154">
         <v>0.42</v>
       </c>
     </row>
-    <row r="65" spans="2:20" ht="28.8">
-      <c r="B65" s="159" t="s">
+    <row r="66" spans="2:20" ht="28.8">
+      <c r="B66" s="159" t="s">
         <v>286</v>
       </c>
-      <c r="C65" s="157">
+      <c r="C66" s="157">
         <v>277.89999999999998</v>
       </c>
-      <c r="D65" s="157">
+      <c r="D66" s="157">
         <v>131.4</v>
       </c>
-      <c r="F65" s="159" t="s">
+      <c r="F66" s="159" t="s">
         <v>286</v>
       </c>
-      <c r="G65" s="157">
+      <c r="G66" s="157">
         <v>39.6</v>
       </c>
-      <c r="H65" s="157">
+      <c r="H66" s="157">
         <v>19.8</v>
       </c>
-      <c r="J65" s="159" t="s">
+      <c r="J66" s="159" t="s">
         <v>291</v>
       </c>
-      <c r="K65" s="157">
+      <c r="K66" s="157">
         <v>3.66</v>
       </c>
     </row>
-    <row r="66" spans="2:20" ht="57.6">
-      <c r="B66" s="156" t="s">
+    <row r="67" spans="2:20" ht="57.6">
+      <c r="B67" s="156" t="s">
         <v>287</v>
       </c>
-      <c r="C66" s="153">
+      <c r="C67" s="153">
         <v>749.7</v>
       </c>
-      <c r="D66" s="152">
+      <c r="D67" s="152">
         <v>558.6</v>
       </c>
-      <c r="F66" s="156" t="s">
+      <c r="F67" s="156" t="s">
         <v>287</v>
       </c>
-      <c r="G66" s="153">
+      <c r="G67" s="153">
         <v>211.7</v>
       </c>
-      <c r="H66" s="152">
+      <c r="H67" s="152">
         <v>181.8</v>
       </c>
-      <c r="J66" s="156" t="s">
+      <c r="J67" s="156" t="s">
         <v>293</v>
       </c>
-      <c r="K66" s="153">
+      <c r="K67" s="153">
         <v>2.99</v>
-      </c>
-    </row>
-    <row r="67" spans="2:20" ht="43.2">
-      <c r="B67" s="161" t="s">
-        <v>295</v>
-      </c>
-      <c r="C67" s="161" t="s">
-        <v>297</v>
-      </c>
-      <c r="D67" s="161" t="s">
-        <v>302</v>
-      </c>
-      <c r="E67" s="161"/>
-      <c r="F67" s="161"/>
-      <c r="G67" s="161" t="s">
-        <v>300</v>
-      </c>
-      <c r="H67" s="161" t="s">
-        <v>303</v>
-      </c>
-      <c r="I67" s="161"/>
-      <c r="J67" s="161"/>
-      <c r="K67" s="161" t="s">
-        <v>306</v>
       </c>
     </row>
     <row r="68" spans="2:20" ht="43.2">
       <c r="B68" s="161" t="s">
-        <v>294</v>
+        <v>295</v>
       </c>
       <c r="C68" s="161" t="s">
-        <v>296</v>
+        <v>297</v>
       </c>
       <c r="D68" s="161" t="s">
-        <v>305</v>
+        <v>302</v>
       </c>
       <c r="E68" s="161"/>
       <c r="F68" s="161"/>
       <c r="G68" s="161" t="s">
-        <v>301</v>
+        <v>300</v>
       </c>
       <c r="H68" s="161" t="s">
-        <v>304</v>
+        <v>303</v>
       </c>
       <c r="I68" s="161"/>
       <c r="J68" s="161"/>
       <c r="K68" s="161" t="s">
+        <v>306</v>
+      </c>
+    </row>
+    <row r="69" spans="2:20" ht="43.2">
+      <c r="B69" s="161" t="s">
+        <v>294</v>
+      </c>
+      <c r="C69" s="161" t="s">
+        <v>296</v>
+      </c>
+      <c r="D69" s="161" t="s">
+        <v>305</v>
+      </c>
+      <c r="E69" s="161"/>
+      <c r="F69" s="161"/>
+      <c r="G69" s="161" t="s">
+        <v>301</v>
+      </c>
+      <c r="H69" s="161" t="s">
+        <v>304</v>
+      </c>
+      <c r="I69" s="161"/>
+      <c r="J69" s="161"/>
+      <c r="K69" s="161" t="s">
         <v>307</v>
       </c>
     </row>
-    <row r="76" spans="2:20">
-      <c r="B76" s="146" t="s">
+    <row r="77" spans="2:20">
+      <c r="B77" s="146" t="s">
         <v>282</v>
       </c>
-      <c r="C76" s="147"/>
-      <c r="D76" s="147"/>
-      <c r="E76" s="147"/>
-      <c r="P76" s="147" t="s">
+      <c r="C77" s="147"/>
+      <c r="D77" s="147"/>
+      <c r="E77" s="147"/>
+      <c r="P77" s="147" t="s">
         <v>313</v>
       </c>
-      <c r="Q76" s="147"/>
-      <c r="R76" s="147"/>
-      <c r="S76" s="147"/>
-      <c r="T76" s="147"/>
-    </row>
-    <row r="78" spans="2:20">
-      <c r="B78" s="146" t="s">
+      <c r="Q77" s="147"/>
+      <c r="R77" s="147"/>
+      <c r="S77" s="147"/>
+      <c r="T77" s="147"/>
+    </row>
+    <row r="79" spans="2:20">
+      <c r="B79" s="146" t="s">
         <v>281</v>
-      </c>
-      <c r="C78" s="147"/>
-      <c r="D78" s="147"/>
-      <c r="E78" s="147"/>
-      <c r="F78" s="147"/>
-      <c r="G78" s="147"/>
-      <c r="H78" s="147"/>
-      <c r="I78" s="147"/>
-      <c r="J78" s="147"/>
-      <c r="K78" s="147"/>
-      <c r="L78" s="147"/>
-      <c r="M78" s="147"/>
-      <c r="N78" s="147"/>
-    </row>
-    <row r="79" spans="2:20">
-      <c r="B79" s="147" t="s">
-        <v>311</v>
       </c>
       <c r="C79" s="147"/>
       <c r="D79" s="147"/>
@@ -7086,8 +7164,8 @@
       <c r="N79" s="147"/>
     </row>
     <row r="80" spans="2:20">
-      <c r="B80" s="146" t="s">
-        <v>312</v>
+      <c r="B80" s="147" t="s">
+        <v>311</v>
       </c>
       <c r="C80" s="147"/>
       <c r="D80" s="147"/>
@@ -7103,7 +7181,9 @@
       <c r="N80" s="147"/>
     </row>
     <row r="81" spans="2:14">
-      <c r="B81" s="147"/>
+      <c r="B81" s="146" t="s">
+        <v>312</v>
+      </c>
       <c r="C81" s="147"/>
       <c r="D81" s="147"/>
       <c r="E81" s="147"/>
@@ -7118,9 +7198,7 @@
       <c r="N81" s="147"/>
     </row>
     <row r="82" spans="2:14">
-      <c r="B82" s="146" t="s">
-        <v>309</v>
-      </c>
+      <c r="B82" s="147"/>
       <c r="C82" s="147"/>
       <c r="D82" s="147"/>
       <c r="E82" s="147"/>
@@ -7135,8 +7213,8 @@
       <c r="N82" s="147"/>
     </row>
     <row r="83" spans="2:14">
-      <c r="B83" s="147" t="s">
-        <v>310</v>
+      <c r="B83" s="146" t="s">
+        <v>309</v>
       </c>
       <c r="C83" s="147"/>
       <c r="D83" s="147"/>
@@ -7151,6 +7229,23 @@
       <c r="M83" s="147"/>
       <c r="N83" s="147"/>
     </row>
+    <row r="84" spans="2:14">
+      <c r="B84" s="147" t="s">
+        <v>310</v>
+      </c>
+      <c r="C84" s="147"/>
+      <c r="D84" s="147"/>
+      <c r="E84" s="147"/>
+      <c r="F84" s="147"/>
+      <c r="G84" s="147"/>
+      <c r="H84" s="147"/>
+      <c r="I84" s="147"/>
+      <c r="J84" s="147"/>
+      <c r="K84" s="147"/>
+      <c r="L84" s="147"/>
+      <c r="M84" s="147"/>
+      <c r="N84" s="147"/>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" r:id="rId1"/>

</xml_diff>

<commit_message>
Open Loop testing values saved and updated on Excel (Boost Converter)
</commit_message>
<xml_diff>
--- a/Excel/Boost Converter Design Params.xlsx
+++ b/Excel/Boost Converter Design Params.xlsx
@@ -8,17 +8,17 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\tytom\Documents\GitHub\311\Excel\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4A94C463-2E29-47D2-95EE-DD776DA90086}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EC7F3BDD-F69B-4F14-99E6-6CA8FAEB6FD6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="2" xr2:uid="{0EA872C3-4804-43CB-9F0B-5F94DB7B4351}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="3" xr2:uid="{0EA872C3-4804-43CB-9F0B-5F94DB7B4351}"/>
   </bookViews>
   <sheets>
     <sheet name="SS_Analysis" sheetId="1" r:id="rId1"/>
     <sheet name="Inductor_Design" sheetId="2" r:id="rId2"/>
     <sheet name="Testing_Openloop" sheetId="4" r:id="rId3"/>
+    <sheet name="Testing_Closedloop" sheetId="5" r:id="rId4"/>
   </sheets>
   <calcPr calcId="191029"/>
-  <fileRecoveryPr repairLoad="1"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="631" uniqueCount="315">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="647" uniqueCount="320">
   <si>
     <t>Parameter</t>
   </si>
@@ -982,6 +982,21 @@
   </si>
   <si>
     <t>MCU_VFB</t>
+  </si>
+  <si>
+    <t>2.5V Vin Results</t>
+  </si>
+  <si>
+    <t>Rl</t>
+  </si>
+  <si>
+    <t>3.5V Vin Results</t>
+  </si>
+  <si>
+    <t>V ripple (mV)</t>
+  </si>
+  <si>
+    <t>Trise (ms)</t>
   </si>
 </sst>
 </file>
@@ -2151,7 +2166,7 @@
     <xf numFmtId="0" fontId="1" fillId="16" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="1" fillId="17" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="166">
+  <cellXfs count="170">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
@@ -2342,6 +2357,14 @@
     <xf numFmtId="0" fontId="9" fillId="8" borderId="66" xfId="5" applyFont="1"/>
     <xf numFmtId="0" fontId="9" fillId="10" borderId="0" xfId="7" applyFont="1"/>
     <xf numFmtId="9" fontId="9" fillId="8" borderId="66" xfId="5" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="0" fontId="0" fillId="11" borderId="0" xfId="8" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="10" borderId="0" xfId="7" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="8" borderId="67" xfId="5" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="8" borderId="66" xfId="5" applyFont="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
   </cellXfs>
   <cellStyles count="15">
     <cellStyle name="20% - Accent1" xfId="2" builtinId="30"/>
@@ -2955,6 +2978,111 @@
 </xdr:wsDr>
 </file>
 
+<file path=xl/drawings/drawing3.xml><?xml version="1.0" encoding="utf-8"?>
+<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>1</xdr:col>
+      <xdr:colOff>21771</xdr:colOff>
+      <xdr:row>12</xdr:row>
+      <xdr:rowOff>19049</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>13</xdr:col>
+      <xdr:colOff>424542</xdr:colOff>
+      <xdr:row>36</xdr:row>
+      <xdr:rowOff>176331</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="3" name="Picture 2">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{F4FFD07B-5FAE-0D56-B693-31F49E9B2EE6}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId1" cstate="print">
+          <a:extLst>
+            <a:ext uri="{28A0092B-C50C-407E-A947-70E740481C1C}">
+              <a14:useLocalDpi xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" val="0"/>
+            </a:ext>
+          </a:extLst>
+        </a:blip>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="631371" y="2239735"/>
+          <a:ext cx="8098971" cy="4598653"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>13</xdr:col>
+      <xdr:colOff>609599</xdr:colOff>
+      <xdr:row>12</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>27</xdr:col>
+      <xdr:colOff>200110</xdr:colOff>
+      <xdr:row>36</xdr:row>
+      <xdr:rowOff>121920</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="5" name="Picture 4">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{D9F36C05-1931-F7E8-9376-25A5C4BBB468}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId2" cstate="print">
+          <a:extLst>
+            <a:ext uri="{28A0092B-C50C-407E-A947-70E740481C1C}">
+              <a14:useLocalDpi xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" val="0"/>
+            </a:ext>
+          </a:extLst>
+        </a:blip>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="8923019" y="2194560"/>
+          <a:ext cx="8124911" cy="4511040"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+</xdr:wsDr>
+</file>
+
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
 <a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
   <a:themeElements>
@@ -6611,7 +6739,7 @@
         <v>314</v>
       </c>
       <c r="H28" s="144">
-        <f t="shared" ref="F28:O28" si="0">H27/2</f>
+        <f t="shared" ref="H28:O28" si="0">H27/2</f>
         <v>2.0449999999999999</v>
       </c>
       <c r="I28" s="144">
@@ -7253,6 +7381,219 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{6D3DD6BC-0BCA-4BA9-9C7E-A308795ECB28}">
+  <dimension ref="B4:R11"/>
+  <sheetFormatPr defaultRowHeight="14.4"/>
+  <cols>
+    <col min="2" max="2" width="11.33203125" customWidth="1"/>
+    <col min="7" max="7" width="12.109375" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="4" spans="2:18">
+      <c r="B4" s="142" t="s">
+        <v>315</v>
+      </c>
+      <c r="C4" s="138"/>
+      <c r="O4" s="166" t="s">
+        <v>317</v>
+      </c>
+      <c r="P4" s="138"/>
+    </row>
+    <row r="5" spans="2:18">
+      <c r="B5" s="167" t="s">
+        <v>316</v>
+      </c>
+      <c r="C5" s="137">
+        <v>5</v>
+      </c>
+      <c r="D5" s="137">
+        <v>10</v>
+      </c>
+      <c r="E5" s="137">
+        <v>50</v>
+      </c>
+      <c r="O5" s="167" t="s">
+        <v>316</v>
+      </c>
+      <c r="P5" s="137">
+        <v>5</v>
+      </c>
+      <c r="Q5" s="137">
+        <v>10</v>
+      </c>
+      <c r="R5" s="137">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="6" spans="2:18">
+      <c r="B6" s="137" t="s">
+        <v>226</v>
+      </c>
+      <c r="C6" s="144">
+        <v>4.7949999999999999</v>
+      </c>
+      <c r="D6" s="144">
+        <v>5.1630000000000003</v>
+      </c>
+      <c r="E6" s="144">
+        <v>5.194</v>
+      </c>
+      <c r="O6" s="137" t="s">
+        <v>226</v>
+      </c>
+      <c r="P6" s="144">
+        <v>5.1630000000000003</v>
+      </c>
+      <c r="Q6" s="144">
+        <v>5.1609999999999996</v>
+      </c>
+      <c r="R6" s="144">
+        <v>5.19</v>
+      </c>
+    </row>
+    <row r="7" spans="2:18">
+      <c r="B7" s="162" t="s">
+        <v>266</v>
+      </c>
+      <c r="C7" s="165">
+        <f>C9/C8</f>
+        <v>0.63833075734157652</v>
+      </c>
+      <c r="D7" s="165">
+        <f>D9/D8</f>
+        <v>0.78412698412698423</v>
+      </c>
+      <c r="E7" s="165">
+        <f>E9/E8</f>
+        <v>0.89473684210526327</v>
+      </c>
+      <c r="O7" s="162" t="s">
+        <v>266</v>
+      </c>
+      <c r="P7" s="165">
+        <f>P9/P8</f>
+        <v>0.76984126984126977</v>
+      </c>
+      <c r="Q7" s="165">
+        <f>Q9/Q8</f>
+        <v>0.8512110726643598</v>
+      </c>
+      <c r="R7" s="165">
+        <f>R9/R8</f>
+        <v>0.90909090909090906</v>
+      </c>
+    </row>
+    <row r="8" spans="2:18">
+      <c r="B8" s="141" t="s">
+        <v>267</v>
+      </c>
+      <c r="C8" s="144">
+        <v>6.47</v>
+      </c>
+      <c r="D8" s="144">
+        <v>3.15</v>
+      </c>
+      <c r="E8" s="144">
+        <v>0.56999999999999995</v>
+      </c>
+      <c r="O8" s="141" t="s">
+        <v>267</v>
+      </c>
+      <c r="P8" s="144">
+        <v>6.3</v>
+      </c>
+      <c r="Q8" s="144">
+        <v>2.89</v>
+      </c>
+      <c r="R8" s="144">
+        <v>0.55000000000000004</v>
+      </c>
+    </row>
+    <row r="9" spans="2:18">
+      <c r="B9" s="141" t="s">
+        <v>15</v>
+      </c>
+      <c r="C9" s="144">
+        <v>4.13</v>
+      </c>
+      <c r="D9" s="144">
+        <v>2.4700000000000002</v>
+      </c>
+      <c r="E9" s="144">
+        <v>0.51</v>
+      </c>
+      <c r="O9" s="141" t="s">
+        <v>15</v>
+      </c>
+      <c r="P9" s="144">
+        <v>4.8499999999999996</v>
+      </c>
+      <c r="Q9" s="144">
+        <v>2.46</v>
+      </c>
+      <c r="R9" s="144">
+        <v>0.5</v>
+      </c>
+    </row>
+    <row r="10" spans="2:18">
+      <c r="B10" s="167" t="s">
+        <v>318</v>
+      </c>
+      <c r="C10" s="168">
+        <v>240</v>
+      </c>
+      <c r="D10" s="168">
+        <v>119</v>
+      </c>
+      <c r="E10" s="168">
+        <v>51</v>
+      </c>
+      <c r="O10" s="167" t="s">
+        <v>318</v>
+      </c>
+      <c r="P10" s="168">
+        <v>141</v>
+      </c>
+      <c r="Q10" s="168">
+        <v>89</v>
+      </c>
+      <c r="R10" s="168">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="11" spans="2:18">
+      <c r="B11" s="167" t="s">
+        <v>319</v>
+      </c>
+      <c r="C11" s="169">
+        <v>118.5</v>
+      </c>
+      <c r="D11" s="169">
+        <v>28.4</v>
+      </c>
+      <c r="E11" s="169">
+        <v>20.8</v>
+      </c>
+      <c r="O11" s="167" t="s">
+        <v>319</v>
+      </c>
+      <c r="P11" s="169">
+        <v>30.1</v>
+      </c>
+      <c r="Q11" s="169">
+        <v>14.9</v>
+      </c>
+      <c r="R11" s="169">
+        <v>15.5</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <drawing r:id="rId1"/>
+</worksheet>
+</file>
+
 <file path=docMetadata/LabelInfo.xml><?xml version="1.0" encoding="utf-8"?>
 <clbl:labelList xmlns:clbl="http://schemas.microsoft.com/office/2020/mipLabelMetadata">
   <clbl:label id="{b75eb9d1-7479-4f8a-9240-cc5b19dbbc64}" enabled="1" method="Standard" siteId="{d1b36e95-0d50-42e9-958f-b63fa906beaa}" removed="0"/>

</xml_diff>

<commit_message>
Tab added for steady-state error to excel
</commit_message>
<xml_diff>
--- a/Excel/Boost Converter Design Params.xlsx
+++ b/Excel/Boost Converter Design Params.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30430"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30527"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\tytom\Documents\GitHub\311\Excel\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/bb665e811a262358/Documents/GitHub/311/Excel/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EC7F3BDD-F69B-4F14-99E6-6CA8FAEB6FD6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="15" documentId="13_ncr:1_{EC7F3BDD-F69B-4F14-99E6-6CA8FAEB6FD6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{1C893AFE-EEF7-4A68-BFC7-AB1589E47531}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="3" xr2:uid="{0EA872C3-4804-43CB-9F0B-5F94DB7B4351}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="3" xr2:uid="{0EA872C3-4804-43CB-9F0B-5F94DB7B4351}"/>
   </bookViews>
   <sheets>
     <sheet name="SS_Analysis" sheetId="1" r:id="rId1"/>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="647" uniqueCount="320">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="649" uniqueCount="321">
   <si>
     <t>Parameter</t>
   </si>
@@ -997,6 +997,9 @@
   </si>
   <si>
     <t>Trise (ms)</t>
+  </si>
+  <si>
+    <t>SS Error (V)</t>
   </si>
 </sst>
 </file>
@@ -1011,7 +1014,7 @@
     <numFmt numFmtId="168" formatCode="0.0000000"/>
     <numFmt numFmtId="169" formatCode="0.0000"/>
   </numFmts>
-  <fonts count="12">
+  <fonts count="12" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -2166,7 +2169,7 @@
     <xf numFmtId="0" fontId="1" fillId="16" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="1" fillId="17" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="170">
+  <cellXfs count="172">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
@@ -2359,12 +2362,14 @@
     <xf numFmtId="9" fontId="9" fillId="8" borderId="66" xfId="5" applyNumberFormat="1" applyFont="1"/>
     <xf numFmtId="0" fontId="0" fillId="11" borderId="0" xfId="8" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="10" borderId="0" xfId="7" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="8" borderId="67" xfId="5" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="9" fillId="8" borderId="67" xfId="5" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="8" borderId="66" xfId="5" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="9" fillId="8" borderId="66" xfId="5" applyFont="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
+    <xf numFmtId="0" fontId="1" fillId="10" borderId="0" xfId="7" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="9" fontId="1" fillId="8" borderId="66" xfId="5" applyNumberFormat="1" applyFont="1"/>
   </cellXfs>
   <cellStyles count="15">
     <cellStyle name="20% - Accent1" xfId="2" builtinId="30"/>
@@ -2984,14 +2989,14 @@
     <xdr:from>
       <xdr:col>1</xdr:col>
       <xdr:colOff>21771</xdr:colOff>
-      <xdr:row>12</xdr:row>
-      <xdr:rowOff>19049</xdr:rowOff>
+      <xdr:row>15</xdr:row>
+      <xdr:rowOff>88321</xdr:rowOff>
     </xdr:from>
     <xdr:to>
       <xdr:col>13</xdr:col>
       <xdr:colOff>424542</xdr:colOff>
-      <xdr:row>36</xdr:row>
-      <xdr:rowOff>176331</xdr:rowOff>
+      <xdr:row>40</xdr:row>
+      <xdr:rowOff>55103</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -3020,8 +3025,8 @@
       </xdr:blipFill>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="631371" y="2239735"/>
-          <a:ext cx="8098971" cy="4598653"/>
+          <a:off x="627907" y="2945821"/>
+          <a:ext cx="8022771" cy="4729282"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -3032,16 +3037,16 @@
   </xdr:twoCellAnchor>
   <xdr:twoCellAnchor editAs="oneCell">
     <xdr:from>
-      <xdr:col>13</xdr:col>
-      <xdr:colOff>609599</xdr:colOff>
-      <xdr:row>12</xdr:row>
-      <xdr:rowOff>0</xdr:rowOff>
+      <xdr:col>14</xdr:col>
+      <xdr:colOff>107371</xdr:colOff>
+      <xdr:row>15</xdr:row>
+      <xdr:rowOff>121227</xdr:rowOff>
     </xdr:from>
     <xdr:to>
       <xdr:col>27</xdr:col>
-      <xdr:colOff>200110</xdr:colOff>
-      <xdr:row>36</xdr:row>
-      <xdr:rowOff>121920</xdr:rowOff>
+      <xdr:colOff>157481</xdr:colOff>
+      <xdr:row>40</xdr:row>
+      <xdr:rowOff>52647</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -3070,8 +3075,8 @@
       </xdr:blipFill>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="8923019" y="2194560"/>
-          <a:ext cx="8124911" cy="4511040"/>
+          <a:off x="8939644" y="2978727"/>
+          <a:ext cx="8076420" cy="4693920"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -3401,30 +3406,30 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E4C28CAE-7D6E-414C-9BF7-B54583CFEE9E}">
   <dimension ref="A1:N129"/>
-  <sheetFormatPr defaultColWidth="12" defaultRowHeight="14.4"/>
+  <sheetFormatPr defaultColWidth="12" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="20.44140625" customWidth="1"/>
-    <col min="2" max="2" width="13.5546875" customWidth="1"/>
-    <col min="3" max="3" width="13.33203125" customWidth="1"/>
-    <col min="4" max="7" width="12.88671875" customWidth="1"/>
+    <col min="1" max="1" width="20.42578125" customWidth="1"/>
+    <col min="2" max="2" width="13.5703125" customWidth="1"/>
+    <col min="3" max="3" width="13.28515625" customWidth="1"/>
+    <col min="4" max="7" width="12.85546875" customWidth="1"/>
     <col min="8" max="8" width="22" customWidth="1"/>
-    <col min="9" max="11" width="12.88671875" customWidth="1"/>
-    <col min="12" max="12" width="17.44140625" customWidth="1"/>
-    <col min="13" max="13" width="18.88671875" customWidth="1"/>
+    <col min="9" max="11" width="12.85546875" customWidth="1"/>
+    <col min="12" max="12" width="17.42578125" customWidth="1"/>
+    <col min="13" max="13" width="18.85546875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" ht="21">
+    <row r="1" spans="1:3" ht="21" x14ac:dyDescent="0.35">
       <c r="A1" s="1" t="s">
         <v>58</v>
       </c>
     </row>
-    <row r="3" spans="1:3" ht="18">
+    <row r="3" spans="1:3" ht="18.75" x14ac:dyDescent="0.3">
       <c r="A3" s="2" t="s">
         <v>137</v>
       </c>
     </row>
-    <row r="4" spans="1:3" ht="15" thickBot="1"/>
-    <row r="5" spans="1:3" ht="15.6" thickTop="1" thickBot="1">
+    <row r="4" spans="1:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
+    <row r="5" spans="1:3" ht="16.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A5" s="3" t="s">
         <v>0</v>
       </c>
@@ -3435,7 +3440,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="6" spans="1:3" ht="15" thickTop="1">
+    <row r="6" spans="1:3" ht="15.75" thickTop="1" x14ac:dyDescent="0.25">
       <c r="A6" s="37" t="s">
         <v>36</v>
       </c>
@@ -3446,7 +3451,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="7" spans="1:3">
+    <row r="7" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A7" s="38" t="s">
         <v>37</v>
       </c>
@@ -3457,7 +3462,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="8" spans="1:3">
+    <row r="8" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A8" s="38" t="s">
         <v>38</v>
       </c>
@@ -3468,7 +3473,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="9" spans="1:3">
+    <row r="9" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A9" s="38" t="s">
         <v>56</v>
       </c>
@@ -3479,7 +3484,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="10" spans="1:3">
+    <row r="10" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A10" s="38" t="s">
         <v>57</v>
       </c>
@@ -3490,7 +3495,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="11" spans="1:3" ht="15" thickBot="1">
+    <row r="11" spans="1:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A11" s="10" t="s">
         <v>5</v>
       </c>
@@ -3501,16 +3506,16 @@
         <v>6</v>
       </c>
     </row>
-    <row r="12" spans="1:3" ht="16.2" thickTop="1">
+    <row r="12" spans="1:3" ht="16.5" thickTop="1" x14ac:dyDescent="0.25">
       <c r="A12" s="13"/>
     </row>
-    <row r="14" spans="1:3" ht="18">
+    <row r="14" spans="1:3" ht="18.75" x14ac:dyDescent="0.3">
       <c r="A14" s="2" t="s">
         <v>55</v>
       </c>
     </row>
-    <row r="15" spans="1:3" ht="15" thickBot="1"/>
-    <row r="16" spans="1:3" ht="15.6" thickTop="1" thickBot="1">
+    <row r="15" spans="1:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
+    <row r="16" spans="1:3" ht="16.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A16" s="3" t="s">
         <v>0</v>
       </c>
@@ -3521,7 +3526,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="17" spans="1:3" ht="15" thickTop="1">
+    <row r="17" spans="1:3" ht="15.75" thickTop="1" x14ac:dyDescent="0.25">
       <c r="A17" s="45" t="s">
         <v>41</v>
       </c>
@@ -3533,7 +3538,7 @@
         <v>102</v>
       </c>
     </row>
-    <row r="18" spans="1:3">
+    <row r="18" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A18" s="47" t="s">
         <v>40</v>
       </c>
@@ -3545,7 +3550,7 @@
         <v>103</v>
       </c>
     </row>
-    <row r="19" spans="1:3">
+    <row r="19" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A19" s="56" t="s">
         <v>59</v>
       </c>
@@ -3557,7 +3562,7 @@
         <v>104</v>
       </c>
     </row>
-    <row r="20" spans="1:3">
+    <row r="20" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A20" s="49" t="s">
         <v>60</v>
       </c>
@@ -3569,7 +3574,7 @@
         <v>105</v>
       </c>
     </row>
-    <row r="21" spans="1:3">
+    <row r="21" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A21" s="52" t="s">
         <v>43</v>
       </c>
@@ -3581,7 +3586,7 @@
         <v>106</v>
       </c>
     </row>
-    <row r="22" spans="1:3">
+    <row r="22" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A22" s="52" t="s">
         <v>146</v>
       </c>
@@ -3593,7 +3598,7 @@
         <v>151</v>
       </c>
     </row>
-    <row r="23" spans="1:3">
+    <row r="23" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A23" s="52" t="s">
         <v>44</v>
       </c>
@@ -3605,7 +3610,7 @@
         <v>152</v>
       </c>
     </row>
-    <row r="24" spans="1:3">
+    <row r="24" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A24" s="93" t="s">
         <v>147</v>
       </c>
@@ -3617,7 +3622,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="25" spans="1:3" ht="15" thickBot="1">
+    <row r="25" spans="1:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A25" s="85" t="s">
         <v>101</v>
       </c>
@@ -3628,14 +3633,14 @@
         <v>8</v>
       </c>
     </row>
-    <row r="26" spans="1:3" ht="15" thickTop="1"/>
-    <row r="28" spans="1:3" ht="18">
+    <row r="26" spans="1:3" ht="15.75" thickTop="1" x14ac:dyDescent="0.25"/>
+    <row r="28" spans="1:3" ht="18.75" x14ac:dyDescent="0.3">
       <c r="A28" s="2" t="s">
         <v>9</v>
       </c>
     </row>
-    <row r="29" spans="1:3" ht="15" thickBot="1"/>
-    <row r="30" spans="1:3" ht="15.6" thickTop="1" thickBot="1">
+    <row r="29" spans="1:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
+    <row r="30" spans="1:3" ht="16.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A30" s="3" t="s">
         <v>0</v>
       </c>
@@ -3646,7 +3651,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="31" spans="1:3" ht="15" thickTop="1">
+    <row r="31" spans="1:3" ht="15.75" thickTop="1" x14ac:dyDescent="0.25">
       <c r="A31" s="4" t="s">
         <v>10</v>
       </c>
@@ -3657,7 +3662,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="32" spans="1:3">
+    <row r="32" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A32" s="95" t="s">
         <v>148</v>
       </c>
@@ -3669,7 +3674,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="33" spans="1:11">
+    <row r="33" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A33" s="15" t="s">
         <v>11</v>
       </c>
@@ -3681,7 +3686,7 @@
         <v>150</v>
       </c>
     </row>
-    <row r="34" spans="1:11">
+    <row r="34" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A34" s="27" t="s">
         <v>149</v>
       </c>
@@ -3693,7 +3698,7 @@
         <v>107</v>
       </c>
     </row>
-    <row r="35" spans="1:11" ht="15" thickBot="1">
+    <row r="35" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A35" s="10" t="s">
         <v>12</v>
       </c>
@@ -3704,14 +3709,14 @@
         <v>107</v>
       </c>
     </row>
-    <row r="36" spans="1:11" ht="15" thickTop="1"/>
-    <row r="38" spans="1:11" ht="18">
+    <row r="36" spans="1:11" ht="15.75" thickTop="1" x14ac:dyDescent="0.25"/>
+    <row r="38" spans="1:11" ht="18.75" x14ac:dyDescent="0.3">
       <c r="A38" s="2" t="s">
         <v>13</v>
       </c>
     </row>
-    <row r="39" spans="1:11" ht="15" thickBot="1"/>
-    <row r="40" spans="1:11" ht="15.6" thickTop="1" thickBot="1">
+    <row r="39" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
+    <row r="40" spans="1:11" ht="16.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A40" s="3" t="s">
         <v>0</v>
       </c>
@@ -3746,7 +3751,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="41" spans="1:11" ht="15" thickTop="1">
+    <row r="41" spans="1:11" ht="15.75" thickTop="1" x14ac:dyDescent="0.25">
       <c r="A41" s="4" t="s">
         <v>14</v>
       </c>
@@ -3781,7 +3786,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="42" spans="1:11">
+    <row r="42" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A42" s="44" t="s">
         <v>39</v>
       </c>
@@ -3816,7 +3821,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="43" spans="1:11">
+    <row r="43" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A43" s="7" t="s">
         <v>15</v>
       </c>
@@ -3852,7 +3857,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="44" spans="1:11">
+    <row r="44" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A44" s="7" t="s">
         <v>16</v>
       </c>
@@ -3892,7 +3897,7 @@
         <v>108</v>
       </c>
     </row>
-    <row r="45" spans="1:11">
+    <row r="45" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A45" s="7" t="s">
         <v>17</v>
       </c>
@@ -3932,7 +3937,7 @@
         <v>109</v>
       </c>
     </row>
-    <row r="46" spans="1:11">
+    <row r="46" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A46" s="38" t="s">
         <v>46</v>
       </c>
@@ -3972,7 +3977,7 @@
         <v>110</v>
       </c>
     </row>
-    <row r="47" spans="1:11">
+    <row r="47" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A47" s="38" t="s">
         <v>45</v>
       </c>
@@ -4012,7 +4017,7 @@
         <v>111</v>
       </c>
     </row>
-    <row r="48" spans="1:11">
+    <row r="48" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A48" s="7" t="s">
         <v>18</v>
       </c>
@@ -4042,7 +4047,7 @@
       </c>
       <c r="K48" s="23"/>
     </row>
-    <row r="49" spans="1:14">
+    <row r="49" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A49" s="7" t="s">
         <v>48</v>
       </c>
@@ -4082,7 +4087,7 @@
         <v>112</v>
       </c>
     </row>
-    <row r="50" spans="1:14">
+    <row r="50" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A50" s="7" t="s">
         <v>153</v>
       </c>
@@ -4122,7 +4127,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="51" spans="1:14">
+    <row r="51" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A51" s="7" t="s">
         <v>47</v>
       </c>
@@ -4162,7 +4167,7 @@
         <v>113</v>
       </c>
     </row>
-    <row r="52" spans="1:14">
+    <row r="52" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A52" s="27" t="s">
         <v>49</v>
       </c>
@@ -4202,7 +4207,7 @@
         <v>114</v>
       </c>
     </row>
-    <row r="53" spans="1:14">
+    <row r="53" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A53" s="27" t="s">
         <v>51</v>
       </c>
@@ -4242,7 +4247,7 @@
         <v>115</v>
       </c>
     </row>
-    <row r="54" spans="1:14">
+    <row r="54" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A54" s="27" t="s">
         <v>50</v>
       </c>
@@ -4282,7 +4287,7 @@
         <v>116</v>
       </c>
     </row>
-    <row r="55" spans="1:14">
+    <row r="55" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A55" s="7" t="s">
         <v>52</v>
       </c>
@@ -4317,7 +4322,7 @@
         <v>117</v>
       </c>
     </row>
-    <row r="56" spans="1:14">
+    <row r="56" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A56" s="27" t="s">
         <v>53</v>
       </c>
@@ -4361,7 +4366,7 @@
         <v>156</v>
       </c>
     </row>
-    <row r="57" spans="1:14" ht="15" thickBot="1">
+    <row r="57" spans="1:14" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A57" s="10" t="s">
         <v>54</v>
       </c>
@@ -4401,20 +4406,20 @@
         <v>119</v>
       </c>
     </row>
-    <row r="58" spans="1:14" ht="15" thickTop="1">
+    <row r="58" spans="1:14" ht="15.75" thickTop="1" x14ac:dyDescent="0.25">
       <c r="B58" s="32"/>
       <c r="C58" s="33"/>
     </row>
-    <row r="59" spans="1:14">
+    <row r="59" spans="1:14" x14ac:dyDescent="0.25">
       <c r="B59" s="32"/>
       <c r="C59" s="33"/>
     </row>
-    <row r="60" spans="1:14" ht="18">
+    <row r="60" spans="1:14" ht="18.75" x14ac:dyDescent="0.3">
       <c r="A60" s="2" t="s">
         <v>19</v>
       </c>
     </row>
-    <row r="62" spans="1:14" ht="15" thickBot="1">
+    <row r="62" spans="1:14" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A62" s="113" t="s">
         <v>0</v>
       </c>
@@ -4447,7 +4452,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="63" spans="1:14" ht="15" thickTop="1">
+    <row r="63" spans="1:14" ht="15.75" thickTop="1" x14ac:dyDescent="0.25">
       <c r="A63" s="7" t="s">
         <v>16</v>
       </c>
@@ -4487,7 +4492,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="64" spans="1:14">
+    <row r="64" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A64" s="7" t="s">
         <v>17</v>
       </c>
@@ -4517,7 +4522,7 @@
       </c>
       <c r="K64" s="23"/>
     </row>
-    <row r="65" spans="1:12">
+    <row r="65" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A65" s="38" t="s">
         <v>158</v>
       </c>
@@ -4552,7 +4557,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="66" spans="1:12">
+    <row r="66" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A66" s="38" t="s">
         <v>159</v>
       </c>
@@ -4587,7 +4592,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="67" spans="1:12">
+    <row r="67" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A67" s="7" t="s">
         <v>18</v>
       </c>
@@ -4612,7 +4617,7 @@
       </c>
       <c r="K67" s="23"/>
     </row>
-    <row r="68" spans="1:12">
+    <row r="68" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A68" s="38" t="s">
         <v>45</v>
       </c>
@@ -4652,7 +4657,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="69" spans="1:12">
+    <row r="69" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A69" s="7" t="s">
         <v>48</v>
       </c>
@@ -4687,7 +4692,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="70" spans="1:12">
+    <row r="70" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A70" s="7" t="s">
         <v>47</v>
       </c>
@@ -4723,7 +4728,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="71" spans="1:12">
+    <row r="71" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A71" s="27" t="s">
         <v>49</v>
       </c>
@@ -4758,7 +4763,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="72" spans="1:12">
+    <row r="72" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A72" s="27" t="s">
         <v>51</v>
       </c>
@@ -4793,7 +4798,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="73" spans="1:12">
+    <row r="73" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A73" s="27" t="s">
         <v>50</v>
       </c>
@@ -4829,7 +4834,7 @@
       </c>
       <c r="L73" s="106"/>
     </row>
-    <row r="74" spans="1:12">
+    <row r="74" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A74" s="7" t="s">
         <v>52</v>
       </c>
@@ -4864,7 +4869,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="75" spans="1:12">
+    <row r="75" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A75" s="27" t="s">
         <v>53</v>
       </c>
@@ -4899,7 +4904,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="76" spans="1:12" ht="15" thickBot="1">
+    <row r="76" spans="1:12" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A76" s="115" t="s">
         <v>54</v>
       </c>
@@ -4935,14 +4940,14 @@
         <v>160</v>
       </c>
     </row>
-    <row r="77" spans="1:12" ht="15" thickTop="1"/>
-    <row r="79" spans="1:12" ht="18">
+    <row r="77" spans="1:12" ht="15.75" thickTop="1" x14ac:dyDescent="0.25"/>
+    <row r="79" spans="1:12" ht="18.75" x14ac:dyDescent="0.3">
       <c r="A79" s="2" t="s">
         <v>22</v>
       </c>
     </row>
-    <row r="80" spans="1:12" ht="15" thickBot="1"/>
-    <row r="81" spans="1:3" ht="15.6" thickTop="1" thickBot="1">
+    <row r="80" spans="1:12" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
+    <row r="81" spans="1:3" ht="16.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A81" s="3" t="s">
         <v>0</v>
       </c>
@@ -4953,7 +4958,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="82" spans="1:3" ht="15" thickTop="1">
+    <row r="82" spans="1:3" ht="15.75" thickTop="1" x14ac:dyDescent="0.25">
       <c r="A82" s="4" t="s">
         <v>122</v>
       </c>
@@ -4964,7 +4969,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="83" spans="1:3">
+    <row r="83" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A83" s="15" t="s">
         <v>123</v>
       </c>
@@ -4975,7 +4980,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="84" spans="1:3">
+    <row r="84" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A84" s="15" t="s">
         <v>23</v>
       </c>
@@ -4986,7 +4991,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="85" spans="1:3" ht="15.6">
+    <row r="85" spans="1:3" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A85" s="52" t="s">
         <v>128</v>
       </c>
@@ -4997,7 +5002,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="86" spans="1:3">
+    <row r="86" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A86" s="52" t="s">
         <v>127</v>
       </c>
@@ -5008,7 +5013,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="87" spans="1:3">
+    <row r="87" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A87" s="52" t="s">
         <v>126</v>
       </c>
@@ -5019,7 +5024,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="88" spans="1:3">
+    <row r="88" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A88" s="52" t="s">
         <v>125</v>
       </c>
@@ -5030,7 +5035,7 @@
         <v>132</v>
       </c>
     </row>
-    <row r="89" spans="1:3">
+    <row r="89" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A89" s="52" t="s">
         <v>129</v>
       </c>
@@ -5041,7 +5046,7 @@
         <v>190</v>
       </c>
     </row>
-    <row r="90" spans="1:3">
+    <row r="90" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A90" s="52" t="s">
         <v>130</v>
       </c>
@@ -5052,7 +5057,7 @@
         <v>191</v>
       </c>
     </row>
-    <row r="91" spans="1:3">
+    <row r="91" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A91" s="52" t="s">
         <v>131</v>
       </c>
@@ -5063,7 +5068,7 @@
         <v>133</v>
       </c>
     </row>
-    <row r="92" spans="1:3">
+    <row r="92" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A92" s="52" t="s">
         <v>27</v>
       </c>
@@ -5074,7 +5079,7 @@
         <v>134</v>
       </c>
     </row>
-    <row r="93" spans="1:3">
+    <row r="93" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A93" s="52" t="s">
         <v>28</v>
       </c>
@@ -5085,7 +5090,7 @@
         <v>135</v>
       </c>
     </row>
-    <row r="94" spans="1:3">
+    <row r="94" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A94" s="52" t="s">
         <v>124</v>
       </c>
@@ -5096,7 +5101,7 @@
         <v>136</v>
       </c>
     </row>
-    <row r="95" spans="1:3">
+    <row r="95" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A95" s="15" t="s">
         <v>120</v>
       </c>
@@ -5107,7 +5112,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="96" spans="1:3">
+    <row r="96" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A96" s="15" t="s">
         <v>121</v>
       </c>
@@ -5118,7 +5123,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="97" spans="1:11">
+    <row r="97" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A97" s="52" t="s">
         <v>163</v>
       </c>
@@ -5129,7 +5134,7 @@
         <v>162</v>
       </c>
     </row>
-    <row r="98" spans="1:11">
+    <row r="98" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A98" s="15" t="s">
         <v>30</v>
       </c>
@@ -5138,7 +5143,7 @@
       </c>
       <c r="C98" s="18"/>
     </row>
-    <row r="99" spans="1:11" ht="15" thickBot="1">
+    <row r="99" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A99" s="10" t="s">
         <v>31</v>
       </c>
@@ -5147,14 +5152,14 @@
       </c>
       <c r="C99" s="19"/>
     </row>
-    <row r="100" spans="1:11" ht="15" thickTop="1"/>
-    <row r="102" spans="1:11" ht="18">
+    <row r="100" spans="1:11" ht="15.75" thickTop="1" x14ac:dyDescent="0.25"/>
+    <row r="102" spans="1:11" ht="18.75" x14ac:dyDescent="0.3">
       <c r="A102" s="2" t="s">
         <v>32</v>
       </c>
     </row>
-    <row r="103" spans="1:11" ht="15" thickBot="1"/>
-    <row r="104" spans="1:11" ht="15.6" thickTop="1" thickBot="1">
+    <row r="103" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
+    <row r="104" spans="1:11" ht="16.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A104" s="3" t="s">
         <v>0</v>
       </c>
@@ -5185,7 +5190,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="105" spans="1:11" ht="15" thickTop="1">
+    <row r="105" spans="1:11" ht="15.75" thickTop="1" x14ac:dyDescent="0.25">
       <c r="A105" s="7" t="s">
         <v>16</v>
       </c>
@@ -5224,7 +5229,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="106" spans="1:11">
+    <row r="106" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A106" s="7" t="s">
         <v>33</v>
       </c>
@@ -5259,7 +5264,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="107" spans="1:11">
+    <row r="107" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A107" s="38" t="s">
         <v>161</v>
       </c>
@@ -5294,7 +5299,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="108" spans="1:11" ht="15" thickBot="1">
+    <row r="108" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A108" s="10" t="s">
         <v>34</v>
       </c>
@@ -5329,14 +5334,14 @@
         <v>35</v>
       </c>
     </row>
-    <row r="109" spans="1:11" ht="15" thickTop="1"/>
-    <row r="111" spans="1:11" ht="18">
+    <row r="109" spans="1:11" ht="15.75" thickTop="1" x14ac:dyDescent="0.25"/>
+    <row r="111" spans="1:11" ht="18.75" x14ac:dyDescent="0.3">
       <c r="A111" s="2" t="s">
         <v>164</v>
       </c>
     </row>
-    <row r="112" spans="1:11" ht="15" thickBot="1"/>
-    <row r="113" spans="1:8" ht="15.6" thickTop="1" thickBot="1">
+    <row r="112" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
+    <row r="113" spans="1:8" ht="16.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A113" s="3" t="s">
         <v>0</v>
       </c>
@@ -5356,7 +5361,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="114" spans="1:8" ht="15" thickTop="1">
+    <row r="114" spans="1:8" ht="15.75" thickTop="1" x14ac:dyDescent="0.25">
       <c r="A114" s="38" t="s">
         <v>165</v>
       </c>
@@ -5376,7 +5381,7 @@
         <v>184</v>
       </c>
     </row>
-    <row r="115" spans="1:8">
+    <row r="115" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A115" s="38" t="s">
         <v>172</v>
       </c>
@@ -5396,7 +5401,7 @@
         <v>184</v>
       </c>
     </row>
-    <row r="116" spans="1:8">
+    <row r="116" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A116" s="38" t="s">
         <v>178</v>
       </c>
@@ -5416,7 +5421,7 @@
         <v>183</v>
       </c>
     </row>
-    <row r="117" spans="1:8" ht="15" thickBot="1">
+    <row r="117" spans="1:8" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A117" s="85" t="s">
         <v>170</v>
       </c>
@@ -5436,7 +5441,7 @@
         <v>177</v>
       </c>
     </row>
-    <row r="118" spans="1:8" ht="15.6" thickTop="1" thickBot="1">
+    <row r="118" spans="1:8" ht="16.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A118" s="85" t="s">
         <v>185</v>
       </c>
@@ -5456,13 +5461,13 @@
         <v>188</v>
       </c>
     </row>
-    <row r="119" spans="1:8" ht="15" thickTop="1"/>
-    <row r="120" spans="1:8">
+    <row r="119" spans="1:8" ht="15.75" thickTop="1" x14ac:dyDescent="0.25"/>
+    <row r="120" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A120" s="129" t="s">
         <v>212</v>
       </c>
     </row>
-    <row r="121" spans="1:8">
+    <row r="121" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A121" s="130" t="s">
         <v>206</v>
       </c>
@@ -5470,12 +5475,12 @@
         <v>203</v>
       </c>
     </row>
-    <row r="122" spans="1:8">
+    <row r="122" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A122" s="130" t="s">
         <v>205</v>
       </c>
     </row>
-    <row r="123" spans="1:8">
+    <row r="123" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A123" s="130" t="s">
         <v>207</v>
       </c>
@@ -5483,7 +5488,7 @@
         <v>204</v>
       </c>
     </row>
-    <row r="124" spans="1:8">
+    <row r="124" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A124" s="130" t="s">
         <v>219</v>
       </c>
@@ -5491,12 +5496,12 @@
         <v>208</v>
       </c>
     </row>
-    <row r="125" spans="1:8">
+    <row r="125" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A125" s="129" t="s">
         <v>213</v>
       </c>
     </row>
-    <row r="126" spans="1:8">
+    <row r="126" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A126" s="130" t="s">
         <v>209</v>
       </c>
@@ -5504,12 +5509,12 @@
         <v>211</v>
       </c>
     </row>
-    <row r="127" spans="1:8">
+    <row r="127" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A127" s="130" t="s">
         <v>210</v>
       </c>
     </row>
-    <row r="128" spans="1:8">
+    <row r="128" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A128" s="130" t="s">
         <v>214</v>
       </c>
@@ -5517,7 +5522,7 @@
         <v>215</v>
       </c>
     </row>
-    <row r="129" spans="1:2">
+    <row r="129" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A129" s="130" t="s">
         <v>216</v>
       </c>
@@ -5536,24 +5541,24 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{3F74A05D-7210-44AC-859D-2846F0884F7B}">
   <dimension ref="A1:G56"/>
-  <sheetFormatPr defaultColWidth="12" defaultRowHeight="14.4"/>
+  <sheetFormatPr defaultColWidth="12" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="24.44140625" customWidth="1"/>
-    <col min="2" max="9" width="12.88671875" customWidth="1"/>
+    <col min="1" max="1" width="24.42578125" customWidth="1"/>
+    <col min="2" max="9" width="12.85546875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5" ht="21">
+    <row r="1" spans="1:5" ht="21" x14ac:dyDescent="0.35">
       <c r="A1" s="1" t="s">
         <v>90</v>
       </c>
     </row>
-    <row r="3" spans="1:5" ht="18">
+    <row r="3" spans="1:5" ht="18.75" x14ac:dyDescent="0.3">
       <c r="A3" s="2" t="s">
         <v>61</v>
       </c>
     </row>
-    <row r="4" spans="1:5" ht="15" thickBot="1"/>
-    <row r="5" spans="1:5" ht="15.6" thickTop="1" thickBot="1">
+    <row r="4" spans="1:5" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
+    <row r="5" spans="1:5" ht="16.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A5" s="3" t="s">
         <v>0</v>
       </c>
@@ -5565,7 +5570,7 @@
       </c>
       <c r="E5" s="73"/>
     </row>
-    <row r="6" spans="1:5" ht="15" thickTop="1">
+    <row r="6" spans="1:5" ht="15.75" thickTop="1" x14ac:dyDescent="0.25">
       <c r="A6" s="37" t="s">
         <v>101</v>
       </c>
@@ -5577,7 +5582,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="7" spans="1:5">
+    <row r="7" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A7" s="38" t="s">
         <v>92</v>
       </c>
@@ -5589,7 +5594,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="8" spans="1:5">
+    <row r="8" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A8" s="38" t="s">
         <v>93</v>
       </c>
@@ -5601,7 +5606,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="9" spans="1:5">
+    <row r="9" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A9" s="38" t="s">
         <v>91</v>
       </c>
@@ -5613,7 +5618,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="10" spans="1:5">
+    <row r="10" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A10" s="7" t="s">
         <v>62</v>
       </c>
@@ -5624,7 +5629,7 @@
         <v>63</v>
       </c>
     </row>
-    <row r="11" spans="1:5" ht="15" thickBot="1">
+    <row r="11" spans="1:5" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A11" s="10" t="s">
         <v>5</v>
       </c>
@@ -5636,18 +5641,18 @@
         <v>6</v>
       </c>
     </row>
-    <row r="12" spans="1:5" ht="16.2" thickTop="1">
+    <row r="12" spans="1:5" ht="16.5" thickTop="1" x14ac:dyDescent="0.25">
       <c r="A12" s="13"/>
     </row>
-    <row r="14" spans="1:5" ht="18">
+    <row r="14" spans="1:5" ht="18.75" x14ac:dyDescent="0.3">
       <c r="A14" s="2" t="s">
         <v>64</v>
       </c>
     </row>
-    <row r="15" spans="1:5" ht="18.600000000000001" thickBot="1">
+    <row r="15" spans="1:5" ht="19.5" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A15" s="2"/>
     </row>
-    <row r="16" spans="1:5" ht="15.6" thickTop="1" thickBot="1">
+    <row r="16" spans="1:5" ht="16.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A16" s="3" t="s">
         <v>0</v>
       </c>
@@ -5658,7 +5663,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="17" spans="1:3" ht="15" thickTop="1">
+    <row r="17" spans="1:3" ht="15.75" thickTop="1" x14ac:dyDescent="0.25">
       <c r="A17" s="59" t="s">
         <v>65</v>
       </c>
@@ -5667,7 +5672,7 @@
       </c>
       <c r="C17" s="61"/>
     </row>
-    <row r="18" spans="1:3">
+    <row r="18" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A18" s="62" t="s">
         <v>67</v>
       </c>
@@ -5676,7 +5681,7 @@
       </c>
       <c r="C18" s="64"/>
     </row>
-    <row r="19" spans="1:3">
+    <row r="19" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A19" s="62" t="s">
         <v>69</v>
       </c>
@@ -5687,7 +5692,7 @@
         <v>70</v>
       </c>
     </row>
-    <row r="20" spans="1:3">
+    <row r="20" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A20" s="62" t="s">
         <v>71</v>
       </c>
@@ -5698,7 +5703,7 @@
         <v>72</v>
       </c>
     </row>
-    <row r="21" spans="1:3">
+    <row r="21" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A21" s="62" t="s">
         <v>73</v>
       </c>
@@ -5709,7 +5714,7 @@
         <v>74</v>
       </c>
     </row>
-    <row r="22" spans="1:3">
+    <row r="22" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A22" s="62" t="s">
         <v>75</v>
       </c>
@@ -5720,7 +5725,7 @@
         <v>70</v>
       </c>
     </row>
-    <row r="23" spans="1:3">
+    <row r="23" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A23" s="62" t="s">
         <v>76</v>
       </c>
@@ -5731,7 +5736,7 @@
         <v>72</v>
       </c>
     </row>
-    <row r="24" spans="1:3">
+    <row r="24" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A24" s="62" t="s">
         <v>77</v>
       </c>
@@ -5743,7 +5748,7 @@
         <v>78</v>
       </c>
     </row>
-    <row r="25" spans="1:3">
+    <row r="25" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A25" s="62" t="s">
         <v>79</v>
       </c>
@@ -5755,7 +5760,7 @@
         <v>80</v>
       </c>
     </row>
-    <row r="26" spans="1:3">
+    <row r="26" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A26" s="67" t="s">
         <v>81</v>
       </c>
@@ -5763,7 +5768,7 @@
         <v>1510</v>
       </c>
     </row>
-    <row r="27" spans="1:3" ht="15" thickBot="1">
+    <row r="27" spans="1:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A27" s="68" t="s">
         <v>82</v>
       </c>
@@ -5772,14 +5777,14 @@
       </c>
       <c r="C27" s="70"/>
     </row>
-    <row r="28" spans="1:3" ht="15" thickTop="1"/>
-    <row r="30" spans="1:3" ht="18">
+    <row r="28" spans="1:3" ht="15.75" thickTop="1" x14ac:dyDescent="0.25"/>
+    <row r="30" spans="1:3" ht="18.75" x14ac:dyDescent="0.3">
       <c r="A30" s="2" t="s">
         <v>83</v>
       </c>
     </row>
-    <row r="31" spans="1:3" ht="15" thickBot="1"/>
-    <row r="32" spans="1:3" ht="15.6" thickTop="1" thickBot="1">
+    <row r="31" spans="1:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
+    <row r="32" spans="1:3" ht="16.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A32" s="3" t="s">
         <v>0</v>
       </c>
@@ -5790,7 +5795,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="33" spans="1:7" ht="15" thickTop="1">
+    <row r="33" spans="1:7" ht="15.75" thickTop="1" x14ac:dyDescent="0.25">
       <c r="A33" s="59" t="s">
         <v>84</v>
       </c>
@@ -5802,7 +5807,7 @@
       </c>
       <c r="G33" s="73"/>
     </row>
-    <row r="34" spans="1:7">
+    <row r="34" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A34" s="74" t="s">
         <v>194</v>
       </c>
@@ -5815,7 +5820,7 @@
       </c>
       <c r="G34" s="73"/>
     </row>
-    <row r="35" spans="1:7">
+    <row r="35" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A35" s="74" t="s">
         <v>85</v>
       </c>
@@ -5829,7 +5834,7 @@
       <c r="F35" s="78"/>
       <c r="G35" s="73"/>
     </row>
-    <row r="36" spans="1:7" ht="15.6">
+    <row r="36" spans="1:7" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A36" s="74" t="s">
         <v>86</v>
       </c>
@@ -5842,7 +5847,7 @@
       <c r="F36" s="13"/>
       <c r="G36" s="13"/>
     </row>
-    <row r="37" spans="1:7">
+    <row r="37" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A37" s="74" t="s">
         <v>87</v>
       </c>
@@ -5854,7 +5859,7 @@
         <v>141</v>
       </c>
     </row>
-    <row r="38" spans="1:7">
+    <row r="38" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A38" s="81" t="s">
         <v>95</v>
       </c>
@@ -5865,7 +5870,7 @@
         <v>72</v>
       </c>
     </row>
-    <row r="39" spans="1:7">
+    <row r="39" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A39" s="81" t="s">
         <v>94</v>
       </c>
@@ -5877,7 +5882,7 @@
         <v>142</v>
       </c>
     </row>
-    <row r="40" spans="1:7">
+    <row r="40" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A40" s="81" t="s">
         <v>193</v>
       </c>
@@ -5886,7 +5891,7 @@
       </c>
       <c r="C40" s="76"/>
     </row>
-    <row r="41" spans="1:7">
+    <row r="41" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A41" s="81" t="s">
         <v>96</v>
       </c>
@@ -5898,7 +5903,7 @@
         <v>143</v>
       </c>
     </row>
-    <row r="42" spans="1:7" ht="15" thickBot="1">
+    <row r="42" spans="1:7" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A42" s="83" t="s">
         <v>88</v>
       </c>
@@ -5910,7 +5915,7 @@
         <v>144</v>
       </c>
     </row>
-    <row r="43" spans="1:7" ht="15" thickTop="1">
+    <row r="43" spans="1:7" ht="15.75" thickTop="1" x14ac:dyDescent="0.25">
       <c r="A43" s="125" t="s">
         <v>197</v>
       </c>
@@ -5922,7 +5927,7 @@
         <v>198</v>
       </c>
     </row>
-    <row r="44" spans="1:7">
+    <row r="44" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A44" s="125" t="s">
         <v>195</v>
       </c>
@@ -5934,7 +5939,7 @@
         <v>199</v>
       </c>
     </row>
-    <row r="45" spans="1:7">
+    <row r="45" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A45" s="125" t="s">
         <v>196</v>
       </c>
@@ -5946,7 +5951,7 @@
         <v>200</v>
       </c>
     </row>
-    <row r="46" spans="1:7">
+    <row r="46" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A46" s="74" t="s">
         <v>192</v>
       </c>
@@ -5958,7 +5963,7 @@
         <v>201</v>
       </c>
     </row>
-    <row r="47" spans="1:7">
+    <row r="47" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A47" s="128" t="s">
         <v>202</v>
       </c>
@@ -5970,13 +5975,13 @@
         <v>70</v>
       </c>
     </row>
-    <row r="49" spans="1:3" ht="18">
+    <row r="49" spans="1:3" ht="18.75" x14ac:dyDescent="0.3">
       <c r="A49" s="2" t="s">
         <v>97</v>
       </c>
     </row>
-    <row r="50" spans="1:3" ht="15" thickBot="1"/>
-    <row r="51" spans="1:3" ht="15.6" thickTop="1" thickBot="1">
+    <row r="50" spans="1:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
+    <row r="51" spans="1:3" ht="16.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A51" s="3" t="s">
         <v>0</v>
       </c>
@@ -5987,7 +5992,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="52" spans="1:3" ht="15" thickTop="1">
+    <row r="52" spans="1:3" ht="15.75" thickTop="1" x14ac:dyDescent="0.25">
       <c r="A52" s="81" t="s">
         <v>98</v>
       </c>
@@ -5998,7 +6003,7 @@
         <v>89</v>
       </c>
     </row>
-    <row r="53" spans="1:3">
+    <row r="53" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A53" s="74" t="s">
         <v>85</v>
       </c>
@@ -6010,7 +6015,7 @@
         <v>63</v>
       </c>
     </row>
-    <row r="54" spans="1:3">
+    <row r="54" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A54" s="81" t="s">
         <v>145</v>
       </c>
@@ -6021,7 +6026,7 @@
         <v>100</v>
       </c>
     </row>
-    <row r="55" spans="1:3" ht="15" thickBot="1">
+    <row r="55" spans="1:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A55" s="82" t="s">
         <v>99</v>
       </c>
@@ -6032,7 +6037,7 @@
         <v>100</v>
       </c>
     </row>
-    <row r="56" spans="1:3" ht="15" thickTop="1"/>
+    <row r="56" spans="1:3" ht="15.75" thickTop="1" x14ac:dyDescent="0.25"/>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
@@ -6042,9 +6047,9 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{86BA37C4-8F32-417F-A8E4-D80C296F90D3}">
   <dimension ref="A2:AD84"/>
-  <sheetFormatPr defaultRowHeight="14.4"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData>
-    <row r="2" spans="2:25">
+    <row r="2" spans="2:25" x14ac:dyDescent="0.25">
       <c r="B2" s="136" t="s">
         <v>220</v>
       </c>
@@ -6052,7 +6057,7 @@
       <c r="D2" s="136"/>
       <c r="E2" s="136"/>
     </row>
-    <row r="3" spans="2:25">
+    <row r="3" spans="2:25" x14ac:dyDescent="0.25">
       <c r="B3" t="s">
         <v>221</v>
       </c>
@@ -6066,7 +6071,7 @@
         <v>224</v>
       </c>
     </row>
-    <row r="4" spans="2:25">
+    <row r="4" spans="2:25" x14ac:dyDescent="0.25">
       <c r="B4">
         <v>5</v>
       </c>
@@ -6086,7 +6091,7 @@
         <v>227</v>
       </c>
     </row>
-    <row r="5" spans="2:25">
+    <row r="5" spans="2:25" x14ac:dyDescent="0.25">
       <c r="B5">
         <v>10</v>
       </c>
@@ -6106,7 +6111,7 @@
         <v>229</v>
       </c>
     </row>
-    <row r="6" spans="2:25">
+    <row r="6" spans="2:25" x14ac:dyDescent="0.25">
       <c r="B6">
         <v>15</v>
       </c>
@@ -6123,7 +6128,7 @@
         <v>231</v>
       </c>
     </row>
-    <row r="7" spans="2:25">
+    <row r="7" spans="2:25" x14ac:dyDescent="0.25">
       <c r="B7">
         <v>20</v>
       </c>
@@ -6137,7 +6142,7 @@
         <v>232</v>
       </c>
     </row>
-    <row r="8" spans="2:25">
+    <row r="8" spans="2:25" x14ac:dyDescent="0.25">
       <c r="B8">
         <v>25</v>
       </c>
@@ -6151,7 +6156,7 @@
         <v>233</v>
       </c>
     </row>
-    <row r="9" spans="2:25">
+    <row r="9" spans="2:25" x14ac:dyDescent="0.25">
       <c r="B9">
         <v>30</v>
       </c>
@@ -6168,7 +6173,7 @@
         <v>235</v>
       </c>
     </row>
-    <row r="10" spans="2:25">
+    <row r="10" spans="2:25" x14ac:dyDescent="0.25">
       <c r="B10">
         <v>35</v>
       </c>
@@ -6185,7 +6190,7 @@
         <v>237</v>
       </c>
     </row>
-    <row r="11" spans="2:25">
+    <row r="11" spans="2:25" x14ac:dyDescent="0.25">
       <c r="B11">
         <v>40</v>
       </c>
@@ -6196,7 +6201,7 @@
         <v>39</v>
       </c>
     </row>
-    <row r="12" spans="2:25">
+    <row r="12" spans="2:25" x14ac:dyDescent="0.25">
       <c r="B12">
         <v>45</v>
       </c>
@@ -6207,7 +6212,7 @@
         <v>47</v>
       </c>
     </row>
-    <row r="13" spans="2:25">
+    <row r="13" spans="2:25" x14ac:dyDescent="0.25">
       <c r="B13">
         <v>50</v>
       </c>
@@ -6221,7 +6226,7 @@
         <v>225</v>
       </c>
     </row>
-    <row r="15" spans="2:25">
+    <row r="15" spans="2:25" x14ac:dyDescent="0.25">
       <c r="B15" s="132" t="s">
         <v>238</v>
       </c>
@@ -6263,7 +6268,7 @@
       <c r="X15" s="132"/>
       <c r="Y15" s="132"/>
     </row>
-    <row r="16" spans="2:25">
+    <row r="16" spans="2:25" x14ac:dyDescent="0.25">
       <c r="B16" s="133" t="s">
         <v>248</v>
       </c>
@@ -6325,7 +6330,7 @@
         <v>3.5</v>
       </c>
     </row>
-    <row r="17" spans="2:30">
+    <row r="17" spans="2:30" x14ac:dyDescent="0.25">
       <c r="B17" s="133" t="s">
         <v>249</v>
       </c>
@@ -6387,7 +6392,7 @@
         <v>0.3</v>
       </c>
     </row>
-    <row r="18" spans="2:30">
+    <row r="18" spans="2:30" x14ac:dyDescent="0.25">
       <c r="B18" s="133" t="s">
         <v>226</v>
       </c>
@@ -6449,7 +6454,7 @@
         <v>259</v>
       </c>
     </row>
-    <row r="22" spans="2:30">
+    <row r="22" spans="2:30" x14ac:dyDescent="0.25">
       <c r="B22" s="138" t="s">
         <v>260</v>
       </c>
@@ -6459,7 +6464,7 @@
       <c r="F22" s="138"/>
       <c r="G22" s="138"/>
     </row>
-    <row r="24" spans="2:30">
+    <row r="24" spans="2:30" x14ac:dyDescent="0.25">
       <c r="B24" s="138" t="s">
         <v>261</v>
       </c>
@@ -6497,7 +6502,7 @@
       <c r="AC24" s="138"/>
       <c r="AD24" s="138"/>
     </row>
-    <row r="25" spans="2:30">
+    <row r="25" spans="2:30" x14ac:dyDescent="0.25">
       <c r="B25" s="137" t="s">
         <v>248</v>
       </c>
@@ -6571,7 +6576,7 @@
         <v>3.5</v>
       </c>
     </row>
-    <row r="26" spans="2:30">
+    <row r="26" spans="2:30" x14ac:dyDescent="0.25">
       <c r="B26" s="137" t="s">
         <v>249</v>
       </c>
@@ -6645,7 +6650,7 @@
         <v>0.3</v>
       </c>
     </row>
-    <row r="27" spans="2:30">
+    <row r="27" spans="2:30" x14ac:dyDescent="0.25">
       <c r="B27" s="137" t="s">
         <v>226</v>
       </c>
@@ -6719,7 +6724,7 @@
         <v>4.55</v>
       </c>
     </row>
-    <row r="28" spans="2:30">
+    <row r="28" spans="2:30" x14ac:dyDescent="0.25">
       <c r="B28" s="141" t="s">
         <v>314</v>
       </c>
@@ -6811,7 +6816,7 @@
         <v>2.2749999999999999</v>
       </c>
     </row>
-    <row r="30" spans="2:30">
+    <row r="30" spans="2:30" x14ac:dyDescent="0.25">
       <c r="B30" s="142" t="s">
         <v>268</v>
       </c>
@@ -6833,7 +6838,7 @@
       <c r="X30" s="138"/>
       <c r="Y30" s="138"/>
     </row>
-    <row r="32" spans="2:30">
+    <row r="32" spans="2:30" x14ac:dyDescent="0.25">
       <c r="B32" s="142" t="s">
         <v>261</v>
       </c>
@@ -6848,7 +6853,7 @@
         <v>272</v>
       </c>
     </row>
-    <row r="33" spans="2:10">
+    <row r="33" spans="2:10" x14ac:dyDescent="0.25">
       <c r="B33" s="137" t="s">
         <v>248</v>
       </c>
@@ -6871,7 +6876,7 @@
         <v>269</v>
       </c>
     </row>
-    <row r="34" spans="2:10">
+    <row r="34" spans="2:10" x14ac:dyDescent="0.25">
       <c r="B34" s="162" t="s">
         <v>249</v>
       </c>
@@ -6894,7 +6899,7 @@
         <v>274</v>
       </c>
     </row>
-    <row r="35" spans="2:10">
+    <row r="35" spans="2:10" x14ac:dyDescent="0.25">
       <c r="B35" s="137" t="s">
         <v>226</v>
       </c>
@@ -6917,7 +6922,7 @@
         <v>273</v>
       </c>
     </row>
-    <row r="36" spans="2:10">
+    <row r="36" spans="2:10" x14ac:dyDescent="0.25">
       <c r="B36" s="162" t="s">
         <v>266</v>
       </c>
@@ -6941,7 +6946,7 @@
         <v>0.86</v>
       </c>
     </row>
-    <row r="37" spans="2:10">
+    <row r="37" spans="2:10" x14ac:dyDescent="0.25">
       <c r="B37" s="141" t="s">
         <v>267</v>
       </c>
@@ -6964,7 +6969,7 @@
         <v>270</v>
       </c>
     </row>
-    <row r="38" spans="2:10">
+    <row r="38" spans="2:10" x14ac:dyDescent="0.25">
       <c r="B38" s="141" t="s">
         <v>15</v>
       </c>
@@ -6987,7 +6992,7 @@
         <v>271</v>
       </c>
     </row>
-    <row r="39" spans="2:10">
+    <row r="39" spans="2:10" x14ac:dyDescent="0.25">
       <c r="B39" s="141" t="s">
         <v>276</v>
       </c>
@@ -7007,17 +7012,17 @@
         <v>2.56</v>
       </c>
     </row>
-    <row r="54" spans="1:22">
+    <row r="54" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A54" t="s">
         <v>299</v>
       </c>
     </row>
-    <row r="56" spans="1:22">
+    <row r="56" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A56" t="s">
         <v>298</v>
       </c>
     </row>
-    <row r="59" spans="1:22">
+    <row r="59" spans="1:22" x14ac:dyDescent="0.25">
       <c r="B59" s="149" t="s">
         <v>283</v>
       </c>
@@ -7039,7 +7044,7 @@
       <c r="U59" s="149"/>
       <c r="V59" s="149"/>
     </row>
-    <row r="61" spans="1:22">
+    <row r="61" spans="1:22" x14ac:dyDescent="0.25">
       <c r="B61" s="148" t="s">
         <v>261</v>
       </c>
@@ -7055,7 +7060,7 @@
       </c>
       <c r="K61" s="149"/>
     </row>
-    <row r="62" spans="1:22">
+    <row r="62" spans="1:22" x14ac:dyDescent="0.25">
       <c r="B62" s="150" t="s">
         <v>248</v>
       </c>
@@ -7081,7 +7086,7 @@
         <v>2.5</v>
       </c>
     </row>
-    <row r="63" spans="1:22">
+    <row r="63" spans="1:22" x14ac:dyDescent="0.25">
       <c r="B63" s="151" t="s">
         <v>249</v>
       </c>
@@ -7107,7 +7112,7 @@
         <v>0.5</v>
       </c>
     </row>
-    <row r="64" spans="1:22" ht="28.8">
+    <row r="64" spans="1:22" ht="30" x14ac:dyDescent="0.25">
       <c r="B64" s="158" t="s">
         <v>284</v>
       </c>
@@ -7133,7 +7138,7 @@
         <v>1.85</v>
       </c>
     </row>
-    <row r="65" spans="2:20" ht="57.6">
+    <row r="65" spans="2:20" ht="60" x14ac:dyDescent="0.25">
       <c r="B65" s="156" t="s">
         <v>285</v>
       </c>
@@ -7159,7 +7164,7 @@
         <v>0.42</v>
       </c>
     </row>
-    <row r="66" spans="2:20" ht="28.8">
+    <row r="66" spans="2:20" ht="30" x14ac:dyDescent="0.25">
       <c r="B66" s="159" t="s">
         <v>286</v>
       </c>
@@ -7185,7 +7190,7 @@
         <v>3.66</v>
       </c>
     </row>
-    <row r="67" spans="2:20" ht="57.6">
+    <row r="67" spans="2:20" ht="60" x14ac:dyDescent="0.25">
       <c r="B67" s="156" t="s">
         <v>287</v>
       </c>
@@ -7211,7 +7216,7 @@
         <v>2.99</v>
       </c>
     </row>
-    <row r="68" spans="2:20" ht="43.2">
+    <row r="68" spans="2:20" ht="45" x14ac:dyDescent="0.25">
       <c r="B68" s="161" t="s">
         <v>295</v>
       </c>
@@ -7235,7 +7240,7 @@
         <v>306</v>
       </c>
     </row>
-    <row r="69" spans="2:20" ht="43.2">
+    <row r="69" spans="2:20" ht="45" x14ac:dyDescent="0.25">
       <c r="B69" s="161" t="s">
         <v>294</v>
       </c>
@@ -7259,7 +7264,7 @@
         <v>307</v>
       </c>
     </row>
-    <row r="77" spans="2:20">
+    <row r="77" spans="2:20" x14ac:dyDescent="0.25">
       <c r="B77" s="146" t="s">
         <v>282</v>
       </c>
@@ -7274,7 +7279,7 @@
       <c r="S77" s="147"/>
       <c r="T77" s="147"/>
     </row>
-    <row r="79" spans="2:20">
+    <row r="79" spans="2:20" x14ac:dyDescent="0.25">
       <c r="B79" s="146" t="s">
         <v>281</v>
       </c>
@@ -7291,7 +7296,7 @@
       <c r="M79" s="147"/>
       <c r="N79" s="147"/>
     </row>
-    <row r="80" spans="2:20">
+    <row r="80" spans="2:20" x14ac:dyDescent="0.25">
       <c r="B80" s="147" t="s">
         <v>311</v>
       </c>
@@ -7308,7 +7313,7 @@
       <c r="M80" s="147"/>
       <c r="N80" s="147"/>
     </row>
-    <row r="81" spans="2:14">
+    <row r="81" spans="2:14" x14ac:dyDescent="0.25">
       <c r="B81" s="146" t="s">
         <v>312</v>
       </c>
@@ -7325,7 +7330,7 @@
       <c r="M81" s="147"/>
       <c r="N81" s="147"/>
     </row>
-    <row r="82" spans="2:14">
+    <row r="82" spans="2:14" x14ac:dyDescent="0.25">
       <c r="B82" s="147"/>
       <c r="C82" s="147"/>
       <c r="D82" s="147"/>
@@ -7340,7 +7345,7 @@
       <c r="M82" s="147"/>
       <c r="N82" s="147"/>
     </row>
-    <row r="83" spans="2:14">
+    <row r="83" spans="2:14" x14ac:dyDescent="0.25">
       <c r="B83" s="146" t="s">
         <v>309</v>
       </c>
@@ -7357,7 +7362,7 @@
       <c r="M83" s="147"/>
       <c r="N83" s="147"/>
     </row>
-    <row r="84" spans="2:14">
+    <row r="84" spans="2:14" x14ac:dyDescent="0.25">
       <c r="B84" s="147" t="s">
         <v>310</v>
       </c>
@@ -7383,14 +7388,15 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{6D3DD6BC-0BCA-4BA9-9C7E-A308795ECB28}">
-  <dimension ref="B4:R11"/>
-  <sheetFormatPr defaultRowHeight="14.4"/>
+  <dimension ref="B4:R12"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="2" max="2" width="11.33203125" customWidth="1"/>
-    <col min="7" max="7" width="12.109375" customWidth="1"/>
+    <col min="2" max="2" width="11.28515625" customWidth="1"/>
+    <col min="7" max="7" width="12.140625" customWidth="1"/>
+    <col min="15" max="15" width="11.28515625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="4" spans="2:18">
+    <row r="4" spans="2:18" x14ac:dyDescent="0.25">
       <c r="B4" s="142" t="s">
         <v>315</v>
       </c>
@@ -7400,7 +7406,7 @@
       </c>
       <c r="P4" s="138"/>
     </row>
-    <row r="5" spans="2:18">
+    <row r="5" spans="2:18" x14ac:dyDescent="0.25">
       <c r="B5" s="167" t="s">
         <v>316</v>
       </c>
@@ -7426,7 +7432,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="6" spans="2:18">
+    <row r="6" spans="2:18" x14ac:dyDescent="0.25">
       <c r="B6" s="137" t="s">
         <v>226</v>
       </c>
@@ -7452,39 +7458,39 @@
         <v>5.19</v>
       </c>
     </row>
-    <row r="7" spans="2:18">
-      <c r="B7" s="162" t="s">
+    <row r="7" spans="2:18" x14ac:dyDescent="0.25">
+      <c r="B7" s="170" t="s">
         <v>266</v>
       </c>
-      <c r="C7" s="165">
+      <c r="C7" s="171">
         <f>C9/C8</f>
         <v>0.63833075734157652</v>
       </c>
-      <c r="D7" s="165">
+      <c r="D7" s="171">
         <f>D9/D8</f>
         <v>0.78412698412698423</v>
       </c>
-      <c r="E7" s="165">
+      <c r="E7" s="171">
         <f>E9/E8</f>
         <v>0.89473684210526327</v>
       </c>
-      <c r="O7" s="162" t="s">
+      <c r="O7" s="170" t="s">
         <v>266</v>
       </c>
-      <c r="P7" s="165">
+      <c r="P7" s="171">
         <f>P9/P8</f>
         <v>0.76984126984126977</v>
       </c>
-      <c r="Q7" s="165">
+      <c r="Q7" s="171">
         <f>Q9/Q8</f>
         <v>0.8512110726643598</v>
       </c>
-      <c r="R7" s="165">
+      <c r="R7" s="171">
         <f>R9/R8</f>
         <v>0.90909090909090906</v>
       </c>
     </row>
-    <row r="8" spans="2:18">
+    <row r="8" spans="2:18" x14ac:dyDescent="0.25">
       <c r="B8" s="141" t="s">
         <v>267</v>
       </c>
@@ -7510,7 +7516,7 @@
         <v>0.55000000000000004</v>
       </c>
     </row>
-    <row r="9" spans="2:18">
+    <row r="9" spans="2:18" x14ac:dyDescent="0.25">
       <c r="B9" s="141" t="s">
         <v>15</v>
       </c>
@@ -7536,8 +7542,8 @@
         <v>0.5</v>
       </c>
     </row>
-    <row r="10" spans="2:18">
-      <c r="B10" s="167" t="s">
+    <row r="10" spans="2:18" x14ac:dyDescent="0.25">
+      <c r="B10" s="162" t="s">
         <v>318</v>
       </c>
       <c r="C10" s="168">
@@ -7549,7 +7555,7 @@
       <c r="E10" s="168">
         <v>51</v>
       </c>
-      <c r="O10" s="167" t="s">
+      <c r="O10" s="162" t="s">
         <v>318</v>
       </c>
       <c r="P10" s="168">
@@ -7562,8 +7568,8 @@
         <v>56</v>
       </c>
     </row>
-    <row r="11" spans="2:18">
-      <c r="B11" s="167" t="s">
+    <row r="11" spans="2:18" x14ac:dyDescent="0.25">
+      <c r="B11" s="162" t="s">
         <v>319</v>
       </c>
       <c r="C11" s="169">
@@ -7575,7 +7581,7 @@
       <c r="E11" s="169">
         <v>20.8</v>
       </c>
-      <c r="O11" s="167" t="s">
+      <c r="O11" s="162" t="s">
         <v>319</v>
       </c>
       <c r="P11" s="169">
@@ -7588,9 +7594,42 @@
         <v>15.5</v>
       </c>
     </row>
+    <row r="12" spans="2:18" x14ac:dyDescent="0.25">
+      <c r="B12" s="162" t="s">
+        <v>320</v>
+      </c>
+      <c r="C12" s="163">
+        <f>5-C6</f>
+        <v>0.20500000000000007</v>
+      </c>
+      <c r="D12" s="163">
+        <f t="shared" ref="D12:E12" si="0">5-D6</f>
+        <v>-0.16300000000000026</v>
+      </c>
+      <c r="E12" s="163">
+        <f t="shared" si="0"/>
+        <v>-0.19399999999999995</v>
+      </c>
+      <c r="O12" s="162" t="s">
+        <v>320</v>
+      </c>
+      <c r="P12" s="163">
+        <f>5-P6</f>
+        <v>-0.16300000000000026</v>
+      </c>
+      <c r="Q12" s="163">
+        <f t="shared" ref="Q12:R12" si="1">5-Q6</f>
+        <v>-0.16099999999999959</v>
+      </c>
+      <c r="R12" s="163">
+        <f t="shared" si="1"/>
+        <v>-0.19000000000000039</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <drawing r:id="rId1"/>
+  <pageSetup orientation="portrait" r:id="rId1"/>
+  <drawing r:id="rId2"/>
 </worksheet>
 </file>
 

</xml_diff>

<commit_message>
MATLAB generated signals for final test on Boost Converter updated
</commit_message>
<xml_diff>
--- a/Excel/Boost Converter Design Params.xlsx
+++ b/Excel/Boost Converter Design Params.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/bb665e811a262358/Documents/GitHub/311/Excel/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="15" documentId="13_ncr:1_{EC7F3BDD-F69B-4F14-99E6-6CA8FAEB6FD6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{1C893AFE-EEF7-4A68-BFC7-AB1589E47531}"/>
+  <xr:revisionPtr revIDLastSave="20" documentId="13_ncr:1_{EC7F3BDD-F69B-4F14-99E6-6CA8FAEB6FD6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{B73A1577-27E3-47D8-9225-D9042D2D34E1}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="3" xr2:uid="{0EA872C3-4804-43CB-9F0B-5F94DB7B4351}"/>
   </bookViews>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="649" uniqueCount="321">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="650" uniqueCount="322">
   <si>
     <t>Parameter</t>
   </si>
@@ -1000,6 +1000,9 @@
   </si>
   <si>
     <t>SS Error (V)</t>
+  </si>
+  <si>
+    <t>OVP x2</t>
   </si>
 </sst>
 </file>
@@ -1106,7 +1109,7 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="18">
+  <fills count="19">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -1205,6 +1208,12 @@
         <bgColor indexed="65"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="4" tint="0.39997558519241921"/>
+        <bgColor indexed="65"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="68">
     <border>
@@ -2152,7 +2161,7 @@
       <diagonal/>
     </border>
   </borders>
-  <cellStyleXfs count="15">
+  <cellStyleXfs count="16">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="1" applyNumberFormat="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="1" fillId="3" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
@@ -2168,8 +2177,9 @@
     <xf numFmtId="0" fontId="1" fillId="15" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="1" fillId="16" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="1" fillId="17" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="1" fillId="18" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="172">
+  <cellXfs count="173">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
@@ -2368,10 +2378,11 @@
     <xf numFmtId="0" fontId="9" fillId="8" borderId="66" xfId="5" applyFont="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="10" borderId="0" xfId="7" applyFont="1" applyBorder="1"/>
     <xf numFmtId="9" fontId="1" fillId="8" borderId="66" xfId="5" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="0" fontId="1" fillId="18" borderId="0" xfId="15"/>
+    <xf numFmtId="0" fontId="9" fillId="18" borderId="0" xfId="15" applyFont="1"/>
   </cellXfs>
-  <cellStyles count="15">
+  <cellStyles count="16">
     <cellStyle name="20% - Accent1" xfId="2" builtinId="30"/>
     <cellStyle name="20% - Accent5" xfId="12" builtinId="46"/>
     <cellStyle name="20% - Accent6" xfId="10" builtinId="50"/>
@@ -2379,6 +2390,7 @@
     <cellStyle name="40% - Accent2" xfId="7" builtinId="35"/>
     <cellStyle name="40% - Accent4" xfId="9" builtinId="43"/>
     <cellStyle name="40% - Accent5" xfId="13" builtinId="47"/>
+    <cellStyle name="60% - Accent1" xfId="15" builtinId="32"/>
     <cellStyle name="60% - Accent2" xfId="8" builtinId="36"/>
     <cellStyle name="60% - Accent5" xfId="14" builtinId="48"/>
     <cellStyle name="Calculation" xfId="4" builtinId="22"/>
@@ -3085,6 +3097,50 @@
     </xdr:pic>
     <xdr:clientData/>
   </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>1</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>42</xdr:row>
+      <xdr:rowOff>71437</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>5</xdr:col>
+      <xdr:colOff>523875</xdr:colOff>
+      <xdr:row>55</xdr:row>
+      <xdr:rowOff>139354</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="2" name="Picture 1">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{B35BFE60-7B0B-E169-734F-CBDE64C681E4}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId3"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="619125" y="8072437"/>
+          <a:ext cx="3143250" cy="2544417"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
 </xdr:wsDr>
 </file>
 
@@ -7388,7 +7444,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{6D3DD6BC-0BCA-4BA9-9C7E-A308795ECB28}">
-  <dimension ref="B4:R12"/>
+  <dimension ref="B4:R42"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="2" max="2" width="11.28515625" customWidth="1"/>
@@ -7459,33 +7515,33 @@
       </c>
     </row>
     <row r="7" spans="2:18" x14ac:dyDescent="0.25">
-      <c r="B7" s="170" t="s">
+      <c r="B7" s="141" t="s">
         <v>266</v>
       </c>
-      <c r="C7" s="171">
+      <c r="C7" s="170">
         <f>C9/C8</f>
         <v>0.63833075734157652</v>
       </c>
-      <c r="D7" s="171">
+      <c r="D7" s="170">
         <f>D9/D8</f>
         <v>0.78412698412698423</v>
       </c>
-      <c r="E7" s="171">
+      <c r="E7" s="170">
         <f>E9/E8</f>
         <v>0.89473684210526327</v>
       </c>
-      <c r="O7" s="170" t="s">
+      <c r="O7" s="141" t="s">
         <v>266</v>
       </c>
-      <c r="P7" s="171">
+      <c r="P7" s="170">
         <f>P9/P8</f>
         <v>0.76984126984126977</v>
       </c>
-      <c r="Q7" s="171">
+      <c r="Q7" s="170">
         <f>Q9/Q8</f>
         <v>0.8512110726643598</v>
       </c>
-      <c r="R7" s="171">
+      <c r="R7" s="170">
         <f>R9/R8</f>
         <v>0.90909090909090906</v>
       </c>
@@ -7625,6 +7681,15 @@
         <f t="shared" si="1"/>
         <v>-0.19000000000000039</v>
       </c>
+    </row>
+    <row r="42" spans="2:6" x14ac:dyDescent="0.25">
+      <c r="B42" s="172" t="s">
+        <v>321</v>
+      </c>
+      <c r="C42" s="171"/>
+      <c r="D42" s="171"/>
+      <c r="E42" s="171"/>
+      <c r="F42" s="171"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>